<commit_message>
Planogram: center cards, Wall 5 Rack (replaces Wall 4 Rack), wall hook zones match 5-rack proportions
- Cards centered horizontally in every zone (screen and PNG), captions centered
- Wall 5 Rack: small, small, tall, small, small; old 'Wall 4 Rack' imports as Wall 5 Rack
- Wall 3 Rack + 2 Gantungan uses the same proportions; hook cards no longer overflow zone
- Excel template: LAYOUT/DAFTAR_FIXTURE updated to Wall 5 Rack

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGHS9u6kQyg6PXbaVYikDd
</commit_message>
<xml_diff>
--- a/template_planogram.xlsx
+++ b/template_planogram.xlsx
@@ -920,7 +920,7 @@
         <v/>
       </c>
       <c r="I2" s="10">
-        <f>IF(OR(B2="",C2=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B2&amp;"|"&amp;C2,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B2="",C2=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B2&amp;"|"&amp;C2,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J2" s="13">
@@ -970,7 +970,7 @@
         <v/>
       </c>
       <c r="I3" s="10">
-        <f>IF(OR(B3="",C3=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B3&amp;"|"&amp;C3,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B3="",C3=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B3&amp;"|"&amp;C3,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J3" s="13">
@@ -1020,7 +1020,7 @@
         <v/>
       </c>
       <c r="I4" s="10">
-        <f>IF(OR(B4="",C4=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B4&amp;"|"&amp;C4,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B4="",C4=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B4&amp;"|"&amp;C4,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J4" s="13">
@@ -1070,7 +1070,7 @@
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>IF(OR(B5="",C5=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B5&amp;"|"&amp;C5,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B5="",C5=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B5&amp;"|"&amp;C5,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J5" s="13">
@@ -1120,7 +1120,7 @@
         <v/>
       </c>
       <c r="I6" s="10">
-        <f>IF(OR(B6="",C6=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B6&amp;"|"&amp;C6,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B6="",C6=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B6&amp;"|"&amp;C6,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J6" s="13">
@@ -1170,7 +1170,7 @@
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>IF(OR(B7="",C7=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B7&amp;"|"&amp;C7,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B7="",C7=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B7&amp;"|"&amp;C7,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J7" s="13">
@@ -1220,7 +1220,7 @@
         <v/>
       </c>
       <c r="I8" s="10">
-        <f>IF(OR(B8="",C8=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B8&amp;"|"&amp;C8,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B8="",C8=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B8&amp;"|"&amp;C8,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J8" s="13">
@@ -1270,7 +1270,7 @@
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>IF(OR(B9="",C9=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B9&amp;"|"&amp;C9,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B9="",C9=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B9&amp;"|"&amp;C9,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J9" s="13">
@@ -1320,7 +1320,7 @@
         <v/>
       </c>
       <c r="I10" s="10">
-        <f>IF(OR(B10="",C10=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B10&amp;"|"&amp;C10,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B10="",C10=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B10&amp;"|"&amp;C10,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J10" s="13">
@@ -1370,7 +1370,7 @@
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>IF(OR(B11="",C11=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B11&amp;"|"&amp;C11,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B11="",C11=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B11&amp;"|"&amp;C11,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J11" s="13">
@@ -1408,7 +1408,7 @@
         <v/>
       </c>
       <c r="I12" s="10">
-        <f>IF(OR(B12="",C12=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B12&amp;"|"&amp;C12,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B12="",C12=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B12&amp;"|"&amp;C12,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J12" s="13">
@@ -1446,7 +1446,7 @@
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>IF(OR(B13="",C13=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B13&amp;"|"&amp;C13,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B13="",C13=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B13&amp;"|"&amp;C13,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J13" s="13">
@@ -1484,7 +1484,7 @@
         <v/>
       </c>
       <c r="I14" s="10">
-        <f>IF(OR(B14="",C14=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B14&amp;"|"&amp;C14,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B14="",C14=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B14&amp;"|"&amp;C14,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J14" s="13">
@@ -1534,7 +1534,7 @@
         <v/>
       </c>
       <c r="I15" s="10">
-        <f>IF(OR(B15="",C15=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B15&amp;"|"&amp;C15,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B15="",C15=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B15&amp;"|"&amp;C15,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J15" s="13">
@@ -1584,7 +1584,7 @@
         <v/>
       </c>
       <c r="I16" s="10">
-        <f>IF(OR(B16="",C16=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B16&amp;"|"&amp;C16,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B16="",C16=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B16&amp;"|"&amp;C16,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J16" s="13">
@@ -1634,7 +1634,7 @@
         <v/>
       </c>
       <c r="I17" s="10">
-        <f>IF(OR(B17="",C17=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B17&amp;"|"&amp;C17,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B17="",C17=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B17&amp;"|"&amp;C17,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J17" s="13">
@@ -1684,7 +1684,7 @@
         <v/>
       </c>
       <c r="I18" s="10">
-        <f>IF(OR(B18="",C18=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B18&amp;"|"&amp;C18,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B18="",C18=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B18&amp;"|"&amp;C18,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J18" s="13">
@@ -1734,7 +1734,7 @@
         <v/>
       </c>
       <c r="I19" s="10">
-        <f>IF(OR(B19="",C19=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B19&amp;"|"&amp;C19,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B19="",C19=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B19&amp;"|"&amp;C19,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J19" s="13">
@@ -1784,7 +1784,7 @@
         <v/>
       </c>
       <c r="I20" s="10">
-        <f>IF(OR(B20="",C20=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B20&amp;"|"&amp;C20,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B20="",C20=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B20&amp;"|"&amp;C20,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J20" s="13">
@@ -1834,7 +1834,7 @@
         <v/>
       </c>
       <c r="I21" s="10">
-        <f>IF(OR(B21="",C21=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B21&amp;"|"&amp;C21,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B21="",C21=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B21&amp;"|"&amp;C21,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J21" s="13">
@@ -1884,7 +1884,7 @@
         <v/>
       </c>
       <c r="I22" s="10">
-        <f>IF(OR(B22="",C22=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B22&amp;"|"&amp;C22,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B22="",C22=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B22&amp;"|"&amp;C22,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J22" s="13">
@@ -1934,7 +1934,7 @@
         <v/>
       </c>
       <c r="I23" s="10">
-        <f>IF(OR(B23="",C23=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B23&amp;"|"&amp;C23,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B23="",C23=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B23&amp;"|"&amp;C23,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J23" s="13">
@@ -1984,7 +1984,7 @@
         <v/>
       </c>
       <c r="I24" s="10">
-        <f>IF(OR(B24="",C24=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B24&amp;"|"&amp;C24,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B24="",C24=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B24&amp;"|"&amp;C24,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J24" s="13">
@@ -2022,7 +2022,7 @@
         <v/>
       </c>
       <c r="I25" s="10">
-        <f>IF(OR(B25="",C25=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B25&amp;"|"&amp;C25,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B25="",C25=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B25&amp;"|"&amp;C25,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J25" s="13">
@@ -2072,7 +2072,7 @@
         <v/>
       </c>
       <c r="I26" s="10">
-        <f>IF(OR(B26="",C26=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B26&amp;"|"&amp;C26,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B26="",C26=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B26&amp;"|"&amp;C26,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J26" s="13">
@@ -2122,7 +2122,7 @@
         <v/>
       </c>
       <c r="I27" s="10">
-        <f>IF(OR(B27="",C27=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B27&amp;"|"&amp;C27,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B27="",C27=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B27&amp;"|"&amp;C27,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J27" s="13">
@@ -2172,7 +2172,7 @@
         <v/>
       </c>
       <c r="I28" s="10">
-        <f>IF(OR(B28="",C28=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B28&amp;"|"&amp;C28,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B28="",C28=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B28&amp;"|"&amp;C28,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J28" s="13">
@@ -2222,7 +2222,7 @@
         <v/>
       </c>
       <c r="I29" s="10">
-        <f>IF(OR(B29="",C29=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B29&amp;"|"&amp;C29,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B29="",C29=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B29&amp;"|"&amp;C29,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J29" s="13">
@@ -2272,7 +2272,7 @@
         <v/>
       </c>
       <c r="I30" s="10">
-        <f>IF(OR(B30="",C30=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B30&amp;"|"&amp;C30,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B30="",C30=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B30&amp;"|"&amp;C30,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J30" s="13">
@@ -2322,7 +2322,7 @@
         <v/>
       </c>
       <c r="I31" s="10">
-        <f>IF(OR(B31="",C31=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B31&amp;"|"&amp;C31,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B31="",C31=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B31&amp;"|"&amp;C31,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J31" s="13">
@@ -2372,7 +2372,7 @@
         <v/>
       </c>
       <c r="I32" s="10">
-        <f>IF(OR(B32="",C32=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B32&amp;"|"&amp;C32,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B32="",C32=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B32&amp;"|"&amp;C32,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J32" s="13">
@@ -2422,7 +2422,7 @@
         <v/>
       </c>
       <c r="I33" s="10">
-        <f>IF(OR(B33="",C33=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B33&amp;"|"&amp;C33,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B33="",C33=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B33&amp;"|"&amp;C33,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J33" s="13">
@@ -2460,7 +2460,7 @@
         <v/>
       </c>
       <c r="I34" s="10">
-        <f>IF(OR(B34="",C34=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B34&amp;"|"&amp;C34,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B34="",C34=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B34&amp;"|"&amp;C34,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J34" s="13">
@@ -2498,7 +2498,7 @@
         <v/>
       </c>
       <c r="I35" s="10">
-        <f>IF(OR(B35="",C35=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B35&amp;"|"&amp;C35,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B35="",C35=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B35&amp;"|"&amp;C35,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J35" s="13">
@@ -2536,7 +2536,7 @@
         <v/>
       </c>
       <c r="I36" s="10">
-        <f>IF(OR(B36="",C36=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B36&amp;"|"&amp;C36,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B36="",C36=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B36&amp;"|"&amp;C36,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J36" s="13">
@@ -2586,7 +2586,7 @@
         <v/>
       </c>
       <c r="I37" s="10">
-        <f>IF(OR(B37="",C37=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B37&amp;"|"&amp;C37,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B37="",C37=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B37&amp;"|"&amp;C37,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J37" s="13">
@@ -2636,7 +2636,7 @@
         <v/>
       </c>
       <c r="I38" s="10">
-        <f>IF(OR(B38="",C38=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B38&amp;"|"&amp;C38,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B38="",C38=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B38&amp;"|"&amp;C38,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J38" s="13">
@@ -2686,7 +2686,7 @@
         <v/>
       </c>
       <c r="I39" s="10">
-        <f>IF(OR(B39="",C39=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B39&amp;"|"&amp;C39,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B39="",C39=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B39&amp;"|"&amp;C39,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J39" s="13">
@@ -2736,7 +2736,7 @@
         <v/>
       </c>
       <c r="I40" s="10">
-        <f>IF(OR(B40="",C40=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B40&amp;"|"&amp;C40,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B40="",C40=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B40&amp;"|"&amp;C40,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J40" s="13">
@@ -2786,7 +2786,7 @@
         <v/>
       </c>
       <c r="I41" s="10">
-        <f>IF(OR(B41="",C41=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B41&amp;"|"&amp;C41,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B41="",C41=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B41&amp;"|"&amp;C41,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J41" s="13">
@@ -2836,7 +2836,7 @@
         <v/>
       </c>
       <c r="I42" s="10">
-        <f>IF(OR(B42="",C42=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B42&amp;"|"&amp;C42,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B42="",C42=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B42&amp;"|"&amp;C42,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J42" s="13">
@@ -2874,7 +2874,7 @@
         <v/>
       </c>
       <c r="I43" s="10">
-        <f>IF(OR(B43="",C43=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B43&amp;"|"&amp;C43,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B43="",C43=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B43&amp;"|"&amp;C43,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J43" s="13">
@@ -2912,7 +2912,7 @@
         <v/>
       </c>
       <c r="I44" s="10">
-        <f>IF(OR(B44="",C44=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B44&amp;"|"&amp;C44,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B44="",C44=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B44&amp;"|"&amp;C44,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J44" s="13">
@@ -2962,7 +2962,7 @@
         <v/>
       </c>
       <c r="I45" s="10">
-        <f>IF(OR(B45="",C45=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B45&amp;"|"&amp;C45,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B45="",C45=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B45&amp;"|"&amp;C45,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J45" s="13">
@@ -3012,7 +3012,7 @@
         <v/>
       </c>
       <c r="I46" s="10">
-        <f>IF(OR(B46="",C46=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B46&amp;"|"&amp;C46,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B46="",C46=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B46&amp;"|"&amp;C46,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J46" s="13">
@@ -3062,7 +3062,7 @@
         <v/>
       </c>
       <c r="I47" s="10">
-        <f>IF(OR(B47="",C47=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B47&amp;"|"&amp;C47,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B47="",C47=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B47&amp;"|"&amp;C47,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J47" s="13">
@@ -3112,7 +3112,7 @@
         <v/>
       </c>
       <c r="I48" s="10">
-        <f>IF(OR(B48="",C48=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B48&amp;"|"&amp;C48,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B48="",C48=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B48&amp;"|"&amp;C48,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J48" s="13">
@@ -3162,7 +3162,7 @@
         <v/>
       </c>
       <c r="I49" s="10">
-        <f>IF(OR(B49="",C49=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B49&amp;"|"&amp;C49,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B49="",C49=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B49&amp;"|"&amp;C49,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J49" s="13">
@@ -3212,7 +3212,7 @@
         <v/>
       </c>
       <c r="I50" s="10">
-        <f>IF(OR(B50="",C50=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B50&amp;"|"&amp;C50,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B50="",C50=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B50&amp;"|"&amp;C50,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J50" s="13">
@@ -3262,7 +3262,7 @@
         <v/>
       </c>
       <c r="I51" s="10">
-        <f>IF(OR(B51="",C51=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B51&amp;"|"&amp;C51,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B51="",C51=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B51&amp;"|"&amp;C51,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J51" s="13">
@@ -3312,7 +3312,7 @@
         <v/>
       </c>
       <c r="I52" s="10">
-        <f>IF(OR(B52="",C52=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B52&amp;"|"&amp;C52,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B52="",C52=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B52&amp;"|"&amp;C52,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J52" s="13">
@@ -3362,7 +3362,7 @@
         <v/>
       </c>
       <c r="I53" s="10">
-        <f>IF(OR(B53="",C53=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B53&amp;"|"&amp;C53,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B53="",C53=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B53&amp;"|"&amp;C53,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J53" s="13">
@@ -3412,7 +3412,7 @@
         <v/>
       </c>
       <c r="I54" s="10">
-        <f>IF(OR(B54="",C54=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B54&amp;"|"&amp;C54,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B54="",C54=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B54&amp;"|"&amp;C54,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J54" s="13">
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="I55" s="10">
-        <f>IF(OR(B55="",C55=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B55&amp;"|"&amp;C55,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B55="",C55=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B55&amp;"|"&amp;C55,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J55" s="13">
@@ -3512,7 +3512,7 @@
         <v/>
       </c>
       <c r="I56" s="10">
-        <f>IF(OR(B56="",C56=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B56&amp;"|"&amp;C56,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B56="",C56=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B56&amp;"|"&amp;C56,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J56" s="13">
@@ -3562,7 +3562,7 @@
         <v/>
       </c>
       <c r="I57" s="10">
-        <f>IF(OR(B57="",C57=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B57&amp;"|"&amp;C57,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B57="",C57=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B57&amp;"|"&amp;C57,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J57" s="13">
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="I58" s="10">
-        <f>IF(OR(B58="",C58=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B58&amp;"|"&amp;C58,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B58="",C58=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B58&amp;"|"&amp;C58,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J58" s="13">
@@ -3662,7 +3662,7 @@
         <v/>
       </c>
       <c r="I59" s="10">
-        <f>IF(OR(B59="",C59=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B59&amp;"|"&amp;C59,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B59="",C59=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B59&amp;"|"&amp;C59,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J59" s="13">
@@ -3712,7 +3712,7 @@
         <v/>
       </c>
       <c r="I60" s="10">
-        <f>IF(OR(B60="",C60=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B60&amp;"|"&amp;C60,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B60="",C60=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B60&amp;"|"&amp;C60,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J60" s="13">
@@ -3762,7 +3762,7 @@
         <v/>
       </c>
       <c r="I61" s="10">
-        <f>IF(OR(B61="",C61=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B61&amp;"|"&amp;C61,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B61="",C61=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B61&amp;"|"&amp;C61,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J61" s="13">
@@ -3812,7 +3812,7 @@
         <v/>
       </c>
       <c r="I62" s="10">
-        <f>IF(OR(B62="",C62=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B62&amp;"|"&amp;C62,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B62="",C62=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B62&amp;"|"&amp;C62,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J62" s="13">
@@ -3862,7 +3862,7 @@
         <v/>
       </c>
       <c r="I63" s="10">
-        <f>IF(OR(B63="",C63=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B63&amp;"|"&amp;C63,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B63="",C63=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B63&amp;"|"&amp;C63,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J63" s="13">
@@ -3912,7 +3912,7 @@
         <v/>
       </c>
       <c r="I64" s="10">
-        <f>IF(OR(B64="",C64=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B64&amp;"|"&amp;C64,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B64="",C64=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B64&amp;"|"&amp;C64,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J64" s="13">
@@ -3962,7 +3962,7 @@
         <v/>
       </c>
       <c r="I65" s="10">
-        <f>IF(OR(B65="",C65=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B65&amp;"|"&amp;C65,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B65="",C65=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B65&amp;"|"&amp;C65,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J65" s="13">
@@ -4012,7 +4012,7 @@
         <v/>
       </c>
       <c r="I66" s="10">
-        <f>IF(OR(B66="",C66=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B66&amp;"|"&amp;C66,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B66="",C66=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B66&amp;"|"&amp;C66,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J66" s="13">
@@ -4062,7 +4062,7 @@
         <v/>
       </c>
       <c r="I67" s="10">
-        <f>IF(OR(B67="",C67=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B67&amp;"|"&amp;C67,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B67="",C67=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B67&amp;"|"&amp;C67,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J67" s="13">
@@ -4112,7 +4112,7 @@
         <v/>
       </c>
       <c r="I68" s="10">
-        <f>IF(OR(B68="",C68=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B68&amp;"|"&amp;C68,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B68="",C68=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B68&amp;"|"&amp;C68,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J68" s="13">
@@ -4162,7 +4162,7 @@
         <v/>
       </c>
       <c r="I69" s="10">
-        <f>IF(OR(B69="",C69=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B69&amp;"|"&amp;C69,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B69="",C69=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B69&amp;"|"&amp;C69,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J69" s="13">
@@ -4212,7 +4212,7 @@
         <v/>
       </c>
       <c r="I70" s="10">
-        <f>IF(OR(B70="",C70=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B70&amp;"|"&amp;C70,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B70="",C70=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B70&amp;"|"&amp;C70,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J70" s="13">
@@ -4262,7 +4262,7 @@
         <v/>
       </c>
       <c r="I71" s="10">
-        <f>IF(OR(B71="",C71=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B71&amp;"|"&amp;C71,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B71="",C71=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B71&amp;"|"&amp;C71,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J71" s="13">
@@ -4312,7 +4312,7 @@
         <v/>
       </c>
       <c r="I72" s="10">
-        <f>IF(OR(B72="",C72=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B72&amp;"|"&amp;C72,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B72="",C72=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B72&amp;"|"&amp;C72,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J72" s="13">
@@ -4362,7 +4362,7 @@
         <v/>
       </c>
       <c r="I73" s="10">
-        <f>IF(OR(B73="",C73=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B73&amp;"|"&amp;C73,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B73="",C73=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B73&amp;"|"&amp;C73,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J73" s="13">
@@ -4412,7 +4412,7 @@
         <v/>
       </c>
       <c r="I74" s="10">
-        <f>IF(OR(B74="",C74=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B74&amp;"|"&amp;C74,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B74="",C74=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B74&amp;"|"&amp;C74,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J74" s="13">
@@ -4462,7 +4462,7 @@
         <v/>
       </c>
       <c r="I75" s="10">
-        <f>IF(OR(B75="",C75=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B75&amp;"|"&amp;C75,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B75="",C75=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B75&amp;"|"&amp;C75,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J75" s="13">
@@ -4512,7 +4512,7 @@
         <v/>
       </c>
       <c r="I76" s="10">
-        <f>IF(OR(B76="",C76=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B76&amp;"|"&amp;C76,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B76="",C76=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B76&amp;"|"&amp;C76,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J76" s="13">
@@ -4562,7 +4562,7 @@
         <v/>
       </c>
       <c r="I77" s="10">
-        <f>IF(OR(B77="",C77=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B77&amp;"|"&amp;C77,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B77="",C77=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B77&amp;"|"&amp;C77,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J77" s="13">
@@ -4612,7 +4612,7 @@
         <v/>
       </c>
       <c r="I78" s="10">
-        <f>IF(OR(B78="",C78=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B78&amp;"|"&amp;C78,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B78="",C78=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B78&amp;"|"&amp;C78,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J78" s="13">
@@ -4662,7 +4662,7 @@
         <v/>
       </c>
       <c r="I79" s="10">
-        <f>IF(OR(B79="",C79=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B79&amp;"|"&amp;C79,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B79="",C79=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B79&amp;"|"&amp;C79,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J79" s="13">
@@ -4712,7 +4712,7 @@
         <v/>
       </c>
       <c r="I80" s="10">
-        <f>IF(OR(B80="",C80=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B80&amp;"|"&amp;C80,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B80="",C80=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B80&amp;"|"&amp;C80,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J80" s="13">
@@ -4762,7 +4762,7 @@
         <v/>
       </c>
       <c r="I81" s="10">
-        <f>IF(OR(B81="",C81=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B81&amp;"|"&amp;C81,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B81="",C81=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B81&amp;"|"&amp;C81,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J81" s="13">
@@ -4812,7 +4812,7 @@
         <v/>
       </c>
       <c r="I82" s="10">
-        <f>IF(OR(B82="",C82=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B82&amp;"|"&amp;C82,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B82="",C82=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B82&amp;"|"&amp;C82,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J82" s="13">
@@ -4862,7 +4862,7 @@
         <v/>
       </c>
       <c r="I83" s="10">
-        <f>IF(OR(B83="",C83=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B83&amp;"|"&amp;C83,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B83="",C83=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B83&amp;"|"&amp;C83,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J83" s="13">
@@ -4912,7 +4912,7 @@
         <v/>
       </c>
       <c r="I84" s="10">
-        <f>IF(OR(B84="",C84=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B84&amp;"|"&amp;C84,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B84="",C84=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B84&amp;"|"&amp;C84,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J84" s="13">
@@ -4962,7 +4962,7 @@
         <v/>
       </c>
       <c r="I85" s="10">
-        <f>IF(OR(B85="",C85=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B85&amp;"|"&amp;C85,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B85="",C85=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B85&amp;"|"&amp;C85,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J85" s="13">
@@ -5012,7 +5012,7 @@
         <v/>
       </c>
       <c r="I86" s="10">
-        <f>IF(OR(B86="",C86=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B86&amp;"|"&amp;C86,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B86="",C86=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B86&amp;"|"&amp;C86,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J86" s="13">
@@ -5062,7 +5062,7 @@
         <v/>
       </c>
       <c r="I87" s="10">
-        <f>IF(OR(B87="",C87=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B87&amp;"|"&amp;C87,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B87="",C87=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B87&amp;"|"&amp;C87,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J87" s="13">
@@ -5112,7 +5112,7 @@
         <v/>
       </c>
       <c r="I88" s="10">
-        <f>IF(OR(B88="",C88=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B88&amp;"|"&amp;C88,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B88="",C88=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B88&amp;"|"&amp;C88,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J88" s="13">
@@ -5162,7 +5162,7 @@
         <v/>
       </c>
       <c r="I89" s="10">
-        <f>IF(OR(B89="",C89=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B89&amp;"|"&amp;C89,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B89="",C89=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B89&amp;"|"&amp;C89,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J89" s="13">
@@ -5212,7 +5212,7 @@
         <v/>
       </c>
       <c r="I90" s="10">
-        <f>IF(OR(B90="",C90=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B90&amp;"|"&amp;C90,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B90="",C90=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B90&amp;"|"&amp;C90,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J90" s="13">
@@ -5262,7 +5262,7 @@
         <v/>
       </c>
       <c r="I91" s="10">
-        <f>IF(OR(B91="",C91=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B91&amp;"|"&amp;C91,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B91="",C91=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B91&amp;"|"&amp;C91,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J91" s="13">
@@ -5312,7 +5312,7 @@
         <v/>
       </c>
       <c r="I92" s="10">
-        <f>IF(OR(B92="",C92=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B92&amp;"|"&amp;C92,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B92="",C92=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B92&amp;"|"&amp;C92,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J92" s="13">
@@ -5362,7 +5362,7 @@
         <v/>
       </c>
       <c r="I93" s="10">
-        <f>IF(OR(B93="",C93=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B93&amp;"|"&amp;C93,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B93="",C93=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B93&amp;"|"&amp;C93,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J93" s="13">
@@ -5412,7 +5412,7 @@
         <v/>
       </c>
       <c r="I94" s="10">
-        <f>IF(OR(B94="",C94=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B94&amp;"|"&amp;C94,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B94="",C94=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B94&amp;"|"&amp;C94,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J94" s="13">
@@ -5462,7 +5462,7 @@
         <v/>
       </c>
       <c r="I95" s="10">
-        <f>IF(OR(B95="",C95=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B95&amp;"|"&amp;C95,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B95="",C95=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B95&amp;"|"&amp;C95,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J95" s="13">
@@ -5512,7 +5512,7 @@
         <v/>
       </c>
       <c r="I96" s="10">
-        <f>IF(OR(B96="",C96=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B96&amp;"|"&amp;C96,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B96="",C96=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B96&amp;"|"&amp;C96,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J96" s="13">
@@ -5562,7 +5562,7 @@
         <v/>
       </c>
       <c r="I97" s="10">
-        <f>IF(OR(B97="",C97=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B97&amp;"|"&amp;C97,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B97="",C97=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B97&amp;"|"&amp;C97,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J97" s="13">
@@ -5612,7 +5612,7 @@
         <v/>
       </c>
       <c r="I98" s="10">
-        <f>IF(OR(B98="",C98=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B98&amp;"|"&amp;C98,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B98="",C98=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B98&amp;"|"&amp;C98,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J98" s="13">
@@ -5662,7 +5662,7 @@
         <v/>
       </c>
       <c r="I99" s="10">
-        <f>IF(OR(B99="",C99=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B99&amp;"|"&amp;C99,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B99="",C99=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B99&amp;"|"&amp;C99,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J99" s="13">
@@ -5712,7 +5712,7 @@
         <v/>
       </c>
       <c r="I100" s="10">
-        <f>IF(OR(B100="",C100=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B100&amp;"|"&amp;C100,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B100="",C100=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B100&amp;"|"&amp;C100,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J100" s="13">
@@ -5762,7 +5762,7 @@
         <v/>
       </c>
       <c r="I101" s="10">
-        <f>IF(OR(B101="",C101=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B101&amp;"|"&amp;C101,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B101="",C101=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B101&amp;"|"&amp;C101,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J101" s="13">
@@ -5812,7 +5812,7 @@
         <v/>
       </c>
       <c r="I102" s="10">
-        <f>IF(OR(B102="",C102=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B102&amp;"|"&amp;C102,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B102="",C102=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B102&amp;"|"&amp;C102,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J102" s="13">
@@ -5862,7 +5862,7 @@
         <v/>
       </c>
       <c r="I103" s="10">
-        <f>IF(OR(B103="",C103=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B103&amp;"|"&amp;C103,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B103="",C103=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B103&amp;"|"&amp;C103,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J103" s="13">
@@ -5912,7 +5912,7 @@
         <v/>
       </c>
       <c r="I104" s="10">
-        <f>IF(OR(B104="",C104=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B104&amp;"|"&amp;C104,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B104="",C104=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B104&amp;"|"&amp;C104,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J104" s="13">
@@ -5962,7 +5962,7 @@
         <v/>
       </c>
       <c r="I105" s="10">
-        <f>IF(OR(B105="",C105=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B105&amp;"|"&amp;C105,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B105="",C105=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B105&amp;"|"&amp;C105,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J105" s="13">
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="I106" s="10">
-        <f>IF(OR(B106="",C106=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B106&amp;"|"&amp;C106,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B106="",C106=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B106&amp;"|"&amp;C106,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J106" s="13">
@@ -6062,7 +6062,7 @@
         <v/>
       </c>
       <c r="I107" s="10">
-        <f>IF(OR(B107="",C107=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B107&amp;"|"&amp;C107,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B107="",C107=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B107&amp;"|"&amp;C107,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J107" s="13">
@@ -6112,7 +6112,7 @@
         <v/>
       </c>
       <c r="I108" s="10">
-        <f>IF(OR(B108="",C108=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B108&amp;"|"&amp;C108,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B108="",C108=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B108&amp;"|"&amp;C108,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J108" s="13">
@@ -6162,7 +6162,7 @@
         <v/>
       </c>
       <c r="I109" s="10">
-        <f>IF(OR(B109="",C109=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B109&amp;"|"&amp;C109,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B109="",C109=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B109&amp;"|"&amp;C109,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J109" s="13">
@@ -6212,7 +6212,7 @@
         <v/>
       </c>
       <c r="I110" s="10">
-        <f>IF(OR(B110="",C110=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B110&amp;"|"&amp;C110,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B110="",C110=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B110&amp;"|"&amp;C110,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J110" s="13">
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="I111" s="10">
-        <f>IF(OR(B111="",C111=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B111&amp;"|"&amp;C111,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B111="",C111=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B111&amp;"|"&amp;C111,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J111" s="13">
@@ -6312,7 +6312,7 @@
         <v/>
       </c>
       <c r="I112" s="10">
-        <f>IF(OR(B112="",C112=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B112&amp;"|"&amp;C112,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B112="",C112=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B112&amp;"|"&amp;C112,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J112" s="13">
@@ -6362,7 +6362,7 @@
         <v/>
       </c>
       <c r="I113" s="10">
-        <f>IF(OR(B113="",C113=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B113&amp;"|"&amp;C113,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B113="",C113=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B113&amp;"|"&amp;C113,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J113" s="13">
@@ -6412,7 +6412,7 @@
         <v/>
       </c>
       <c r="I114" s="10">
-        <f>IF(OR(B114="",C114=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B114&amp;"|"&amp;C114,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B114="",C114=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B114&amp;"|"&amp;C114,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J114" s="13">
@@ -6462,7 +6462,7 @@
         <v/>
       </c>
       <c r="I115" s="10">
-        <f>IF(OR(B115="",C115=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B115&amp;"|"&amp;C115,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B115="",C115=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B115&amp;"|"&amp;C115,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J115" s="13">
@@ -6512,7 +6512,7 @@
         <v/>
       </c>
       <c r="I116" s="10">
-        <f>IF(OR(B116="",C116=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B116&amp;"|"&amp;C116,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B116="",C116=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B116&amp;"|"&amp;C116,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J116" s="13">
@@ -6562,7 +6562,7 @@
         <v/>
       </c>
       <c r="I117" s="10">
-        <f>IF(OR(B117="",C117=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B117&amp;"|"&amp;C117,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B117="",C117=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B117&amp;"|"&amp;C117,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J117" s="13">
@@ -6590,7 +6590,7 @@
         <v/>
       </c>
       <c r="I118" s="10">
-        <f>IF(OR(B118="",C118=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B118&amp;"|"&amp;C118,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B118="",C118=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B118&amp;"|"&amp;C118,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J118" s="13">
@@ -6618,7 +6618,7 @@
         <v/>
       </c>
       <c r="I119" s="10">
-        <f>IF(OR(B119="",C119=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B119&amp;"|"&amp;C119,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B119="",C119=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B119&amp;"|"&amp;C119,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J119" s="13">
@@ -6646,7 +6646,7 @@
         <v/>
       </c>
       <c r="I120" s="10">
-        <f>IF(OR(B120="",C120=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B120&amp;"|"&amp;C120,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B120="",C120=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B120&amp;"|"&amp;C120,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J120" s="13">
@@ -6674,7 +6674,7 @@
         <v/>
       </c>
       <c r="I121" s="10">
-        <f>IF(OR(B121="",C121=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B121&amp;"|"&amp;C121,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B121="",C121=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B121&amp;"|"&amp;C121,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J121" s="13">
@@ -6702,7 +6702,7 @@
         <v/>
       </c>
       <c r="I122" s="10">
-        <f>IF(OR(B122="",C122=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B122&amp;"|"&amp;C122,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B122="",C122=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B122&amp;"|"&amp;C122,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J122" s="13">
@@ -6730,7 +6730,7 @@
         <v/>
       </c>
       <c r="I123" s="10">
-        <f>IF(OR(B123="",C123=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B123&amp;"|"&amp;C123,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B123="",C123=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B123&amp;"|"&amp;C123,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J123" s="13">
@@ -6758,7 +6758,7 @@
         <v/>
       </c>
       <c r="I124" s="10">
-        <f>IF(OR(B124="",C124=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B124&amp;"|"&amp;C124,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B124="",C124=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B124&amp;"|"&amp;C124,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J124" s="13">
@@ -6786,7 +6786,7 @@
         <v/>
       </c>
       <c r="I125" s="10">
-        <f>IF(OR(B125="",C125=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B125&amp;"|"&amp;C125,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B125="",C125=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B125&amp;"|"&amp;C125,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J125" s="13">
@@ -6814,7 +6814,7 @@
         <v/>
       </c>
       <c r="I126" s="10">
-        <f>IF(OR(B126="",C126=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B126&amp;"|"&amp;C126,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B126="",C126=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B126&amp;"|"&amp;C126,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J126" s="13">
@@ -6842,7 +6842,7 @@
         <v/>
       </c>
       <c r="I127" s="10">
-        <f>IF(OR(B127="",C127=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B127&amp;"|"&amp;C127,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B127="",C127=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B127&amp;"|"&amp;C127,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J127" s="13">
@@ -6870,7 +6870,7 @@
         <v/>
       </c>
       <c r="I128" s="10">
-        <f>IF(OR(B128="",C128=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B128&amp;"|"&amp;C128,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B128="",C128=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B128&amp;"|"&amp;C128,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J128" s="13">
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="I129" s="10">
-        <f>IF(OR(B129="",C129=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B129&amp;"|"&amp;C129,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B129="",C129=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B129&amp;"|"&amp;C129,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J129" s="13">
@@ -6926,7 +6926,7 @@
         <v/>
       </c>
       <c r="I130" s="10">
-        <f>IF(OR(B130="",C130=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B130&amp;"|"&amp;C130,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B130="",C130=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B130&amp;"|"&amp;C130,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J130" s="13">
@@ -6954,7 +6954,7 @@
         <v/>
       </c>
       <c r="I131" s="10">
-        <f>IF(OR(B131="",C131=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B131&amp;"|"&amp;C131,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B131="",C131=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B131&amp;"|"&amp;C131,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J131" s="13">
@@ -6982,7 +6982,7 @@
         <v/>
       </c>
       <c r="I132" s="10">
-        <f>IF(OR(B132="",C132=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B132&amp;"|"&amp;C132,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B132="",C132=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B132&amp;"|"&amp;C132,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J132" s="13">
@@ -7010,7 +7010,7 @@
         <v/>
       </c>
       <c r="I133" s="10">
-        <f>IF(OR(B133="",C133=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B133&amp;"|"&amp;C133,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B133="",C133=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B133&amp;"|"&amp;C133,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J133" s="13">
@@ -7038,7 +7038,7 @@
         <v/>
       </c>
       <c r="I134" s="10">
-        <f>IF(OR(B134="",C134=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B134&amp;"|"&amp;C134,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B134="",C134=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B134&amp;"|"&amp;C134,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J134" s="13">
@@ -7066,7 +7066,7 @@
         <v/>
       </c>
       <c r="I135" s="10">
-        <f>IF(OR(B135="",C135=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B135&amp;"|"&amp;C135,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B135="",C135=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B135&amp;"|"&amp;C135,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J135" s="13">
@@ -7094,7 +7094,7 @@
         <v/>
       </c>
       <c r="I136" s="10">
-        <f>IF(OR(B136="",C136=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B136&amp;"|"&amp;C136,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B136="",C136=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B136&amp;"|"&amp;C136,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J136" s="13">
@@ -7122,7 +7122,7 @@
         <v/>
       </c>
       <c r="I137" s="10">
-        <f>IF(OR(B137="",C137=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B137&amp;"|"&amp;C137,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B137="",C137=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B137&amp;"|"&amp;C137,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J137" s="13">
@@ -7150,7 +7150,7 @@
         <v/>
       </c>
       <c r="I138" s="10">
-        <f>IF(OR(B138="",C138=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B138&amp;"|"&amp;C138,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B138="",C138=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B138&amp;"|"&amp;C138,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J138" s="13">
@@ -7178,7 +7178,7 @@
         <v/>
       </c>
       <c r="I139" s="10">
-        <f>IF(OR(B139="",C139=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B139&amp;"|"&amp;C139,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B139="",C139=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B139&amp;"|"&amp;C139,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J139" s="13">
@@ -7206,7 +7206,7 @@
         <v/>
       </c>
       <c r="I140" s="10">
-        <f>IF(OR(B140="",C140=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B140&amp;"|"&amp;C140,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B140="",C140=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B140&amp;"|"&amp;C140,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J140" s="13">
@@ -7234,7 +7234,7 @@
         <v/>
       </c>
       <c r="I141" s="10">
-        <f>IF(OR(B141="",C141=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B141&amp;"|"&amp;C141,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B141="",C141=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B141&amp;"|"&amp;C141,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J141" s="13">
@@ -7262,7 +7262,7 @@
         <v/>
       </c>
       <c r="I142" s="10">
-        <f>IF(OR(B142="",C142=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B142&amp;"|"&amp;C142,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B142="",C142=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B142&amp;"|"&amp;C142,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J142" s="13">
@@ -7290,7 +7290,7 @@
         <v/>
       </c>
       <c r="I143" s="10">
-        <f>IF(OR(B143="",C143=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B143&amp;"|"&amp;C143,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B143="",C143=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B143&amp;"|"&amp;C143,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J143" s="13">
@@ -7318,7 +7318,7 @@
         <v/>
       </c>
       <c r="I144" s="10">
-        <f>IF(OR(B144="",C144=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B144&amp;"|"&amp;C144,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B144="",C144=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B144&amp;"|"&amp;C144,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J144" s="13">
@@ -7346,7 +7346,7 @@
         <v/>
       </c>
       <c r="I145" s="10">
-        <f>IF(OR(B145="",C145=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B145&amp;"|"&amp;C145,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B145="",C145=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B145&amp;"|"&amp;C145,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J145" s="13">
@@ -7374,7 +7374,7 @@
         <v/>
       </c>
       <c r="I146" s="10">
-        <f>IF(OR(B146="",C146=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B146&amp;"|"&amp;C146,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B146="",C146=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B146&amp;"|"&amp;C146,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J146" s="13">
@@ -7402,7 +7402,7 @@
         <v/>
       </c>
       <c r="I147" s="10">
-        <f>IF(OR(B147="",C147=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B147&amp;"|"&amp;C147,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B147="",C147=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B147&amp;"|"&amp;C147,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J147" s="13">
@@ -7430,7 +7430,7 @@
         <v/>
       </c>
       <c r="I148" s="10">
-        <f>IF(OR(B148="",C148=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B148&amp;"|"&amp;C148,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B148="",C148=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B148&amp;"|"&amp;C148,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J148" s="13">
@@ -7458,7 +7458,7 @@
         <v/>
       </c>
       <c r="I149" s="10">
-        <f>IF(OR(B149="",C149=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B149&amp;"|"&amp;C149,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B149="",C149=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B149&amp;"|"&amp;C149,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J149" s="13">
@@ -7486,7 +7486,7 @@
         <v/>
       </c>
       <c r="I150" s="10">
-        <f>IF(OR(B150="",C150=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B150&amp;"|"&amp;C150,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B150="",C150=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B150&amp;"|"&amp;C150,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J150" s="13">
@@ -7514,7 +7514,7 @@
         <v/>
       </c>
       <c r="I151" s="10">
-        <f>IF(OR(B151="",C151=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B151&amp;"|"&amp;C151,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B151="",C151=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B151&amp;"|"&amp;C151,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J151" s="13">
@@ -7542,7 +7542,7 @@
         <v/>
       </c>
       <c r="I152" s="10">
-        <f>IF(OR(B152="",C152=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B152&amp;"|"&amp;C152,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B152="",C152=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B152&amp;"|"&amp;C152,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J152" s="13">
@@ -7570,7 +7570,7 @@
         <v/>
       </c>
       <c r="I153" s="10">
-        <f>IF(OR(B153="",C153=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B153&amp;"|"&amp;C153,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B153="",C153=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B153&amp;"|"&amp;C153,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J153" s="13">
@@ -7598,7 +7598,7 @@
         <v/>
       </c>
       <c r="I154" s="10">
-        <f>IF(OR(B154="",C154=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B154&amp;"|"&amp;C154,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B154="",C154=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B154&amp;"|"&amp;C154,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J154" s="13">
@@ -7626,7 +7626,7 @@
         <v/>
       </c>
       <c r="I155" s="10">
-        <f>IF(OR(B155="",C155=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B155&amp;"|"&amp;C155,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B155="",C155=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B155&amp;"|"&amp;C155,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J155" s="13">
@@ -7654,7 +7654,7 @@
         <v/>
       </c>
       <c r="I156" s="10">
-        <f>IF(OR(B156="",C156=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B156&amp;"|"&amp;C156,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B156="",C156=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B156&amp;"|"&amp;C156,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J156" s="13">
@@ -7682,7 +7682,7 @@
         <v/>
       </c>
       <c r="I157" s="10">
-        <f>IF(OR(B157="",C157=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B157&amp;"|"&amp;C157,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B157="",C157=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B157&amp;"|"&amp;C157,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J157" s="13">
@@ -7710,7 +7710,7 @@
         <v/>
       </c>
       <c r="I158" s="10">
-        <f>IF(OR(B158="",C158=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B158&amp;"|"&amp;C158,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B158="",C158=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B158&amp;"|"&amp;C158,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J158" s="13">
@@ -7738,7 +7738,7 @@
         <v/>
       </c>
       <c r="I159" s="10">
-        <f>IF(OR(B159="",C159=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B159&amp;"|"&amp;C159,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B159="",C159=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B159&amp;"|"&amp;C159,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J159" s="13">
@@ -7766,7 +7766,7 @@
         <v/>
       </c>
       <c r="I160" s="10">
-        <f>IF(OR(B160="",C160=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B160&amp;"|"&amp;C160,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B160="",C160=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B160&amp;"|"&amp;C160,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J160" s="13">
@@ -7794,7 +7794,7 @@
         <v/>
       </c>
       <c r="I161" s="10">
-        <f>IF(OR(B161="",C161=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B161&amp;"|"&amp;C161,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B161="",C161=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B161&amp;"|"&amp;C161,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J161" s="13">
@@ -7822,7 +7822,7 @@
         <v/>
       </c>
       <c r="I162" s="10">
-        <f>IF(OR(B162="",C162=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B162&amp;"|"&amp;C162,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B162="",C162=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B162&amp;"|"&amp;C162,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J162" s="13">
@@ -7850,7 +7850,7 @@
         <v/>
       </c>
       <c r="I163" s="10">
-        <f>IF(OR(B163="",C163=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B163&amp;"|"&amp;C163,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B163="",C163=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B163&amp;"|"&amp;C163,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J163" s="13">
@@ -7878,7 +7878,7 @@
         <v/>
       </c>
       <c r="I164" s="10">
-        <f>IF(OR(B164="",C164=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B164&amp;"|"&amp;C164,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B164="",C164=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B164&amp;"|"&amp;C164,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J164" s="13">
@@ -7906,7 +7906,7 @@
         <v/>
       </c>
       <c r="I165" s="10">
-        <f>IF(OR(B165="",C165=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B165&amp;"|"&amp;C165,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B165="",C165=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B165&amp;"|"&amp;C165,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J165" s="13">
@@ -7934,7 +7934,7 @@
         <v/>
       </c>
       <c r="I166" s="10">
-        <f>IF(OR(B166="",C166=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B166&amp;"|"&amp;C166,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B166="",C166=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B166&amp;"|"&amp;C166,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J166" s="13">
@@ -7962,7 +7962,7 @@
         <v/>
       </c>
       <c r="I167" s="10">
-        <f>IF(OR(B167="",C167=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B167&amp;"|"&amp;C167,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B167="",C167=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B167&amp;"|"&amp;C167,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J167" s="13">
@@ -7990,7 +7990,7 @@
         <v/>
       </c>
       <c r="I168" s="10">
-        <f>IF(OR(B168="",C168=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B168&amp;"|"&amp;C168,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B168="",C168=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B168&amp;"|"&amp;C168,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J168" s="13">
@@ -8018,7 +8018,7 @@
         <v/>
       </c>
       <c r="I169" s="10">
-        <f>IF(OR(B169="",C169=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B169&amp;"|"&amp;C169,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B169="",C169=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B169&amp;"|"&amp;C169,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J169" s="13">
@@ -8046,7 +8046,7 @@
         <v/>
       </c>
       <c r="I170" s="10">
-        <f>IF(OR(B170="",C170=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B170&amp;"|"&amp;C170,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B170="",C170=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B170&amp;"|"&amp;C170,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J170" s="13">
@@ -8074,7 +8074,7 @@
         <v/>
       </c>
       <c r="I171" s="10">
-        <f>IF(OR(B171="",C171=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B171&amp;"|"&amp;C171,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B171="",C171=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B171&amp;"|"&amp;C171,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J171" s="13">
@@ -8102,7 +8102,7 @@
         <v/>
       </c>
       <c r="I172" s="10">
-        <f>IF(OR(B172="",C172=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B172&amp;"|"&amp;C172,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B172="",C172=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B172&amp;"|"&amp;C172,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J172" s="13">
@@ -8130,7 +8130,7 @@
         <v/>
       </c>
       <c r="I173" s="10">
-        <f>IF(OR(B173="",C173=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B173&amp;"|"&amp;C173,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B173="",C173=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B173&amp;"|"&amp;C173,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J173" s="13">
@@ -8158,7 +8158,7 @@
         <v/>
       </c>
       <c r="I174" s="10">
-        <f>IF(OR(B174="",C174=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B174&amp;"|"&amp;C174,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B174="",C174=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B174&amp;"|"&amp;C174,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J174" s="13">
@@ -8186,7 +8186,7 @@
         <v/>
       </c>
       <c r="I175" s="10">
-        <f>IF(OR(B175="",C175=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B175&amp;"|"&amp;C175,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B175="",C175=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B175&amp;"|"&amp;C175,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J175" s="13">
@@ -8214,7 +8214,7 @@
         <v/>
       </c>
       <c r="I176" s="10">
-        <f>IF(OR(B176="",C176=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B176&amp;"|"&amp;C176,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B176="",C176=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B176&amp;"|"&amp;C176,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J176" s="13">
@@ -8242,7 +8242,7 @@
         <v/>
       </c>
       <c r="I177" s="10">
-        <f>IF(OR(B177="",C177=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B177&amp;"|"&amp;C177,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B177="",C177=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B177&amp;"|"&amp;C177,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J177" s="13">
@@ -8270,7 +8270,7 @@
         <v/>
       </c>
       <c r="I178" s="10">
-        <f>IF(OR(B178="",C178=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B178&amp;"|"&amp;C178,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B178="",C178=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B178&amp;"|"&amp;C178,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J178" s="13">
@@ -8298,7 +8298,7 @@
         <v/>
       </c>
       <c r="I179" s="10">
-        <f>IF(OR(B179="",C179=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B179&amp;"|"&amp;C179,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B179="",C179=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B179&amp;"|"&amp;C179,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J179" s="13">
@@ -8326,7 +8326,7 @@
         <v/>
       </c>
       <c r="I180" s="10">
-        <f>IF(OR(B180="",C180=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B180&amp;"|"&amp;C180,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B180="",C180=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B180&amp;"|"&amp;C180,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J180" s="13">
@@ -8354,7 +8354,7 @@
         <v/>
       </c>
       <c r="I181" s="10">
-        <f>IF(OR(B181="",C181=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B181&amp;"|"&amp;C181,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B181="",C181=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B181&amp;"|"&amp;C181,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J181" s="13">
@@ -8382,7 +8382,7 @@
         <v/>
       </c>
       <c r="I182" s="10">
-        <f>IF(OR(B182="",C182=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B182&amp;"|"&amp;C182,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B182="",C182=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B182&amp;"|"&amp;C182,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J182" s="13">
@@ -8410,7 +8410,7 @@
         <v/>
       </c>
       <c r="I183" s="10">
-        <f>IF(OR(B183="",C183=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B183&amp;"|"&amp;C183,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B183="",C183=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B183&amp;"|"&amp;C183,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J183" s="13">
@@ -8438,7 +8438,7 @@
         <v/>
       </c>
       <c r="I184" s="10">
-        <f>IF(OR(B184="",C184=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B184&amp;"|"&amp;C184,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B184="",C184=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B184&amp;"|"&amp;C184,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J184" s="13">
@@ -8466,7 +8466,7 @@
         <v/>
       </c>
       <c r="I185" s="10">
-        <f>IF(OR(B185="",C185=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B185&amp;"|"&amp;C185,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B185="",C185=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B185&amp;"|"&amp;C185,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J185" s="13">
@@ -8494,7 +8494,7 @@
         <v/>
       </c>
       <c r="I186" s="10">
-        <f>IF(OR(B186="",C186=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B186&amp;"|"&amp;C186,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B186="",C186=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B186&amp;"|"&amp;C186,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J186" s="13">
@@ -8522,7 +8522,7 @@
         <v/>
       </c>
       <c r="I187" s="10">
-        <f>IF(OR(B187="",C187=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B187&amp;"|"&amp;C187,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B187="",C187=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B187&amp;"|"&amp;C187,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J187" s="13">
@@ -8550,7 +8550,7 @@
         <v/>
       </c>
       <c r="I188" s="10">
-        <f>IF(OR(B188="",C188=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B188&amp;"|"&amp;C188,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B188="",C188=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B188&amp;"|"&amp;C188,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J188" s="13">
@@ -8578,7 +8578,7 @@
         <v/>
       </c>
       <c r="I189" s="10">
-        <f>IF(OR(B189="",C189=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B189&amp;"|"&amp;C189,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B189="",C189=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B189&amp;"|"&amp;C189,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J189" s="13">
@@ -8606,7 +8606,7 @@
         <v/>
       </c>
       <c r="I190" s="10">
-        <f>IF(OR(B190="",C190=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B190&amp;"|"&amp;C190,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B190="",C190=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B190&amp;"|"&amp;C190,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J190" s="13">
@@ -8634,7 +8634,7 @@
         <v/>
       </c>
       <c r="I191" s="10">
-        <f>IF(OR(B191="",C191=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B191&amp;"|"&amp;C191,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B191="",C191=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B191&amp;"|"&amp;C191,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J191" s="13">
@@ -8662,7 +8662,7 @@
         <v/>
       </c>
       <c r="I192" s="10">
-        <f>IF(OR(B192="",C192=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B192&amp;"|"&amp;C192,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B192="",C192=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B192&amp;"|"&amp;C192,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J192" s="13">
@@ -8690,7 +8690,7 @@
         <v/>
       </c>
       <c r="I193" s="10">
-        <f>IF(OR(B193="",C193=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B193&amp;"|"&amp;C193,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B193="",C193=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B193&amp;"|"&amp;C193,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J193" s="13">
@@ -8718,7 +8718,7 @@
         <v/>
       </c>
       <c r="I194" s="10">
-        <f>IF(OR(B194="",C194=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B194&amp;"|"&amp;C194,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B194="",C194=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B194&amp;"|"&amp;C194,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J194" s="13">
@@ -8746,7 +8746,7 @@
         <v/>
       </c>
       <c r="I195" s="10">
-        <f>IF(OR(B195="",C195=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B195&amp;"|"&amp;C195,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B195="",C195=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B195&amp;"|"&amp;C195,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J195" s="13">
@@ -8774,7 +8774,7 @@
         <v/>
       </c>
       <c r="I196" s="10">
-        <f>IF(OR(B196="",C196=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B196&amp;"|"&amp;C196,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B196="",C196=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B196&amp;"|"&amp;C196,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J196" s="13">
@@ -8802,7 +8802,7 @@
         <v/>
       </c>
       <c r="I197" s="10">
-        <f>IF(OR(B197="",C197=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B197&amp;"|"&amp;C197,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B197="",C197=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B197&amp;"|"&amp;C197,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J197" s="13">
@@ -8830,7 +8830,7 @@
         <v/>
       </c>
       <c r="I198" s="10">
-        <f>IF(OR(B198="",C198=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B198&amp;"|"&amp;C198,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B198="",C198=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B198&amp;"|"&amp;C198,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J198" s="13">
@@ -8858,7 +8858,7 @@
         <v/>
       </c>
       <c r="I199" s="10">
-        <f>IF(OR(B199="",C199=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B199&amp;"|"&amp;C199,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B199="",C199=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B199&amp;"|"&amp;C199,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J199" s="13">
@@ -8886,7 +8886,7 @@
         <v/>
       </c>
       <c r="I200" s="10">
-        <f>IF(OR(B200="",C200=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B200&amp;"|"&amp;C200,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B200="",C200=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B200&amp;"|"&amp;C200,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J200" s="13">
@@ -8914,7 +8914,7 @@
         <v/>
       </c>
       <c r="I201" s="10">
-        <f>IF(OR(B201="",C201=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B201&amp;"|"&amp;C201,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B201="",C201=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B201&amp;"|"&amp;C201,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J201" s="13">
@@ -8942,7 +8942,7 @@
         <v/>
       </c>
       <c r="I202" s="10">
-        <f>IF(OR(B202="",C202=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B202&amp;"|"&amp;C202,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B202="",C202=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B202&amp;"|"&amp;C202,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J202" s="13">
@@ -8970,7 +8970,7 @@
         <v/>
       </c>
       <c r="I203" s="10">
-        <f>IF(OR(B203="",C203=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B203&amp;"|"&amp;C203,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B203="",C203=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B203&amp;"|"&amp;C203,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J203" s="13">
@@ -8998,7 +8998,7 @@
         <v/>
       </c>
       <c r="I204" s="10">
-        <f>IF(OR(B204="",C204=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B204&amp;"|"&amp;C204,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B204="",C204=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B204&amp;"|"&amp;C204,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J204" s="13">
@@ -9026,7 +9026,7 @@
         <v/>
       </c>
       <c r="I205" s="10">
-        <f>IF(OR(B205="",C205=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B205&amp;"|"&amp;C205,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B205="",C205=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B205&amp;"|"&amp;C205,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J205" s="13">
@@ -9054,7 +9054,7 @@
         <v/>
       </c>
       <c r="I206" s="10">
-        <f>IF(OR(B206="",C206=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B206&amp;"|"&amp;C206,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B206="",C206=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B206&amp;"|"&amp;C206,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J206" s="13">
@@ -9082,7 +9082,7 @@
         <v/>
       </c>
       <c r="I207" s="10">
-        <f>IF(OR(B207="",C207=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B207&amp;"|"&amp;C207,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B207="",C207=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B207&amp;"|"&amp;C207,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J207" s="13">
@@ -9110,7 +9110,7 @@
         <v/>
       </c>
       <c r="I208" s="10">
-        <f>IF(OR(B208="",C208=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B208&amp;"|"&amp;C208,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B208="",C208=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B208&amp;"|"&amp;C208,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J208" s="13">
@@ -9138,7 +9138,7 @@
         <v/>
       </c>
       <c r="I209" s="10">
-        <f>IF(OR(B209="",C209=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B209&amp;"|"&amp;C209,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B209="",C209=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B209&amp;"|"&amp;C209,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J209" s="13">
@@ -9166,7 +9166,7 @@
         <v/>
       </c>
       <c r="I210" s="10">
-        <f>IF(OR(B210="",C210=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B210&amp;"|"&amp;C210,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B210="",C210=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B210&amp;"|"&amp;C210,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J210" s="13">
@@ -9194,7 +9194,7 @@
         <v/>
       </c>
       <c r="I211" s="10">
-        <f>IF(OR(B211="",C211=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B211&amp;"|"&amp;C211,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B211="",C211=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B211&amp;"|"&amp;C211,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J211" s="13">
@@ -9222,7 +9222,7 @@
         <v/>
       </c>
       <c r="I212" s="10">
-        <f>IF(OR(B212="",C212=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B212&amp;"|"&amp;C212,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B212="",C212=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B212&amp;"|"&amp;C212,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J212" s="13">
@@ -9250,7 +9250,7 @@
         <v/>
       </c>
       <c r="I213" s="10">
-        <f>IF(OR(B213="",C213=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B213&amp;"|"&amp;C213,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B213="",C213=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B213&amp;"|"&amp;C213,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J213" s="13">
@@ -9278,7 +9278,7 @@
         <v/>
       </c>
       <c r="I214" s="10">
-        <f>IF(OR(B214="",C214=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B214&amp;"|"&amp;C214,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B214="",C214=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B214&amp;"|"&amp;C214,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J214" s="13">
@@ -9306,7 +9306,7 @@
         <v/>
       </c>
       <c r="I215" s="10">
-        <f>IF(OR(B215="",C215=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B215&amp;"|"&amp;C215,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B215="",C215=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B215&amp;"|"&amp;C215,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J215" s="13">
@@ -9334,7 +9334,7 @@
         <v/>
       </c>
       <c r="I216" s="10">
-        <f>IF(OR(B216="",C216=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B216&amp;"|"&amp;C216,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B216="",C216=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B216&amp;"|"&amp;C216,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J216" s="13">
@@ -9362,7 +9362,7 @@
         <v/>
       </c>
       <c r="I217" s="10">
-        <f>IF(OR(B217="",C217=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B217&amp;"|"&amp;C217,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B217="",C217=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B217&amp;"|"&amp;C217,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J217" s="13">
@@ -9390,7 +9390,7 @@
         <v/>
       </c>
       <c r="I218" s="10">
-        <f>IF(OR(B218="",C218=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B218&amp;"|"&amp;C218,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B218="",C218=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B218&amp;"|"&amp;C218,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J218" s="13">
@@ -9418,7 +9418,7 @@
         <v/>
       </c>
       <c r="I219" s="10">
-        <f>IF(OR(B219="",C219=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B219&amp;"|"&amp;C219,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B219="",C219=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B219&amp;"|"&amp;C219,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J219" s="13">
@@ -9446,7 +9446,7 @@
         <v/>
       </c>
       <c r="I220" s="10">
-        <f>IF(OR(B220="",C220=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B220&amp;"|"&amp;C220,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B220="",C220=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B220&amp;"|"&amp;C220,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J220" s="13">
@@ -9474,7 +9474,7 @@
         <v/>
       </c>
       <c r="I221" s="10">
-        <f>IF(OR(B221="",C221=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B221&amp;"|"&amp;C221,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B221="",C221=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B221&amp;"|"&amp;C221,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J221" s="13">
@@ -9502,7 +9502,7 @@
         <v/>
       </c>
       <c r="I222" s="10">
-        <f>IF(OR(B222="",C222=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B222&amp;"|"&amp;C222,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B222="",C222=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B222&amp;"|"&amp;C222,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J222" s="13">
@@ -9530,7 +9530,7 @@
         <v/>
       </c>
       <c r="I223" s="10">
-        <f>IF(OR(B223="",C223=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B223&amp;"|"&amp;C223,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B223="",C223=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B223&amp;"|"&amp;C223,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J223" s="13">
@@ -9558,7 +9558,7 @@
         <v/>
       </c>
       <c r="I224" s="10">
-        <f>IF(OR(B224="",C224=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B224&amp;"|"&amp;C224,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B224="",C224=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B224&amp;"|"&amp;C224,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J224" s="13">
@@ -9586,7 +9586,7 @@
         <v/>
       </c>
       <c r="I225" s="10">
-        <f>IF(OR(B225="",C225=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B225&amp;"|"&amp;C225,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B225="",C225=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B225&amp;"|"&amp;C225,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J225" s="13">
@@ -9614,7 +9614,7 @@
         <v/>
       </c>
       <c r="I226" s="10">
-        <f>IF(OR(B226="",C226=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B226&amp;"|"&amp;C226,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B226="",C226=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B226&amp;"|"&amp;C226,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J226" s="13">
@@ -9642,7 +9642,7 @@
         <v/>
       </c>
       <c r="I227" s="10">
-        <f>IF(OR(B227="",C227=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B227&amp;"|"&amp;C227,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B227="",C227=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B227&amp;"|"&amp;C227,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J227" s="13">
@@ -9670,7 +9670,7 @@
         <v/>
       </c>
       <c r="I228" s="10">
-        <f>IF(OR(B228="",C228=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B228&amp;"|"&amp;C228,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B228="",C228=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B228&amp;"|"&amp;C228,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J228" s="13">
@@ -9698,7 +9698,7 @@
         <v/>
       </c>
       <c r="I229" s="10">
-        <f>IF(OR(B229="",C229=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B229&amp;"|"&amp;C229,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B229="",C229=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B229&amp;"|"&amp;C229,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J229" s="13">
@@ -9726,7 +9726,7 @@
         <v/>
       </c>
       <c r="I230" s="10">
-        <f>IF(OR(B230="",C230=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B230&amp;"|"&amp;C230,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B230="",C230=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B230&amp;"|"&amp;C230,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J230" s="13">
@@ -9754,7 +9754,7 @@
         <v/>
       </c>
       <c r="I231" s="10">
-        <f>IF(OR(B231="",C231=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B231&amp;"|"&amp;C231,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B231="",C231=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B231&amp;"|"&amp;C231,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J231" s="13">
@@ -9782,7 +9782,7 @@
         <v/>
       </c>
       <c r="I232" s="10">
-        <f>IF(OR(B232="",C232=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B232&amp;"|"&amp;C232,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B232="",C232=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B232&amp;"|"&amp;C232,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J232" s="13">
@@ -9810,7 +9810,7 @@
         <v/>
       </c>
       <c r="I233" s="10">
-        <f>IF(OR(B233="",C233=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B233&amp;"|"&amp;C233,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B233="",C233=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B233&amp;"|"&amp;C233,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J233" s="13">
@@ -9838,7 +9838,7 @@
         <v/>
       </c>
       <c r="I234" s="10">
-        <f>IF(OR(B234="",C234=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B234&amp;"|"&amp;C234,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B234="",C234=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B234&amp;"|"&amp;C234,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J234" s="13">
@@ -9866,7 +9866,7 @@
         <v/>
       </c>
       <c r="I235" s="10">
-        <f>IF(OR(B235="",C235=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B235&amp;"|"&amp;C235,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B235="",C235=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B235&amp;"|"&amp;C235,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J235" s="13">
@@ -9894,7 +9894,7 @@
         <v/>
       </c>
       <c r="I236" s="10">
-        <f>IF(OR(B236="",C236=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B236&amp;"|"&amp;C236,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B236="",C236=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B236&amp;"|"&amp;C236,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J236" s="13">
@@ -9922,7 +9922,7 @@
         <v/>
       </c>
       <c r="I237" s="10">
-        <f>IF(OR(B237="",C237=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B237&amp;"|"&amp;C237,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B237="",C237=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B237&amp;"|"&amp;C237,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J237" s="13">
@@ -9950,7 +9950,7 @@
         <v/>
       </c>
       <c r="I238" s="10">
-        <f>IF(OR(B238="",C238=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B238&amp;"|"&amp;C238,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B238="",C238=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B238&amp;"|"&amp;C238,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J238" s="13">
@@ -9978,7 +9978,7 @@
         <v/>
       </c>
       <c r="I239" s="10">
-        <f>IF(OR(B239="",C239=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B239&amp;"|"&amp;C239,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B239="",C239=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B239&amp;"|"&amp;C239,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J239" s="13">
@@ -10006,7 +10006,7 @@
         <v/>
       </c>
       <c r="I240" s="10">
-        <f>IF(OR(B240="",C240=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B240&amp;"|"&amp;C240,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B240="",C240=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B240&amp;"|"&amp;C240,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J240" s="13">
@@ -10034,7 +10034,7 @@
         <v/>
       </c>
       <c r="I241" s="10">
-        <f>IF(OR(B241="",C241=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B241&amp;"|"&amp;C241,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B241="",C241=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B241&amp;"|"&amp;C241,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J241" s="13">
@@ -10062,7 +10062,7 @@
         <v/>
       </c>
       <c r="I242" s="10">
-        <f>IF(OR(B242="",C242=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B242&amp;"|"&amp;C242,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B242="",C242=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B242&amp;"|"&amp;C242,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J242" s="13">
@@ -10090,7 +10090,7 @@
         <v/>
       </c>
       <c r="I243" s="10">
-        <f>IF(OR(B243="",C243=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B243&amp;"|"&amp;C243,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B243="",C243=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B243&amp;"|"&amp;C243,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J243" s="13">
@@ -10118,7 +10118,7 @@
         <v/>
       </c>
       <c r="I244" s="10">
-        <f>IF(OR(B244="",C244=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B244&amp;"|"&amp;C244,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B244="",C244=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B244&amp;"|"&amp;C244,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J244" s="13">
@@ -10146,7 +10146,7 @@
         <v/>
       </c>
       <c r="I245" s="10">
-        <f>IF(OR(B245="",C245=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B245&amp;"|"&amp;C245,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B245="",C245=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B245&amp;"|"&amp;C245,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J245" s="13">
@@ -10174,7 +10174,7 @@
         <v/>
       </c>
       <c r="I246" s="10">
-        <f>IF(OR(B246="",C246=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B246&amp;"|"&amp;C246,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B246="",C246=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B246&amp;"|"&amp;C246,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J246" s="13">
@@ -10202,7 +10202,7 @@
         <v/>
       </c>
       <c r="I247" s="10">
-        <f>IF(OR(B247="",C247=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B247&amp;"|"&amp;C247,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B247="",C247=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B247&amp;"|"&amp;C247,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J247" s="13">
@@ -10230,7 +10230,7 @@
         <v/>
       </c>
       <c r="I248" s="10">
-        <f>IF(OR(B248="",C248=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B248&amp;"|"&amp;C248,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B248="",C248=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B248&amp;"|"&amp;C248,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J248" s="13">
@@ -10258,7 +10258,7 @@
         <v/>
       </c>
       <c r="I249" s="10">
-        <f>IF(OR(B249="",C249=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B249&amp;"|"&amp;C249,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B249="",C249=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B249&amp;"|"&amp;C249,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J249" s="13">
@@ -10286,7 +10286,7 @@
         <v/>
       </c>
       <c r="I250" s="10">
-        <f>IF(OR(B250="",C250=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B250&amp;"|"&amp;C250,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B250="",C250=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B250&amp;"|"&amp;C250,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J250" s="13">
@@ -10314,7 +10314,7 @@
         <v/>
       </c>
       <c r="I251" s="10">
-        <f>IF(OR(B251="",C251=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B251&amp;"|"&amp;C251,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B251="",C251=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B251&amp;"|"&amp;C251,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J251" s="13">
@@ -10342,7 +10342,7 @@
         <v/>
       </c>
       <c r="I252" s="10">
-        <f>IF(OR(B252="",C252=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B252&amp;"|"&amp;C252,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B252="",C252=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B252&amp;"|"&amp;C252,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J252" s="13">
@@ -10370,7 +10370,7 @@
         <v/>
       </c>
       <c r="I253" s="10">
-        <f>IF(OR(B253="",C253=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B253&amp;"|"&amp;C253,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B253="",C253=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B253&amp;"|"&amp;C253,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J253" s="13">
@@ -10398,7 +10398,7 @@
         <v/>
       </c>
       <c r="I254" s="10">
-        <f>IF(OR(B254="",C254=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B254&amp;"|"&amp;C254,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B254="",C254=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B254&amp;"|"&amp;C254,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J254" s="13">
@@ -10426,7 +10426,7 @@
         <v/>
       </c>
       <c r="I255" s="10">
-        <f>IF(OR(B255="",C255=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B255&amp;"|"&amp;C255,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B255="",C255=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B255&amp;"|"&amp;C255,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J255" s="13">
@@ -10454,7 +10454,7 @@
         <v/>
       </c>
       <c r="I256" s="10">
-        <f>IF(OR(B256="",C256=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B256&amp;"|"&amp;C256,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B256="",C256=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B256&amp;"|"&amp;C256,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J256" s="13">
@@ -10482,7 +10482,7 @@
         <v/>
       </c>
       <c r="I257" s="10">
-        <f>IF(OR(B257="",C257=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B257&amp;"|"&amp;C257,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B257="",C257=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B257&amp;"|"&amp;C257,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J257" s="13">
@@ -10510,7 +10510,7 @@
         <v/>
       </c>
       <c r="I258" s="10">
-        <f>IF(OR(B258="",C258=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B258&amp;"|"&amp;C258,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B258="",C258=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B258&amp;"|"&amp;C258,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J258" s="13">
@@ -10538,7 +10538,7 @@
         <v/>
       </c>
       <c r="I259" s="10">
-        <f>IF(OR(B259="",C259=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B259&amp;"|"&amp;C259,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B259="",C259=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B259&amp;"|"&amp;C259,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J259" s="13">
@@ -10566,7 +10566,7 @@
         <v/>
       </c>
       <c r="I260" s="10">
-        <f>IF(OR(B260="",C260=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B260&amp;"|"&amp;C260,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B260="",C260=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B260&amp;"|"&amp;C260,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J260" s="13">
@@ -10594,7 +10594,7 @@
         <v/>
       </c>
       <c r="I261" s="10">
-        <f>IF(OR(B261="",C261=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B261&amp;"|"&amp;C261,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B261="",C261=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B261&amp;"|"&amp;C261,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J261" s="13">
@@ -10622,7 +10622,7 @@
         <v/>
       </c>
       <c r="I262" s="10">
-        <f>IF(OR(B262="",C262=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B262&amp;"|"&amp;C262,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B262="",C262=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B262&amp;"|"&amp;C262,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J262" s="13">
@@ -10650,7 +10650,7 @@
         <v/>
       </c>
       <c r="I263" s="10">
-        <f>IF(OR(B263="",C263=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B263&amp;"|"&amp;C263,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B263="",C263=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B263&amp;"|"&amp;C263,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J263" s="13">
@@ -10678,7 +10678,7 @@
         <v/>
       </c>
       <c r="I264" s="10">
-        <f>IF(OR(B264="",C264=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B264&amp;"|"&amp;C264,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B264="",C264=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B264&amp;"|"&amp;C264,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J264" s="13">
@@ -10706,7 +10706,7 @@
         <v/>
       </c>
       <c r="I265" s="10">
-        <f>IF(OR(B265="",C265=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B265&amp;"|"&amp;C265,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B265="",C265=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B265&amp;"|"&amp;C265,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J265" s="13">
@@ -10734,7 +10734,7 @@
         <v/>
       </c>
       <c r="I266" s="10">
-        <f>IF(OR(B266="",C266=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B266&amp;"|"&amp;C266,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B266="",C266=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B266&amp;"|"&amp;C266,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J266" s="13">
@@ -10762,7 +10762,7 @@
         <v/>
       </c>
       <c r="I267" s="10">
-        <f>IF(OR(B267="",C267=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B267&amp;"|"&amp;C267,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B267="",C267=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B267&amp;"|"&amp;C267,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J267" s="13">
@@ -10790,7 +10790,7 @@
         <v/>
       </c>
       <c r="I268" s="10">
-        <f>IF(OR(B268="",C268=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B268&amp;"|"&amp;C268,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B268="",C268=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B268&amp;"|"&amp;C268,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J268" s="13">
@@ -10818,7 +10818,7 @@
         <v/>
       </c>
       <c r="I269" s="10">
-        <f>IF(OR(B269="",C269=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B269&amp;"|"&amp;C269,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B269="",C269=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B269&amp;"|"&amp;C269,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J269" s="13">
@@ -10846,7 +10846,7 @@
         <v/>
       </c>
       <c r="I270" s="10">
-        <f>IF(OR(B270="",C270=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B270&amp;"|"&amp;C270,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B270="",C270=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B270&amp;"|"&amp;C270,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J270" s="13">
@@ -10874,7 +10874,7 @@
         <v/>
       </c>
       <c r="I271" s="10">
-        <f>IF(OR(B271="",C271=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B271&amp;"|"&amp;C271,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B271="",C271=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B271&amp;"|"&amp;C271,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J271" s="13">
@@ -10902,7 +10902,7 @@
         <v/>
       </c>
       <c r="I272" s="10">
-        <f>IF(OR(B272="",C272=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B272&amp;"|"&amp;C272,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B272="",C272=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B272&amp;"|"&amp;C272,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J272" s="13">
@@ -10930,7 +10930,7 @@
         <v/>
       </c>
       <c r="I273" s="10">
-        <f>IF(OR(B273="",C273=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B273&amp;"|"&amp;C273,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B273="",C273=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B273&amp;"|"&amp;C273,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J273" s="13">
@@ -10958,7 +10958,7 @@
         <v/>
       </c>
       <c r="I274" s="10">
-        <f>IF(OR(B274="",C274=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B274&amp;"|"&amp;C274,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B274="",C274=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B274&amp;"|"&amp;C274,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J274" s="13">
@@ -10986,7 +10986,7 @@
         <v/>
       </c>
       <c r="I275" s="10">
-        <f>IF(OR(B275="",C275=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B275&amp;"|"&amp;C275,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B275="",C275=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B275&amp;"|"&amp;C275,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J275" s="13">
@@ -11014,7 +11014,7 @@
         <v/>
       </c>
       <c r="I276" s="10">
-        <f>IF(OR(B276="",C276=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B276&amp;"|"&amp;C276,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B276="",C276=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B276&amp;"|"&amp;C276,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J276" s="13">
@@ -11042,7 +11042,7 @@
         <v/>
       </c>
       <c r="I277" s="10">
-        <f>IF(OR(B277="",C277=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B277&amp;"|"&amp;C277,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B277="",C277=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B277&amp;"|"&amp;C277,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J277" s="13">
@@ -11070,7 +11070,7 @@
         <v/>
       </c>
       <c r="I278" s="10">
-        <f>IF(OR(B278="",C278=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B278&amp;"|"&amp;C278,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B278="",C278=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B278&amp;"|"&amp;C278,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J278" s="13">
@@ -11098,7 +11098,7 @@
         <v/>
       </c>
       <c r="I279" s="10">
-        <f>IF(OR(B279="",C279=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B279&amp;"|"&amp;C279,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B279="",C279=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B279&amp;"|"&amp;C279,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J279" s="13">
@@ -11126,7 +11126,7 @@
         <v/>
       </c>
       <c r="I280" s="10">
-        <f>IF(OR(B280="",C280=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B280&amp;"|"&amp;C280,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B280="",C280=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B280&amp;"|"&amp;C280,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J280" s="13">
@@ -11154,7 +11154,7 @@
         <v/>
       </c>
       <c r="I281" s="10">
-        <f>IF(OR(B281="",C281=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B281&amp;"|"&amp;C281,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B281="",C281=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B281&amp;"|"&amp;C281,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J281" s="13">
@@ -11182,7 +11182,7 @@
         <v/>
       </c>
       <c r="I282" s="10">
-        <f>IF(OR(B282="",C282=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B282&amp;"|"&amp;C282,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B282="",C282=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B282&amp;"|"&amp;C282,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J282" s="13">
@@ -11210,7 +11210,7 @@
         <v/>
       </c>
       <c r="I283" s="10">
-        <f>IF(OR(B283="",C283=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B283&amp;"|"&amp;C283,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B283="",C283=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B283&amp;"|"&amp;C283,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J283" s="13">
@@ -11238,7 +11238,7 @@
         <v/>
       </c>
       <c r="I284" s="10">
-        <f>IF(OR(B284="",C284=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B284&amp;"|"&amp;C284,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B284="",C284=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B284&amp;"|"&amp;C284,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J284" s="13">
@@ -11266,7 +11266,7 @@
         <v/>
       </c>
       <c r="I285" s="10">
-        <f>IF(OR(B285="",C285=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B285&amp;"|"&amp;C285,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B285="",C285=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B285&amp;"|"&amp;C285,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J285" s="13">
@@ -11294,7 +11294,7 @@
         <v/>
       </c>
       <c r="I286" s="10">
-        <f>IF(OR(B286="",C286=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B286&amp;"|"&amp;C286,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B286="",C286=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B286&amp;"|"&amp;C286,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J286" s="13">
@@ -11322,7 +11322,7 @@
         <v/>
       </c>
       <c r="I287" s="10">
-        <f>IF(OR(B287="",C287=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B287&amp;"|"&amp;C287,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B287="",C287=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B287&amp;"|"&amp;C287,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J287" s="13">
@@ -11350,7 +11350,7 @@
         <v/>
       </c>
       <c r="I288" s="10">
-        <f>IF(OR(B288="",C288=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B288&amp;"|"&amp;C288,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B288="",C288=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B288&amp;"|"&amp;C288,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J288" s="13">
@@ -11378,7 +11378,7 @@
         <v/>
       </c>
       <c r="I289" s="10">
-        <f>IF(OR(B289="",C289=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B289&amp;"|"&amp;C289,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B289="",C289=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B289&amp;"|"&amp;C289,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J289" s="13">
@@ -11406,7 +11406,7 @@
         <v/>
       </c>
       <c r="I290" s="10">
-        <f>IF(OR(B290="",C290=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B290&amp;"|"&amp;C290,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B290="",C290=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B290&amp;"|"&amp;C290,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J290" s="13">
@@ -11434,7 +11434,7 @@
         <v/>
       </c>
       <c r="I291" s="10">
-        <f>IF(OR(B291="",C291=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B291&amp;"|"&amp;C291,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B291="",C291=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B291&amp;"|"&amp;C291,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J291" s="13">
@@ -11462,7 +11462,7 @@
         <v/>
       </c>
       <c r="I292" s="10">
-        <f>IF(OR(B292="",C292=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B292&amp;"|"&amp;C292,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B292="",C292=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B292&amp;"|"&amp;C292,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J292" s="13">
@@ -11490,7 +11490,7 @@
         <v/>
       </c>
       <c r="I293" s="10">
-        <f>IF(OR(B293="",C293=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B293&amp;"|"&amp;C293,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B293="",C293=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B293&amp;"|"&amp;C293,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J293" s="13">
@@ -11518,7 +11518,7 @@
         <v/>
       </c>
       <c r="I294" s="10">
-        <f>IF(OR(B294="",C294=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B294&amp;"|"&amp;C294,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B294="",C294=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B294&amp;"|"&amp;C294,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J294" s="13">
@@ -11546,7 +11546,7 @@
         <v/>
       </c>
       <c r="I295" s="10">
-        <f>IF(OR(B295="",C295=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B295&amp;"|"&amp;C295,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B295="",C295=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B295&amp;"|"&amp;C295,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J295" s="13">
@@ -11574,7 +11574,7 @@
         <v/>
       </c>
       <c r="I296" s="10">
-        <f>IF(OR(B296="",C296=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B296&amp;"|"&amp;C296,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B296="",C296=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B296&amp;"|"&amp;C296,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J296" s="13">
@@ -11602,7 +11602,7 @@
         <v/>
       </c>
       <c r="I297" s="10">
-        <f>IF(OR(B297="",C297=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B297&amp;"|"&amp;C297,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B297="",C297=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B297&amp;"|"&amp;C297,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J297" s="13">
@@ -11630,7 +11630,7 @@
         <v/>
       </c>
       <c r="I298" s="10">
-        <f>IF(OR(B298="",C298=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B298&amp;"|"&amp;C298,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B298="",C298=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B298&amp;"|"&amp;C298,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J298" s="13">
@@ -11658,7 +11658,7 @@
         <v/>
       </c>
       <c r="I299" s="10">
-        <f>IF(OR(B299="",C299=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B299&amp;"|"&amp;C299,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B299="",C299=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B299&amp;"|"&amp;C299,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J299" s="13">
@@ -11686,7 +11686,7 @@
         <v/>
       </c>
       <c r="I300" s="10">
-        <f>IF(OR(B300="",C300=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B300&amp;"|"&amp;C300,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B300="",C300=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B300&amp;"|"&amp;C300,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J300" s="13">
@@ -11714,7 +11714,7 @@
         <v/>
       </c>
       <c r="I301" s="10">
-        <f>IF(OR(B301="",C301=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B301&amp;"|"&amp;C301,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B301="",C301=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B301&amp;"|"&amp;C301,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J301" s="13">
@@ -11742,7 +11742,7 @@
         <v/>
       </c>
       <c r="I302" s="10">
-        <f>IF(OR(B302="",C302=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B302&amp;"|"&amp;C302,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B302="",C302=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B302&amp;"|"&amp;C302,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J302" s="13">
@@ -11770,7 +11770,7 @@
         <v/>
       </c>
       <c r="I303" s="10">
-        <f>IF(OR(B303="",C303=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B303&amp;"|"&amp;C303,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B303="",C303=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B303&amp;"|"&amp;C303,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J303" s="13">
@@ -11798,7 +11798,7 @@
         <v/>
       </c>
       <c r="I304" s="10">
-        <f>IF(OR(B304="",C304=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B304&amp;"|"&amp;C304,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B304="",C304=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B304&amp;"|"&amp;C304,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J304" s="13">
@@ -11826,7 +11826,7 @@
         <v/>
       </c>
       <c r="I305" s="10">
-        <f>IF(OR(B305="",C305=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B305&amp;"|"&amp;C305,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B305="",C305=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B305&amp;"|"&amp;C305,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J305" s="13">
@@ -11854,7 +11854,7 @@
         <v/>
       </c>
       <c r="I306" s="10">
-        <f>IF(OR(B306="",C306=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B306&amp;"|"&amp;C306,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B306="",C306=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B306&amp;"|"&amp;C306,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J306" s="13">
@@ -11882,7 +11882,7 @@
         <v/>
       </c>
       <c r="I307" s="10">
-        <f>IF(OR(B307="",C307=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B307&amp;"|"&amp;C307,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B307="",C307=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B307&amp;"|"&amp;C307,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J307" s="13">
@@ -11910,7 +11910,7 @@
         <v/>
       </c>
       <c r="I308" s="10">
-        <f>IF(OR(B308="",C308=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B308&amp;"|"&amp;C308,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B308="",C308=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B308&amp;"|"&amp;C308,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J308" s="13">
@@ -11938,7 +11938,7 @@
         <v/>
       </c>
       <c r="I309" s="10">
-        <f>IF(OR(B309="",C309=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B309&amp;"|"&amp;C309,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B309="",C309=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B309&amp;"|"&amp;C309,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J309" s="13">
@@ -11966,7 +11966,7 @@
         <v/>
       </c>
       <c r="I310" s="10">
-        <f>IF(OR(B310="",C310=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B310&amp;"|"&amp;C310,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B310="",C310=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B310&amp;"|"&amp;C310,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J310" s="13">
@@ -11994,7 +11994,7 @@
         <v/>
       </c>
       <c r="I311" s="10">
-        <f>IF(OR(B311="",C311=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B311&amp;"|"&amp;C311,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B311="",C311=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B311&amp;"|"&amp;C311,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J311" s="13">
@@ -12022,7 +12022,7 @@
         <v/>
       </c>
       <c r="I312" s="10">
-        <f>IF(OR(B312="",C312=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B312&amp;"|"&amp;C312,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B312="",C312=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B312&amp;"|"&amp;C312,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J312" s="13">
@@ -12050,7 +12050,7 @@
         <v/>
       </c>
       <c r="I313" s="10">
-        <f>IF(OR(B313="",C313=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B313&amp;"|"&amp;C313,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B313="",C313=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B313&amp;"|"&amp;C313,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J313" s="13">
@@ -12078,7 +12078,7 @@
         <v/>
       </c>
       <c r="I314" s="10">
-        <f>IF(OR(B314="",C314=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B314&amp;"|"&amp;C314,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B314="",C314=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B314&amp;"|"&amp;C314,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J314" s="13">
@@ -12106,7 +12106,7 @@
         <v/>
       </c>
       <c r="I315" s="10">
-        <f>IF(OR(B315="",C315=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B315&amp;"|"&amp;C315,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B315="",C315=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B315&amp;"|"&amp;C315,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J315" s="13">
@@ -12134,7 +12134,7 @@
         <v/>
       </c>
       <c r="I316" s="10">
-        <f>IF(OR(B316="",C316=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B316&amp;"|"&amp;C316,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B316="",C316=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B316&amp;"|"&amp;C316,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J316" s="13">
@@ -12162,7 +12162,7 @@
         <v/>
       </c>
       <c r="I317" s="10">
-        <f>IF(OR(B317="",C317=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B317&amp;"|"&amp;C317,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B317="",C317=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B317&amp;"|"&amp;C317,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J317" s="13">
@@ -12190,7 +12190,7 @@
         <v/>
       </c>
       <c r="I318" s="10">
-        <f>IF(OR(B318="",C318=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B318&amp;"|"&amp;C318,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B318="",C318=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B318&amp;"|"&amp;C318,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J318" s="13">
@@ -12218,7 +12218,7 @@
         <v/>
       </c>
       <c r="I319" s="10">
-        <f>IF(OR(B319="",C319=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B319&amp;"|"&amp;C319,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B319="",C319=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B319&amp;"|"&amp;C319,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J319" s="13">
@@ -12246,7 +12246,7 @@
         <v/>
       </c>
       <c r="I320" s="10">
-        <f>IF(OR(B320="",C320=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B320&amp;"|"&amp;C320,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B320="",C320=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B320&amp;"|"&amp;C320,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J320" s="13">
@@ -12274,7 +12274,7 @@
         <v/>
       </c>
       <c r="I321" s="10">
-        <f>IF(OR(B321="",C321=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B321&amp;"|"&amp;C321,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B321="",C321=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B321&amp;"|"&amp;C321,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J321" s="13">
@@ -12302,7 +12302,7 @@
         <v/>
       </c>
       <c r="I322" s="10">
-        <f>IF(OR(B322="",C322=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B322&amp;"|"&amp;C322,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B322="",C322=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B322&amp;"|"&amp;C322,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J322" s="13">
@@ -12330,7 +12330,7 @@
         <v/>
       </c>
       <c r="I323" s="10">
-        <f>IF(OR(B323="",C323=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B323&amp;"|"&amp;C323,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B323="",C323=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B323&amp;"|"&amp;C323,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J323" s="13">
@@ -12358,7 +12358,7 @@
         <v/>
       </c>
       <c r="I324" s="10">
-        <f>IF(OR(B324="",C324=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B324&amp;"|"&amp;C324,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B324="",C324=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B324&amp;"|"&amp;C324,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J324" s="13">
@@ -12386,7 +12386,7 @@
         <v/>
       </c>
       <c r="I325" s="10">
-        <f>IF(OR(B325="",C325=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B325&amp;"|"&amp;C325,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B325="",C325=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B325&amp;"|"&amp;C325,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J325" s="13">
@@ -12414,7 +12414,7 @@
         <v/>
       </c>
       <c r="I326" s="10">
-        <f>IF(OR(B326="",C326=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B326&amp;"|"&amp;C326,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B326="",C326=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B326&amp;"|"&amp;C326,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J326" s="13">
@@ -12442,7 +12442,7 @@
         <v/>
       </c>
       <c r="I327" s="10">
-        <f>IF(OR(B327="",C327=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B327&amp;"|"&amp;C327,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B327="",C327=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B327&amp;"|"&amp;C327,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J327" s="13">
@@ -12470,7 +12470,7 @@
         <v/>
       </c>
       <c r="I328" s="10">
-        <f>IF(OR(B328="",C328=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B328&amp;"|"&amp;C328,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B328="",C328=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B328&amp;"|"&amp;C328,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J328" s="13">
@@ -12498,7 +12498,7 @@
         <v/>
       </c>
       <c r="I329" s="10">
-        <f>IF(OR(B329="",C329=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B329&amp;"|"&amp;C329,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B329="",C329=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B329&amp;"|"&amp;C329,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J329" s="13">
@@ -12526,7 +12526,7 @@
         <v/>
       </c>
       <c r="I330" s="10">
-        <f>IF(OR(B330="",C330=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B330&amp;"|"&amp;C330,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B330="",C330=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B330&amp;"|"&amp;C330,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J330" s="13">
@@ -12554,7 +12554,7 @@
         <v/>
       </c>
       <c r="I331" s="10">
-        <f>IF(OR(B331="",C331=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B331&amp;"|"&amp;C331,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B331="",C331=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B331&amp;"|"&amp;C331,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J331" s="13">
@@ -12582,7 +12582,7 @@
         <v/>
       </c>
       <c r="I332" s="10">
-        <f>IF(OR(B332="",C332=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B332&amp;"|"&amp;C332,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B332="",C332=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B332&amp;"|"&amp;C332,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J332" s="13">
@@ -12610,7 +12610,7 @@
         <v/>
       </c>
       <c r="I333" s="10">
-        <f>IF(OR(B333="",C333=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B333&amp;"|"&amp;C333,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B333="",C333=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B333&amp;"|"&amp;C333,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J333" s="13">
@@ -12638,7 +12638,7 @@
         <v/>
       </c>
       <c r="I334" s="10">
-        <f>IF(OR(B334="",C334=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B334&amp;"|"&amp;C334,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B334="",C334=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B334&amp;"|"&amp;C334,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J334" s="13">
@@ -12666,7 +12666,7 @@
         <v/>
       </c>
       <c r="I335" s="10">
-        <f>IF(OR(B335="",C335=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B335&amp;"|"&amp;C335,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B335="",C335=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B335&amp;"|"&amp;C335,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J335" s="13">
@@ -12694,7 +12694,7 @@
         <v/>
       </c>
       <c r="I336" s="10">
-        <f>IF(OR(B336="",C336=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B336&amp;"|"&amp;C336,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B336="",C336=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B336&amp;"|"&amp;C336,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J336" s="13">
@@ -12722,7 +12722,7 @@
         <v/>
       </c>
       <c r="I337" s="10">
-        <f>IF(OR(B337="",C337=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B337&amp;"|"&amp;C337,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B337="",C337=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B337&amp;"|"&amp;C337,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J337" s="13">
@@ -12750,7 +12750,7 @@
         <v/>
       </c>
       <c r="I338" s="10">
-        <f>IF(OR(B338="",C338=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B338&amp;"|"&amp;C338,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B338="",C338=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B338&amp;"|"&amp;C338,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J338" s="13">
@@ -12778,7 +12778,7 @@
         <v/>
       </c>
       <c r="I339" s="10">
-        <f>IF(OR(B339="",C339=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B339&amp;"|"&amp;C339,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B339="",C339=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B339&amp;"|"&amp;C339,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J339" s="13">
@@ -12806,7 +12806,7 @@
         <v/>
       </c>
       <c r="I340" s="10">
-        <f>IF(OR(B340="",C340=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B340&amp;"|"&amp;C340,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B340="",C340=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B340&amp;"|"&amp;C340,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J340" s="13">
@@ -12834,7 +12834,7 @@
         <v/>
       </c>
       <c r="I341" s="10">
-        <f>IF(OR(B341="",C341=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B341&amp;"|"&amp;C341,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B341="",C341=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B341&amp;"|"&amp;C341,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J341" s="13">
@@ -12862,7 +12862,7 @@
         <v/>
       </c>
       <c r="I342" s="10">
-        <f>IF(OR(B342="",C342=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B342&amp;"|"&amp;C342,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B342="",C342=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B342&amp;"|"&amp;C342,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J342" s="13">
@@ -12890,7 +12890,7 @@
         <v/>
       </c>
       <c r="I343" s="10">
-        <f>IF(OR(B343="",C343=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B343&amp;"|"&amp;C343,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B343="",C343=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B343&amp;"|"&amp;C343,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J343" s="13">
@@ -12918,7 +12918,7 @@
         <v/>
       </c>
       <c r="I344" s="10">
-        <f>IF(OR(B344="",C344=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B344&amp;"|"&amp;C344,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B344="",C344=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B344&amp;"|"&amp;C344,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J344" s="13">
@@ -12946,7 +12946,7 @@
         <v/>
       </c>
       <c r="I345" s="10">
-        <f>IF(OR(B345="",C345=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B345&amp;"|"&amp;C345,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B345="",C345=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B345&amp;"|"&amp;C345,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J345" s="13">
@@ -12974,7 +12974,7 @@
         <v/>
       </c>
       <c r="I346" s="10">
-        <f>IF(OR(B346="",C346=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B346&amp;"|"&amp;C346,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B346="",C346=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B346&amp;"|"&amp;C346,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J346" s="13">
@@ -13002,7 +13002,7 @@
         <v/>
       </c>
       <c r="I347" s="10">
-        <f>IF(OR(B347="",C347=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B347&amp;"|"&amp;C347,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B347="",C347=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B347&amp;"|"&amp;C347,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J347" s="13">
@@ -13030,7 +13030,7 @@
         <v/>
       </c>
       <c r="I348" s="10">
-        <f>IF(OR(B348="",C348=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B348&amp;"|"&amp;C348,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B348="",C348=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B348&amp;"|"&amp;C348,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J348" s="13">
@@ -13058,7 +13058,7 @@
         <v/>
       </c>
       <c r="I349" s="10">
-        <f>IF(OR(B349="",C349=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B349&amp;"|"&amp;C349,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B349="",C349=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B349&amp;"|"&amp;C349,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J349" s="13">
@@ -13086,7 +13086,7 @@
         <v/>
       </c>
       <c r="I350" s="10">
-        <f>IF(OR(B350="",C350=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B350&amp;"|"&amp;C350,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B350="",C350=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B350&amp;"|"&amp;C350,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J350" s="13">
@@ -13114,7 +13114,7 @@
         <v/>
       </c>
       <c r="I351" s="10">
-        <f>IF(OR(B351="",C351=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B351&amp;"|"&amp;C351,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B351="",C351=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B351&amp;"|"&amp;C351,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J351" s="13">
@@ -13142,7 +13142,7 @@
         <v/>
       </c>
       <c r="I352" s="10">
-        <f>IF(OR(B352="",C352=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B352&amp;"|"&amp;C352,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B352="",C352=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B352&amp;"|"&amp;C352,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J352" s="13">
@@ -13170,7 +13170,7 @@
         <v/>
       </c>
       <c r="I353" s="10">
-        <f>IF(OR(B353="",C353=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B353&amp;"|"&amp;C353,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B353="",C353=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B353&amp;"|"&amp;C353,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J353" s="13">
@@ -13198,7 +13198,7 @@
         <v/>
       </c>
       <c r="I354" s="10">
-        <f>IF(OR(B354="",C354=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B354&amp;"|"&amp;C354,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B354="",C354=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B354&amp;"|"&amp;C354,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J354" s="13">
@@ -13226,7 +13226,7 @@
         <v/>
       </c>
       <c r="I355" s="10">
-        <f>IF(OR(B355="",C355=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B355&amp;"|"&amp;C355,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B355="",C355=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B355&amp;"|"&amp;C355,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J355" s="13">
@@ -13254,7 +13254,7 @@
         <v/>
       </c>
       <c r="I356" s="10">
-        <f>IF(OR(B356="",C356=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B356&amp;"|"&amp;C356,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B356="",C356=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B356&amp;"|"&amp;C356,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J356" s="13">
@@ -13282,7 +13282,7 @@
         <v/>
       </c>
       <c r="I357" s="10">
-        <f>IF(OR(B357="",C357=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B357&amp;"|"&amp;C357,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B357="",C357=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B357&amp;"|"&amp;C357,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J357" s="13">
@@ -13310,7 +13310,7 @@
         <v/>
       </c>
       <c r="I358" s="10">
-        <f>IF(OR(B358="",C358=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B358&amp;"|"&amp;C358,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B358="",C358=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B358&amp;"|"&amp;C358,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J358" s="13">
@@ -13338,7 +13338,7 @@
         <v/>
       </c>
       <c r="I359" s="10">
-        <f>IF(OR(B359="",C359=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B359&amp;"|"&amp;C359,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B359="",C359=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B359&amp;"|"&amp;C359,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J359" s="13">
@@ -13366,7 +13366,7 @@
         <v/>
       </c>
       <c r="I360" s="10">
-        <f>IF(OR(B360="",C360=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B360&amp;"|"&amp;C360,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B360="",C360=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B360&amp;"|"&amp;C360,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J360" s="13">
@@ -13394,7 +13394,7 @@
         <v/>
       </c>
       <c r="I361" s="10">
-        <f>IF(OR(B361="",C361=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B361&amp;"|"&amp;C361,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B361="",C361=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B361&amp;"|"&amp;C361,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J361" s="13">
@@ -13422,7 +13422,7 @@
         <v/>
       </c>
       <c r="I362" s="10">
-        <f>IF(OR(B362="",C362=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B362&amp;"|"&amp;C362,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B362="",C362=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B362&amp;"|"&amp;C362,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J362" s="13">
@@ -13450,7 +13450,7 @@
         <v/>
       </c>
       <c r="I363" s="10">
-        <f>IF(OR(B363="",C363=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B363&amp;"|"&amp;C363,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B363="",C363=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B363&amp;"|"&amp;C363,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J363" s="13">
@@ -13478,7 +13478,7 @@
         <v/>
       </c>
       <c r="I364" s="10">
-        <f>IF(OR(B364="",C364=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B364&amp;"|"&amp;C364,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B364="",C364=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B364&amp;"|"&amp;C364,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J364" s="13">
@@ -13506,7 +13506,7 @@
         <v/>
       </c>
       <c r="I365" s="10">
-        <f>IF(OR(B365="",C365=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B365&amp;"|"&amp;C365,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B365="",C365=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B365&amp;"|"&amp;C365,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J365" s="13">
@@ -13534,7 +13534,7 @@
         <v/>
       </c>
       <c r="I366" s="10">
-        <f>IF(OR(B366="",C366=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B366&amp;"|"&amp;C366,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B366="",C366=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B366&amp;"|"&amp;C366,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J366" s="13">
@@ -13562,7 +13562,7 @@
         <v/>
       </c>
       <c r="I367" s="10">
-        <f>IF(OR(B367="",C367=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B367&amp;"|"&amp;C367,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B367="",C367=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B367&amp;"|"&amp;C367,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J367" s="13">
@@ -13590,7 +13590,7 @@
         <v/>
       </c>
       <c r="I368" s="10">
-        <f>IF(OR(B368="",C368=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B368&amp;"|"&amp;C368,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B368="",C368=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B368&amp;"|"&amp;C368,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J368" s="13">
@@ -13618,7 +13618,7 @@
         <v/>
       </c>
       <c r="I369" s="10">
-        <f>IF(OR(B369="",C369=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B369&amp;"|"&amp;C369,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B369="",C369=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B369&amp;"|"&amp;C369,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J369" s="13">
@@ -13646,7 +13646,7 @@
         <v/>
       </c>
       <c r="I370" s="10">
-        <f>IF(OR(B370="",C370=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B370&amp;"|"&amp;C370,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B370="",C370=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B370&amp;"|"&amp;C370,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J370" s="13">
@@ -13674,7 +13674,7 @@
         <v/>
       </c>
       <c r="I371" s="10">
-        <f>IF(OR(B371="",C371=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B371&amp;"|"&amp;C371,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B371="",C371=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B371&amp;"|"&amp;C371,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J371" s="13">
@@ -13702,7 +13702,7 @@
         <v/>
       </c>
       <c r="I372" s="10">
-        <f>IF(OR(B372="",C372=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B372&amp;"|"&amp;C372,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B372="",C372=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B372&amp;"|"&amp;C372,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J372" s="13">
@@ -13730,7 +13730,7 @@
         <v/>
       </c>
       <c r="I373" s="10">
-        <f>IF(OR(B373="",C373=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B373&amp;"|"&amp;C373,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B373="",C373=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B373&amp;"|"&amp;C373,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J373" s="13">
@@ -13758,7 +13758,7 @@
         <v/>
       </c>
       <c r="I374" s="10">
-        <f>IF(OR(B374="",C374=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B374&amp;"|"&amp;C374,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B374="",C374=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B374&amp;"|"&amp;C374,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J374" s="13">
@@ -13786,7 +13786,7 @@
         <v/>
       </c>
       <c r="I375" s="10">
-        <f>IF(OR(B375="",C375=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B375&amp;"|"&amp;C375,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B375="",C375=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B375&amp;"|"&amp;C375,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J375" s="13">
@@ -13814,7 +13814,7 @@
         <v/>
       </c>
       <c r="I376" s="10">
-        <f>IF(OR(B376="",C376=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B376&amp;"|"&amp;C376,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B376="",C376=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B376&amp;"|"&amp;C376,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J376" s="13">
@@ -13842,7 +13842,7 @@
         <v/>
       </c>
       <c r="I377" s="10">
-        <f>IF(OR(B377="",C377=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B377&amp;"|"&amp;C377,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B377="",C377=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B377&amp;"|"&amp;C377,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J377" s="13">
@@ -13870,7 +13870,7 @@
         <v/>
       </c>
       <c r="I378" s="10">
-        <f>IF(OR(B378="",C378=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B378&amp;"|"&amp;C378,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B378="",C378=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B378&amp;"|"&amp;C378,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J378" s="13">
@@ -13898,7 +13898,7 @@
         <v/>
       </c>
       <c r="I379" s="10">
-        <f>IF(OR(B379="",C379=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B379&amp;"|"&amp;C379,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B379="",C379=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B379&amp;"|"&amp;C379,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J379" s="13">
@@ -13926,7 +13926,7 @@
         <v/>
       </c>
       <c r="I380" s="10">
-        <f>IF(OR(B380="",C380=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B380&amp;"|"&amp;C380,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B380="",C380=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B380&amp;"|"&amp;C380,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J380" s="13">
@@ -13954,7 +13954,7 @@
         <v/>
       </c>
       <c r="I381" s="10">
-        <f>IF(OR(B381="",C381=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B381&amp;"|"&amp;C381,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B381="",C381=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B381&amp;"|"&amp;C381,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J381" s="13">
@@ -13982,7 +13982,7 @@
         <v/>
       </c>
       <c r="I382" s="10">
-        <f>IF(OR(B382="",C382=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B382&amp;"|"&amp;C382,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B382="",C382=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B382&amp;"|"&amp;C382,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J382" s="13">
@@ -14010,7 +14010,7 @@
         <v/>
       </c>
       <c r="I383" s="10">
-        <f>IF(OR(B383="",C383=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B383&amp;"|"&amp;C383,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B383="",C383=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B383&amp;"|"&amp;C383,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J383" s="13">
@@ -14038,7 +14038,7 @@
         <v/>
       </c>
       <c r="I384" s="10">
-        <f>IF(OR(B384="",C384=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B384&amp;"|"&amp;C384,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B384="",C384=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B384&amp;"|"&amp;C384,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J384" s="13">
@@ -14066,7 +14066,7 @@
         <v/>
       </c>
       <c r="I385" s="10">
-        <f>IF(OR(B385="",C385=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B385&amp;"|"&amp;C385,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B385="",C385=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B385&amp;"|"&amp;C385,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J385" s="13">
@@ -14094,7 +14094,7 @@
         <v/>
       </c>
       <c r="I386" s="10">
-        <f>IF(OR(B386="",C386=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B386&amp;"|"&amp;C386,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B386="",C386=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B386&amp;"|"&amp;C386,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J386" s="13">
@@ -14122,7 +14122,7 @@
         <v/>
       </c>
       <c r="I387" s="10">
-        <f>IF(OR(B387="",C387=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B387&amp;"|"&amp;C387,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B387="",C387=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B387&amp;"|"&amp;C387,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J387" s="13">
@@ -14150,7 +14150,7 @@
         <v/>
       </c>
       <c r="I388" s="10">
-        <f>IF(OR(B388="",C388=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B388&amp;"|"&amp;C388,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B388="",C388=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B388&amp;"|"&amp;C388,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J388" s="13">
@@ -14178,7 +14178,7 @@
         <v/>
       </c>
       <c r="I389" s="10">
-        <f>IF(OR(B389="",C389=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B389&amp;"|"&amp;C389,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B389="",C389=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B389&amp;"|"&amp;C389,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J389" s="13">
@@ -14206,7 +14206,7 @@
         <v/>
       </c>
       <c r="I390" s="10">
-        <f>IF(OR(B390="",C390=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B390&amp;"|"&amp;C390,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B390="",C390=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B390&amp;"|"&amp;C390,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J390" s="13">
@@ -14234,7 +14234,7 @@
         <v/>
       </c>
       <c r="I391" s="10">
-        <f>IF(OR(B391="",C391=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B391&amp;"|"&amp;C391,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B391="",C391=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B391&amp;"|"&amp;C391,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J391" s="13">
@@ -14262,7 +14262,7 @@
         <v/>
       </c>
       <c r="I392" s="10">
-        <f>IF(OR(B392="",C392=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B392&amp;"|"&amp;C392,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B392="",C392=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B392&amp;"|"&amp;C392,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J392" s="13">
@@ -14290,7 +14290,7 @@
         <v/>
       </c>
       <c r="I393" s="10">
-        <f>IF(OR(B393="",C393=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B393&amp;"|"&amp;C393,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B393="",C393=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B393&amp;"|"&amp;C393,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J393" s="13">
@@ -14318,7 +14318,7 @@
         <v/>
       </c>
       <c r="I394" s="10">
-        <f>IF(OR(B394="",C394=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B394&amp;"|"&amp;C394,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B394="",C394=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B394&amp;"|"&amp;C394,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J394" s="13">
@@ -14346,7 +14346,7 @@
         <v/>
       </c>
       <c r="I395" s="10">
-        <f>IF(OR(B395="",C395=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B395&amp;"|"&amp;C395,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B395="",C395=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B395&amp;"|"&amp;C395,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J395" s="13">
@@ -14374,7 +14374,7 @@
         <v/>
       </c>
       <c r="I396" s="10">
-        <f>IF(OR(B396="",C396=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B396&amp;"|"&amp;C396,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B396="",C396=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B396&amp;"|"&amp;C396,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J396" s="13">
@@ -14402,7 +14402,7 @@
         <v/>
       </c>
       <c r="I397" s="10">
-        <f>IF(OR(B397="",C397=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B397&amp;"|"&amp;C397,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B397="",C397=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B397&amp;"|"&amp;C397,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J397" s="13">
@@ -14430,7 +14430,7 @@
         <v/>
       </c>
       <c r="I398" s="10">
-        <f>IF(OR(B398="",C398=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B398&amp;"|"&amp;C398,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B398="",C398=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B398&amp;"|"&amp;C398,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J398" s="13">
@@ -14458,7 +14458,7 @@
         <v/>
       </c>
       <c r="I399" s="10">
-        <f>IF(OR(B399="",C399=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B399&amp;"|"&amp;C399,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B399="",C399=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B399&amp;"|"&amp;C399,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J399" s="13">
@@ -14486,7 +14486,7 @@
         <v/>
       </c>
       <c r="I400" s="10">
-        <f>IF(OR(B400="",C400=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B400&amp;"|"&amp;C400,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B400="",C400=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B400&amp;"|"&amp;C400,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J400" s="13">
@@ -14514,7 +14514,7 @@
         <v/>
       </c>
       <c r="I401" s="10">
-        <f>IF(OR(B401="",C401=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B401&amp;"|"&amp;C401,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B401="",C401=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B401&amp;"|"&amp;C401,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J401" s="13">
@@ -14542,7 +14542,7 @@
         <v/>
       </c>
       <c r="I402" s="10">
-        <f>IF(OR(B402="",C402=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B402&amp;"|"&amp;C402,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B402="",C402=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B402&amp;"|"&amp;C402,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J402" s="13">
@@ -14570,7 +14570,7 @@
         <v/>
       </c>
       <c r="I403" s="10">
-        <f>IF(OR(B403="",C403=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B403&amp;"|"&amp;C403,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B403="",C403=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B403&amp;"|"&amp;C403,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J403" s="13">
@@ -14598,7 +14598,7 @@
         <v/>
       </c>
       <c r="I404" s="10">
-        <f>IF(OR(B404="",C404=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B404&amp;"|"&amp;C404,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B404="",C404=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B404&amp;"|"&amp;C404,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J404" s="13">
@@ -14626,7 +14626,7 @@
         <v/>
       </c>
       <c r="I405" s="10">
-        <f>IF(OR(B405="",C405=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B405&amp;"|"&amp;C405,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B405="",C405=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B405&amp;"|"&amp;C405,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J405" s="13">
@@ -14654,7 +14654,7 @@
         <v/>
       </c>
       <c r="I406" s="10">
-        <f>IF(OR(B406="",C406=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B406&amp;"|"&amp;C406,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B406="",C406=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B406&amp;"|"&amp;C406,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J406" s="13">
@@ -14682,7 +14682,7 @@
         <v/>
       </c>
       <c r="I407" s="10">
-        <f>IF(OR(B407="",C407=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B407&amp;"|"&amp;C407,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B407="",C407=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B407&amp;"|"&amp;C407,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J407" s="13">
@@ -14710,7 +14710,7 @@
         <v/>
       </c>
       <c r="I408" s="10">
-        <f>IF(OR(B408="",C408=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B408&amp;"|"&amp;C408,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B408="",C408=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B408&amp;"|"&amp;C408,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J408" s="13">
@@ -14738,7 +14738,7 @@
         <v/>
       </c>
       <c r="I409" s="10">
-        <f>IF(OR(B409="",C409=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B409&amp;"|"&amp;C409,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B409="",C409=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B409&amp;"|"&amp;C409,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J409" s="13">
@@ -14766,7 +14766,7 @@
         <v/>
       </c>
       <c r="I410" s="10">
-        <f>IF(OR(B410="",C410=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B410&amp;"|"&amp;C410,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B410="",C410=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B410&amp;"|"&amp;C410,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J410" s="13">
@@ -14794,7 +14794,7 @@
         <v/>
       </c>
       <c r="I411" s="10">
-        <f>IF(OR(B411="",C411=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B411&amp;"|"&amp;C411,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B411="",C411=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B411&amp;"|"&amp;C411,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J411" s="13">
@@ -14822,7 +14822,7 @@
         <v/>
       </c>
       <c r="I412" s="10">
-        <f>IF(OR(B412="",C412=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B412&amp;"|"&amp;C412,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B412="",C412=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B412&amp;"|"&amp;C412,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J412" s="13">
@@ -14850,7 +14850,7 @@
         <v/>
       </c>
       <c r="I413" s="10">
-        <f>IF(OR(B413="",C413=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B413&amp;"|"&amp;C413,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B413="",C413=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B413&amp;"|"&amp;C413,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J413" s="13">
@@ -14878,7 +14878,7 @@
         <v/>
       </c>
       <c r="I414" s="10">
-        <f>IF(OR(B414="",C414=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B414&amp;"|"&amp;C414,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B414="",C414=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B414&amp;"|"&amp;C414,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J414" s="13">
@@ -14906,7 +14906,7 @@
         <v/>
       </c>
       <c r="I415" s="10">
-        <f>IF(OR(B415="",C415=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B415&amp;"|"&amp;C415,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B415="",C415=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B415&amp;"|"&amp;C415,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J415" s="13">
@@ -14934,7 +14934,7 @@
         <v/>
       </c>
       <c r="I416" s="10">
-        <f>IF(OR(B416="",C416=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B416&amp;"|"&amp;C416,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B416="",C416=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B416&amp;"|"&amp;C416,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J416" s="13">
@@ -14962,7 +14962,7 @@
         <v/>
       </c>
       <c r="I417" s="10">
-        <f>IF(OR(B417="",C417=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B417&amp;"|"&amp;C417,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B417="",C417=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B417&amp;"|"&amp;C417,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J417" s="13">
@@ -14990,7 +14990,7 @@
         <v/>
       </c>
       <c r="I418" s="10">
-        <f>IF(OR(B418="",C418=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B418&amp;"|"&amp;C418,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B418="",C418=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B418&amp;"|"&amp;C418,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J418" s="13">
@@ -15018,7 +15018,7 @@
         <v/>
       </c>
       <c r="I419" s="10">
-        <f>IF(OR(B419="",C419=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B419&amp;"|"&amp;C419,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B419="",C419=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B419&amp;"|"&amp;C419,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J419" s="13">
@@ -15046,7 +15046,7 @@
         <v/>
       </c>
       <c r="I420" s="10">
-        <f>IF(OR(B420="",C420=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B420&amp;"|"&amp;C420,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B420="",C420=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B420&amp;"|"&amp;C420,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J420" s="13">
@@ -15074,7 +15074,7 @@
         <v/>
       </c>
       <c r="I421" s="10">
-        <f>IF(OR(B421="",C421=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B421&amp;"|"&amp;C421,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B421="",C421=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B421&amp;"|"&amp;C421,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J421" s="13">
@@ -15102,7 +15102,7 @@
         <v/>
       </c>
       <c r="I422" s="10">
-        <f>IF(OR(B422="",C422=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B422&amp;"|"&amp;C422,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B422="",C422=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B422&amp;"|"&amp;C422,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J422" s="13">
@@ -15130,7 +15130,7 @@
         <v/>
       </c>
       <c r="I423" s="10">
-        <f>IF(OR(B423="",C423=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B423&amp;"|"&amp;C423,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B423="",C423=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B423&amp;"|"&amp;C423,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J423" s="13">
@@ -15158,7 +15158,7 @@
         <v/>
       </c>
       <c r="I424" s="10">
-        <f>IF(OR(B424="",C424=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B424&amp;"|"&amp;C424,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B424="",C424=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B424&amp;"|"&amp;C424,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J424" s="13">
@@ -15186,7 +15186,7 @@
         <v/>
       </c>
       <c r="I425" s="10">
-        <f>IF(OR(B425="",C425=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B425&amp;"|"&amp;C425,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B425="",C425=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B425&amp;"|"&amp;C425,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J425" s="13">
@@ -15214,7 +15214,7 @@
         <v/>
       </c>
       <c r="I426" s="10">
-        <f>IF(OR(B426="",C426=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B426&amp;"|"&amp;C426,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B426="",C426=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B426&amp;"|"&amp;C426,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J426" s="13">
@@ -15242,7 +15242,7 @@
         <v/>
       </c>
       <c r="I427" s="10">
-        <f>IF(OR(B427="",C427=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B427&amp;"|"&amp;C427,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B427="",C427=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B427&amp;"|"&amp;C427,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J427" s="13">
@@ -15270,7 +15270,7 @@
         <v/>
       </c>
       <c r="I428" s="10">
-        <f>IF(OR(B428="",C428=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B428&amp;"|"&amp;C428,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B428="",C428=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B428&amp;"|"&amp;C428,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J428" s="13">
@@ -15298,7 +15298,7 @@
         <v/>
       </c>
       <c r="I429" s="10">
-        <f>IF(OR(B429="",C429=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B429&amp;"|"&amp;C429,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B429="",C429=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B429&amp;"|"&amp;C429,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J429" s="13">
@@ -15326,7 +15326,7 @@
         <v/>
       </c>
       <c r="I430" s="10">
-        <f>IF(OR(B430="",C430=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B430&amp;"|"&amp;C430,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B430="",C430=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B430&amp;"|"&amp;C430,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J430" s="13">
@@ -15354,7 +15354,7 @@
         <v/>
       </c>
       <c r="I431" s="10">
-        <f>IF(OR(B431="",C431=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B431&amp;"|"&amp;C431,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B431="",C431=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B431&amp;"|"&amp;C431,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J431" s="13">
@@ -15382,7 +15382,7 @@
         <v/>
       </c>
       <c r="I432" s="10">
-        <f>IF(OR(B432="",C432=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B432&amp;"|"&amp;C432,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B432="",C432=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B432&amp;"|"&amp;C432,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J432" s="13">
@@ -15410,7 +15410,7 @@
         <v/>
       </c>
       <c r="I433" s="10">
-        <f>IF(OR(B433="",C433=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B433&amp;"|"&amp;C433,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B433="",C433=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B433&amp;"|"&amp;C433,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J433" s="13">
@@ -15438,7 +15438,7 @@
         <v/>
       </c>
       <c r="I434" s="10">
-        <f>IF(OR(B434="",C434=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B434&amp;"|"&amp;C434,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B434="",C434=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B434&amp;"|"&amp;C434,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J434" s="13">
@@ -15466,7 +15466,7 @@
         <v/>
       </c>
       <c r="I435" s="10">
-        <f>IF(OR(B435="",C435=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B435&amp;"|"&amp;C435,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B435="",C435=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B435&amp;"|"&amp;C435,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J435" s="13">
@@ -15494,7 +15494,7 @@
         <v/>
       </c>
       <c r="I436" s="10">
-        <f>IF(OR(B436="",C436=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B436&amp;"|"&amp;C436,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B436="",C436=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B436&amp;"|"&amp;C436,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J436" s="13">
@@ -15522,7 +15522,7 @@
         <v/>
       </c>
       <c r="I437" s="10">
-        <f>IF(OR(B437="",C437=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B437&amp;"|"&amp;C437,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B437="",C437=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B437&amp;"|"&amp;C437,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J437" s="13">
@@ -15550,7 +15550,7 @@
         <v/>
       </c>
       <c r="I438" s="10">
-        <f>IF(OR(B438="",C438=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B438&amp;"|"&amp;C438,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B438="",C438=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B438&amp;"|"&amp;C438,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J438" s="13">
@@ -15578,7 +15578,7 @@
         <v/>
       </c>
       <c r="I439" s="10">
-        <f>IF(OR(B439="",C439=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B439&amp;"|"&amp;C439,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B439="",C439=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B439&amp;"|"&amp;C439,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J439" s="13">
@@ -15606,7 +15606,7 @@
         <v/>
       </c>
       <c r="I440" s="10">
-        <f>IF(OR(B440="",C440=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B440&amp;"|"&amp;C440,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B440="",C440=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B440&amp;"|"&amp;C440,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J440" s="13">
@@ -15634,7 +15634,7 @@
         <v/>
       </c>
       <c r="I441" s="10">
-        <f>IF(OR(B441="",C441=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B441&amp;"|"&amp;C441,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B441="",C441=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B441&amp;"|"&amp;C441,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J441" s="13">
@@ -15662,7 +15662,7 @@
         <v/>
       </c>
       <c r="I442" s="10">
-        <f>IF(OR(B442="",C442=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B442&amp;"|"&amp;C442,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B442="",C442=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B442&amp;"|"&amp;C442,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J442" s="13">
@@ -15690,7 +15690,7 @@
         <v/>
       </c>
       <c r="I443" s="10">
-        <f>IF(OR(B443="",C443=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B443&amp;"|"&amp;C443,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B443="",C443=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B443&amp;"|"&amp;C443,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J443" s="13">
@@ -15718,7 +15718,7 @@
         <v/>
       </c>
       <c r="I444" s="10">
-        <f>IF(OR(B444="",C444=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B444&amp;"|"&amp;C444,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B444="",C444=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B444&amp;"|"&amp;C444,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J444" s="13">
@@ -15746,7 +15746,7 @@
         <v/>
       </c>
       <c r="I445" s="10">
-        <f>IF(OR(B445="",C445=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B445&amp;"|"&amp;C445,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B445="",C445=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B445&amp;"|"&amp;C445,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J445" s="13">
@@ -15774,7 +15774,7 @@
         <v/>
       </c>
       <c r="I446" s="10">
-        <f>IF(OR(B446="",C446=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B446&amp;"|"&amp;C446,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B446="",C446=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B446&amp;"|"&amp;C446,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J446" s="13">
@@ -15802,7 +15802,7 @@
         <v/>
       </c>
       <c r="I447" s="10">
-        <f>IF(OR(B447="",C447=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B447&amp;"|"&amp;C447,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B447="",C447=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B447&amp;"|"&amp;C447,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J447" s="13">
@@ -15830,7 +15830,7 @@
         <v/>
       </c>
       <c r="I448" s="10">
-        <f>IF(OR(B448="",C448=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B448&amp;"|"&amp;C448,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B448="",C448=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B448&amp;"|"&amp;C448,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J448" s="13">
@@ -15858,7 +15858,7 @@
         <v/>
       </c>
       <c r="I449" s="10">
-        <f>IF(OR(B449="",C449=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B449&amp;"|"&amp;C449,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B449="",C449=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B449&amp;"|"&amp;C449,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J449" s="13">
@@ -15886,7 +15886,7 @@
         <v/>
       </c>
       <c r="I450" s="10">
-        <f>IF(OR(B450="",C450=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B450&amp;"|"&amp;C450,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B450="",C450=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B450&amp;"|"&amp;C450,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J450" s="13">
@@ -15914,7 +15914,7 @@
         <v/>
       </c>
       <c r="I451" s="10">
-        <f>IF(OR(B451="",C451=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B451&amp;"|"&amp;C451,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B451="",C451=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B451&amp;"|"&amp;C451,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J451" s="13">
@@ -15942,7 +15942,7 @@
         <v/>
       </c>
       <c r="I452" s="10">
-        <f>IF(OR(B452="",C452=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B452&amp;"|"&amp;C452,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B452="",C452=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B452&amp;"|"&amp;C452,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J452" s="13">
@@ -15970,7 +15970,7 @@
         <v/>
       </c>
       <c r="I453" s="10">
-        <f>IF(OR(B453="",C453=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B453&amp;"|"&amp;C453,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B453="",C453=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B453&amp;"|"&amp;C453,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J453" s="13">
@@ -15998,7 +15998,7 @@
         <v/>
       </c>
       <c r="I454" s="10">
-        <f>IF(OR(B454="",C454=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B454&amp;"|"&amp;C454,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B454="",C454=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B454&amp;"|"&amp;C454,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J454" s="13">
@@ -16026,7 +16026,7 @@
         <v/>
       </c>
       <c r="I455" s="10">
-        <f>IF(OR(B455="",C455=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B455&amp;"|"&amp;C455,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B455="",C455=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B455&amp;"|"&amp;C455,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J455" s="13">
@@ -16054,7 +16054,7 @@
         <v/>
       </c>
       <c r="I456" s="10">
-        <f>IF(OR(B456="",C456=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B456&amp;"|"&amp;C456,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B456="",C456=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B456&amp;"|"&amp;C456,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J456" s="13">
@@ -16082,7 +16082,7 @@
         <v/>
       </c>
       <c r="I457" s="10">
-        <f>IF(OR(B457="",C457=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B457&amp;"|"&amp;C457,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B457="",C457=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B457&amp;"|"&amp;C457,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J457" s="13">
@@ -16110,7 +16110,7 @@
         <v/>
       </c>
       <c r="I458" s="10">
-        <f>IF(OR(B458="",C458=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B458&amp;"|"&amp;C458,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B458="",C458=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B458&amp;"|"&amp;C458,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J458" s="13">
@@ -16138,7 +16138,7 @@
         <v/>
       </c>
       <c r="I459" s="10">
-        <f>IF(OR(B459="",C459=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B459&amp;"|"&amp;C459,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B459="",C459=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B459&amp;"|"&amp;C459,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J459" s="13">
@@ -16166,7 +16166,7 @@
         <v/>
       </c>
       <c r="I460" s="10">
-        <f>IF(OR(B460="",C460=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B460&amp;"|"&amp;C460,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B460="",C460=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B460&amp;"|"&amp;C460,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J460" s="13">
@@ -16194,7 +16194,7 @@
         <v/>
       </c>
       <c r="I461" s="10">
-        <f>IF(OR(B461="",C461=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B461&amp;"|"&amp;C461,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B461="",C461=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B461&amp;"|"&amp;C461,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J461" s="13">
@@ -16222,7 +16222,7 @@
         <v/>
       </c>
       <c r="I462" s="10">
-        <f>IF(OR(B462="",C462=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B462&amp;"|"&amp;C462,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B462="",C462=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B462&amp;"|"&amp;C462,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J462" s="13">
@@ -16250,7 +16250,7 @@
         <v/>
       </c>
       <c r="I463" s="10">
-        <f>IF(OR(B463="",C463=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B463&amp;"|"&amp;C463,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B463="",C463=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B463&amp;"|"&amp;C463,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J463" s="13">
@@ -16278,7 +16278,7 @@
         <v/>
       </c>
       <c r="I464" s="10">
-        <f>IF(OR(B464="",C464=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B464&amp;"|"&amp;C464,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B464="",C464=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B464&amp;"|"&amp;C464,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J464" s="13">
@@ -16306,7 +16306,7 @@
         <v/>
       </c>
       <c r="I465" s="10">
-        <f>IF(OR(B465="",C465=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B465&amp;"|"&amp;C465,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B465="",C465=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B465&amp;"|"&amp;C465,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J465" s="13">
@@ -16334,7 +16334,7 @@
         <v/>
       </c>
       <c r="I466" s="10">
-        <f>IF(OR(B466="",C466=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B466&amp;"|"&amp;C466,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B466="",C466=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B466&amp;"|"&amp;C466,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J466" s="13">
@@ -16362,7 +16362,7 @@
         <v/>
       </c>
       <c r="I467" s="10">
-        <f>IF(OR(B467="",C467=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B467&amp;"|"&amp;C467,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B467="",C467=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B467&amp;"|"&amp;C467,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J467" s="13">
@@ -16390,7 +16390,7 @@
         <v/>
       </c>
       <c r="I468" s="10">
-        <f>IF(OR(B468="",C468=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B468&amp;"|"&amp;C468,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B468="",C468=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B468&amp;"|"&amp;C468,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J468" s="13">
@@ -16418,7 +16418,7 @@
         <v/>
       </c>
       <c r="I469" s="10">
-        <f>IF(OR(B469="",C469=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B469&amp;"|"&amp;C469,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B469="",C469=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B469&amp;"|"&amp;C469,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J469" s="13">
@@ -16446,7 +16446,7 @@
         <v/>
       </c>
       <c r="I470" s="10">
-        <f>IF(OR(B470="",C470=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B470&amp;"|"&amp;C470,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B470="",C470=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B470&amp;"|"&amp;C470,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J470" s="13">
@@ -16474,7 +16474,7 @@
         <v/>
       </c>
       <c r="I471" s="10">
-        <f>IF(OR(B471="",C471=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B471&amp;"|"&amp;C471,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B471="",C471=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B471&amp;"|"&amp;C471,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J471" s="13">
@@ -16502,7 +16502,7 @@
         <v/>
       </c>
       <c r="I472" s="10">
-        <f>IF(OR(B472="",C472=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B472&amp;"|"&amp;C472,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B472="",C472=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B472&amp;"|"&amp;C472,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J472" s="13">
@@ -16530,7 +16530,7 @@
         <v/>
       </c>
       <c r="I473" s="10">
-        <f>IF(OR(B473="",C473=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B473&amp;"|"&amp;C473,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B473="",C473=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B473&amp;"|"&amp;C473,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J473" s="13">
@@ -16558,7 +16558,7 @@
         <v/>
       </c>
       <c r="I474" s="10">
-        <f>IF(OR(B474="",C474=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B474&amp;"|"&amp;C474,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B474="",C474=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B474&amp;"|"&amp;C474,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J474" s="13">
@@ -16586,7 +16586,7 @@
         <v/>
       </c>
       <c r="I475" s="10">
-        <f>IF(OR(B475="",C475=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B475&amp;"|"&amp;C475,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B475="",C475=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B475&amp;"|"&amp;C475,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J475" s="13">
@@ -16614,7 +16614,7 @@
         <v/>
       </c>
       <c r="I476" s="10">
-        <f>IF(OR(B476="",C476=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B476&amp;"|"&amp;C476,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B476="",C476=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B476&amp;"|"&amp;C476,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J476" s="13">
@@ -16642,7 +16642,7 @@
         <v/>
       </c>
       <c r="I477" s="10">
-        <f>IF(OR(B477="",C477=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B477&amp;"|"&amp;C477,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B477="",C477=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B477&amp;"|"&amp;C477,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J477" s="13">
@@ -16670,7 +16670,7 @@
         <v/>
       </c>
       <c r="I478" s="10">
-        <f>IF(OR(B478="",C478=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B478&amp;"|"&amp;C478,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B478="",C478=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B478&amp;"|"&amp;C478,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J478" s="13">
@@ -16698,7 +16698,7 @@
         <v/>
       </c>
       <c r="I479" s="10">
-        <f>IF(OR(B479="",C479=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B479&amp;"|"&amp;C479,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B479="",C479=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B479&amp;"|"&amp;C479,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J479" s="13">
@@ -16726,7 +16726,7 @@
         <v/>
       </c>
       <c r="I480" s="10">
-        <f>IF(OR(B480="",C480=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B480&amp;"|"&amp;C480,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B480="",C480=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B480&amp;"|"&amp;C480,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J480" s="13">
@@ -16754,7 +16754,7 @@
         <v/>
       </c>
       <c r="I481" s="10">
-        <f>IF(OR(B481="",C481=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B481&amp;"|"&amp;C481,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B481="",C481=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B481&amp;"|"&amp;C481,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J481" s="13">
@@ -16782,7 +16782,7 @@
         <v/>
       </c>
       <c r="I482" s="10">
-        <f>IF(OR(B482="",C482=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B482&amp;"|"&amp;C482,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B482="",C482=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B482&amp;"|"&amp;C482,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J482" s="13">
@@ -16810,7 +16810,7 @@
         <v/>
       </c>
       <c r="I483" s="10">
-        <f>IF(OR(B483="",C483=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B483&amp;"|"&amp;C483,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B483="",C483=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B483&amp;"|"&amp;C483,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J483" s="13">
@@ -16838,7 +16838,7 @@
         <v/>
       </c>
       <c r="I484" s="10">
-        <f>IF(OR(B484="",C484=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B484&amp;"|"&amp;C484,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B484="",C484=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B484&amp;"|"&amp;C484,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J484" s="13">
@@ -16866,7 +16866,7 @@
         <v/>
       </c>
       <c r="I485" s="10">
-        <f>IF(OR(B485="",C485=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B485&amp;"|"&amp;C485,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B485="",C485=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B485&amp;"|"&amp;C485,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J485" s="13">
@@ -16894,7 +16894,7 @@
         <v/>
       </c>
       <c r="I486" s="10">
-        <f>IF(OR(B486="",C486=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B486&amp;"|"&amp;C486,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B486="",C486=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B486&amp;"|"&amp;C486,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J486" s="13">
@@ -16922,7 +16922,7 @@
         <v/>
       </c>
       <c r="I487" s="10">
-        <f>IF(OR(B487="",C487=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B487&amp;"|"&amp;C487,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B487="",C487=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B487&amp;"|"&amp;C487,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J487" s="13">
@@ -16950,7 +16950,7 @@
         <v/>
       </c>
       <c r="I488" s="10">
-        <f>IF(OR(B488="",C488=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B488&amp;"|"&amp;C488,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B488="",C488=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B488&amp;"|"&amp;C488,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J488" s="13">
@@ -16978,7 +16978,7 @@
         <v/>
       </c>
       <c r="I489" s="10">
-        <f>IF(OR(B489="",C489=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B489&amp;"|"&amp;C489,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B489="",C489=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B489&amp;"|"&amp;C489,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J489" s="13">
@@ -17006,7 +17006,7 @@
         <v/>
       </c>
       <c r="I490" s="10">
-        <f>IF(OR(B490="",C490=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B490&amp;"|"&amp;C490,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B490="",C490=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B490&amp;"|"&amp;C490,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J490" s="13">
@@ -17034,7 +17034,7 @@
         <v/>
       </c>
       <c r="I491" s="10">
-        <f>IF(OR(B491="",C491=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B491&amp;"|"&amp;C491,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B491="",C491=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B491&amp;"|"&amp;C491,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J491" s="13">
@@ -17062,7 +17062,7 @@
         <v/>
       </c>
       <c r="I492" s="10">
-        <f>IF(OR(B492="",C492=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B492&amp;"|"&amp;C492,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B492="",C492=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B492&amp;"|"&amp;C492,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J492" s="13">
@@ -17090,7 +17090,7 @@
         <v/>
       </c>
       <c r="I493" s="10">
-        <f>IF(OR(B493="",C493=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B493&amp;"|"&amp;C493,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B493="",C493=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B493&amp;"|"&amp;C493,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J493" s="13">
@@ -17118,7 +17118,7 @@
         <v/>
       </c>
       <c r="I494" s="10">
-        <f>IF(OR(B494="",C494=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B494&amp;"|"&amp;C494,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B494="",C494=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B494&amp;"|"&amp;C494,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J494" s="13">
@@ -17146,7 +17146,7 @@
         <v/>
       </c>
       <c r="I495" s="10">
-        <f>IF(OR(B495="",C495=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B495&amp;"|"&amp;C495,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B495="",C495=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B495&amp;"|"&amp;C495,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J495" s="13">
@@ -17174,7 +17174,7 @@
         <v/>
       </c>
       <c r="I496" s="10">
-        <f>IF(OR(B496="",C496=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B496&amp;"|"&amp;C496,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B496="",C496=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B496&amp;"|"&amp;C496,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J496" s="13">
@@ -17202,7 +17202,7 @@
         <v/>
       </c>
       <c r="I497" s="10">
-        <f>IF(OR(B497="",C497=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B497&amp;"|"&amp;C497,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B497="",C497=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B497&amp;"|"&amp;C497,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J497" s="13">
@@ -17230,7 +17230,7 @@
         <v/>
       </c>
       <c r="I498" s="10">
-        <f>IF(OR(B498="",C498=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B498&amp;"|"&amp;C498,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B498="",C498=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B498&amp;"|"&amp;C498,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J498" s="13">
@@ -17258,7 +17258,7 @@
         <v/>
       </c>
       <c r="I499" s="10">
-        <f>IF(OR(B499="",C499=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B499&amp;"|"&amp;C499,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B499="",C499=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B499&amp;"|"&amp;C499,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J499" s="13">
@@ -17286,7 +17286,7 @@
         <v/>
       </c>
       <c r="I500" s="10">
-        <f>IF(OR(B500="",C500=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$33,MATCH(B500&amp;"|"&amp;C500,LAYOUT!$E$2:$E$33,0)),"zona tidak ada di layout"))</f>
+        <f>IF(OR(B500="",C500=""),"",IFERROR(INDEX(LAYOUT!$D$2:$D$34,MATCH(B500&amp;"|"&amp;C500,LAYOUT!$E$2:$E$34,0)),"zona tidak ada di layout"))</f>
         <v/>
       </c>
       <c r="J500" s="13">
@@ -17386,7 +17386,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Wall 4 Rack</t>
+          <t>Wall 5 Rack</t>
         </is>
       </c>
       <c r="C3" s="9" t="n"/>
@@ -17682,7 +17682,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Jenis fixture" error="Pilih jenis fixture dari daftar." type="list">
-      <formula1>"Wall 6 Rack,Wall 4 Rack,Wall 3 Rack + 2 Gantungan,Gondola 4 Rack,Gondola Full Gantungan,Gondola 1 Rack + 3 Gantungan,Endcap 4 Rack,Pallet 90x90"</formula1>
+      <formula1>"Wall 6 Rack,Wall 5 Rack,Wall 3 Rack + 2 Gantungan,Gondola 4 Rack,Gondola Full Gantungan,Gondola 1 Rack + 3 Gantungan,Endcap 4 Rack,Pallet 90x90"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17695,7 +17695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -17879,7 +17879,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Wall 4 Rack</t>
+          <t>Wall 5 Rack</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -17903,7 +17903,7 @@
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Wall 4 Rack</t>
+          <t>Wall 5 Rack</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -17927,7 +17927,7 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Wall 4 Rack</t>
+          <t>Wall 5 Rack</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -17951,7 +17951,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Wall 4 Rack</t>
+          <t>Wall 5 Rack</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -17975,7 +17975,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Wall 3 Rack + 2 Gantungan</t>
+          <t>Wall 5 Rack</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -17984,11 +17984,11 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Gantungan</t>
+          <t>Rak</t>
         </is>
       </c>
       <c r="E12" s="17">
@@ -18008,7 +18008,7 @@
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
@@ -18032,11 +18032,11 @@
         </is>
       </c>
       <c r="C14" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Rak</t>
+          <t>Gantungan</t>
         </is>
       </c>
       <c r="E14" s="17">
@@ -18056,7 +18056,7 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -18080,7 +18080,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -18095,16 +18095,16 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Gondola 4 Rack</t>
+          <t>Wall 3 Rack + 2 Gantungan</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>120x50x150</t>
+          <t>120x50x270 / 120x50x240</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -18128,7 +18128,7 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -18152,7 +18152,7 @@
         </is>
       </c>
       <c r="C19" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
@@ -18176,7 +18176,7 @@
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
@@ -18191,7 +18191,7 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Gondola Full Gantungan</t>
+          <t>Gondola 4 Rack</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -18200,11 +18200,11 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Gantungan</t>
+          <t>Rak</t>
         </is>
       </c>
       <c r="E21" s="17">
@@ -18224,7 +18224,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -18248,7 +18248,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
@@ -18272,7 +18272,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -18287,7 +18287,7 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Gondola 1 Rack + 3 Gantungan</t>
+          <t>Gondola Full Gantungan</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
@@ -18296,11 +18296,11 @@
         </is>
       </c>
       <c r="C25" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Rak</t>
+          <t>Gantungan</t>
         </is>
       </c>
       <c r="E25" s="17">
@@ -18320,11 +18320,11 @@
         </is>
       </c>
       <c r="C26" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Gantungan</t>
+          <t>Rak</t>
         </is>
       </c>
       <c r="E26" s="17">
@@ -18344,7 +18344,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -18368,7 +18368,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
@@ -18383,20 +18383,20 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Endcap 4 Rack</t>
+          <t>Gondola 1 Rack + 3 Gantungan</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>100x50x150</t>
+          <t>120x50x150</t>
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Rak</t>
+          <t>Gantungan</t>
         </is>
       </c>
       <c r="E29" s="17">
@@ -18416,7 +18416,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
@@ -18440,7 +18440,7 @@
         </is>
       </c>
       <c r="C31" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
@@ -18464,7 +18464,7 @@
         </is>
       </c>
       <c r="C32" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
@@ -18479,16 +18479,16 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>Pallet 90x90</t>
+          <t>Endcap 4 Rack</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>90x90x100</t>
+          <t>100x50x150</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -18500,8 +18500,32 @@
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Pallet 90x90</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>90x90x100</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Rak</t>
+        </is>
+      </c>
+      <c r="E34" s="17">
+        <f>A34&amp;"|"&amp;C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Sheet ini referensi (jangan diubah). Zona dihitung dari atas ke bawah.</t>
         </is>

</xml_diff>

<commit_message>
Template visual catalog for all 12 fixture types on the start screen; SAMBUNG sheet (per-category connected run templates, optional series per row) read by the app with a 'Template sambungan dari Excel' picker; PLT-02 sample pallet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KGdyTJhm5K5VodWjT1gUuo
</commit_message>
<xml_diff>
--- a/template_planogram.xlsx
+++ b/template_planogram.xlsx
@@ -10,13 +10,15 @@
     <sheet name="PETUNJUK" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="DATA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="DIMENSI" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DAFTAR_FIXTURE" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="LAYOUT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SAMBUNG" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DAFTAR_FIXTURE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="LAYOUT" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="FIXTURE_IDS">OFFSET(DAFTAR_FIXTURE!$A$2,0,0,MAX(1,COUNTA(DAFTAR_FIXTURE!$A$2:$A$51)),1)</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DATA'!$A$1:$Z$500</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DIMENSI'!$A$1:$K$500</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'SAMBUNG'!$A$1:$I$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -614,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B69"/>
+  <dimension ref="A1:B119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1004,36 +1006,96 @@
       <c r="B41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>SHEET SAMBUNG (OPSIONAL) — template urutan fixture yang disambung, per kategori</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Fungsi</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Menyimpan urutan fixture yang tampil menempel (Sambung visual) di aplikasi. Muncul sebagai pilihan "Template sambungan dari Excel". Kosong = tidak ada template.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>SAMBUNGAN *</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Nama rangkaian, bebas (mis. WALL-RUN-1). Baris dengan nama sama = satu rangkaian.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>KATEGORI *</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Wall, Gondola, atau Pallet. Satu rangkaian satu kategori. Endcap tidak ikut sambung.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>URUTAN *</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Nomor urut dari kiri ke kanan, mulai 1.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>ID FIXTURE *</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Pilih dari dropdown (sheet DAFTAR_FIXTURE). Jenis fixture harus sesuai KATEGORI.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>SERIES</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>Opsional. Kosong = semua isi fixture tampil. Diisi = hanya produk series itu yang tampil di fixture tersebut.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Kolom otomatis</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Jenis fixture, kategori fixture, dan STATUS (OK atau CEK + penyebab). Jangan diisi atau dihapus.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1115,6 +1177,56 @@
       <c r="A69" s="2" t="n"/>
       <c r="B69" s="2" t="n"/>
     </row>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -35550,6 +35662,4160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I200"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>SAMBUNGAN *</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>KATEGORI *</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>URUTAN *</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>ID FIXTURE *</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>SERIES (opsional)</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>CATATAN (opsional)</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>JENIS FIXTURE (otomatis)</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>KATEGORI FIXTURE (otomatis)</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>STATUS (otomatis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>WALL-RUN-1</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Wall</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>WLL-01</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr"/>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>contoh: hapus lalu isi sambungan Anda</t>
+        </is>
+      </c>
+      <c r="G2" s="12">
+        <f>IF(D2="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D2,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H2" s="12">
+        <f>IF(G2="","",IF(LEFT(G2,4)="Wall","Wall",IF(LEFT(G2,7)="Gondola","Gondola",IF(LEFT(G2,6)="Pallet","Pallet",IF(LEFT(G2,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I2" s="12">
+        <f>IF(A2="","",IF(D2="","CEK ID FIXTURE kosong",IF(G2="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H2="Endcap","CEK Endcap tidak ikut sambung",IF(H2&lt;&gt;B2,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C2="","CEK URUTAN kosong",IF(AND(E2&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E2)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>WALL-RUN-1</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Wall</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>WLL-02</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr"/>
+      <c r="F3" s="10" t="inlineStr"/>
+      <c r="G3" s="12">
+        <f>IF(D3="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D3,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H3" s="12">
+        <f>IF(G3="","",IF(LEFT(G3,4)="Wall","Wall",IF(LEFT(G3,7)="Gondola","Gondola",IF(LEFT(G3,6)="Pallet","Pallet",IF(LEFT(G3,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I3" s="12">
+        <f>IF(A3="","",IF(D3="","CEK ID FIXTURE kosong",IF(G3="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H3="Endcap","CEK Endcap tidak ikut sambung",IF(H3&lt;&gt;B3,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C3="","CEK URUTAN kosong",IF(AND(E3&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E3)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>GONDOLA-RUN-1</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Gondola</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>GND-01</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr"/>
+      <c r="F4" s="10" t="inlineStr"/>
+      <c r="G4" s="12">
+        <f>IF(D4="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D4,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H4" s="12">
+        <f>IF(G4="","",IF(LEFT(G4,4)="Wall","Wall",IF(LEFT(G4,7)="Gondola","Gondola",IF(LEFT(G4,6)="Pallet","Pallet",IF(LEFT(G4,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I4" s="12">
+        <f>IF(A4="","",IF(D4="","CEK ID FIXTURE kosong",IF(G4="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H4="Endcap","CEK Endcap tidak ikut sambung",IF(H4&lt;&gt;B4,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C4="","CEK URUTAN kosong",IF(AND(E4&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E4)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>GONDOLA-RUN-1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Gondola</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>GND-02</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>TANTA NYLON</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>isi SERIES = hanya series itu yang tampil</t>
+        </is>
+      </c>
+      <c r="G5" s="12">
+        <f>IF(D5="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D5,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H5" s="12">
+        <f>IF(G5="","",IF(LEFT(G5,4)="Wall","Wall",IF(LEFT(G5,7)="Gondola","Gondola",IF(LEFT(G5,6)="Pallet","Pallet",IF(LEFT(G5,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I5" s="12">
+        <f>IF(A5="","",IF(D5="","CEK ID FIXTURE kosong",IF(G5="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H5="Endcap","CEK Endcap tidak ikut sambung",IF(H5&lt;&gt;B5,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C5="","CEK URUTAN kosong",IF(AND(E5&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E5)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>PALLET-RUN-1</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Pallet</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>PLT-01</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr"/>
+      <c r="F6" s="10" t="inlineStr"/>
+      <c r="G6" s="12">
+        <f>IF(D6="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D6,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>IF(G6="","",IF(LEFT(G6,4)="Wall","Wall",IF(LEFT(G6,7)="Gondola","Gondola",IF(LEFT(G6,6)="Pallet","Pallet",IF(LEFT(G6,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I6" s="12">
+        <f>IF(A6="","",IF(D6="","CEK ID FIXTURE kosong",IF(G6="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H6="Endcap","CEK Endcap tidak ikut sambung",IF(H6&lt;&gt;B6,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C6="","CEK URUTAN kosong",IF(AND(E6&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E6)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="12">
+        <f>IF(D7="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D7,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H7" s="12">
+        <f>IF(G7="","",IF(LEFT(G7,4)="Wall","Wall",IF(LEFT(G7,7)="Gondola","Gondola",IF(LEFT(G7,6)="Pallet","Pallet",IF(LEFT(G7,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I7" s="12">
+        <f>IF(A7="","",IF(D7="","CEK ID FIXTURE kosong",IF(G7="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H7="Endcap","CEK Endcap tidak ikut sambung",IF(H7&lt;&gt;B7,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C7="","CEK URUTAN kosong",IF(AND(E7&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E7)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="12">
+        <f>IF(D8="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D8,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H8" s="12">
+        <f>IF(G8="","",IF(LEFT(G8,4)="Wall","Wall",IF(LEFT(G8,7)="Gondola","Gondola",IF(LEFT(G8,6)="Pallet","Pallet",IF(LEFT(G8,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I8" s="12">
+        <f>IF(A8="","",IF(D8="","CEK ID FIXTURE kosong",IF(G8="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H8="Endcap","CEK Endcap tidak ikut sambung",IF(H8&lt;&gt;B8,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C8="","CEK URUTAN kosong",IF(AND(E8&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E8)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="12">
+        <f>IF(D9="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D9,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H9" s="12">
+        <f>IF(G9="","",IF(LEFT(G9,4)="Wall","Wall",IF(LEFT(G9,7)="Gondola","Gondola",IF(LEFT(G9,6)="Pallet","Pallet",IF(LEFT(G9,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I9" s="12">
+        <f>IF(A9="","",IF(D9="","CEK ID FIXTURE kosong",IF(G9="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H9="Endcap","CEK Endcap tidak ikut sambung",IF(H9&lt;&gt;B9,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C9="","CEK URUTAN kosong",IF(AND(E9&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E9)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="12">
+        <f>IF(D10="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D10,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H10" s="12">
+        <f>IF(G10="","",IF(LEFT(G10,4)="Wall","Wall",IF(LEFT(G10,7)="Gondola","Gondola",IF(LEFT(G10,6)="Pallet","Pallet",IF(LEFT(G10,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I10" s="12">
+        <f>IF(A10="","",IF(D10="","CEK ID FIXTURE kosong",IF(G10="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H10="Endcap","CEK Endcap tidak ikut sambung",IF(H10&lt;&gt;B10,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C10="","CEK URUTAN kosong",IF(AND(E10&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E10)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="12">
+        <f>IF(D11="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D11,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H11" s="12">
+        <f>IF(G11="","",IF(LEFT(G11,4)="Wall","Wall",IF(LEFT(G11,7)="Gondola","Gondola",IF(LEFT(G11,6)="Pallet","Pallet",IF(LEFT(G11,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I11" s="12">
+        <f>IF(A11="","",IF(D11="","CEK ID FIXTURE kosong",IF(G11="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H11="Endcap","CEK Endcap tidak ikut sambung",IF(H11&lt;&gt;B11,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C11="","CEK URUTAN kosong",IF(AND(E11&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E11)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="12">
+        <f>IF(D12="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D12,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H12" s="12">
+        <f>IF(G12="","",IF(LEFT(G12,4)="Wall","Wall",IF(LEFT(G12,7)="Gondola","Gondola",IF(LEFT(G12,6)="Pallet","Pallet",IF(LEFT(G12,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I12" s="12">
+        <f>IF(A12="","",IF(D12="","CEK ID FIXTURE kosong",IF(G12="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H12="Endcap","CEK Endcap tidak ikut sambung",IF(H12&lt;&gt;B12,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C12="","CEK URUTAN kosong",IF(AND(E12&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E12)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="12">
+        <f>IF(D13="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D13,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H13" s="12">
+        <f>IF(G13="","",IF(LEFT(G13,4)="Wall","Wall",IF(LEFT(G13,7)="Gondola","Gondola",IF(LEFT(G13,6)="Pallet","Pallet",IF(LEFT(G13,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I13" s="12">
+        <f>IF(A13="","",IF(D13="","CEK ID FIXTURE kosong",IF(G13="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H13="Endcap","CEK Endcap tidak ikut sambung",IF(H13&lt;&gt;B13,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C13="","CEK URUTAN kosong",IF(AND(E13&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E13)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="12">
+        <f>IF(D14="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D14,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H14" s="12">
+        <f>IF(G14="","",IF(LEFT(G14,4)="Wall","Wall",IF(LEFT(G14,7)="Gondola","Gondola",IF(LEFT(G14,6)="Pallet","Pallet",IF(LEFT(G14,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I14" s="12">
+        <f>IF(A14="","",IF(D14="","CEK ID FIXTURE kosong",IF(G14="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H14="Endcap","CEK Endcap tidak ikut sambung",IF(H14&lt;&gt;B14,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C14="","CEK URUTAN kosong",IF(AND(E14&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E14)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="12">
+        <f>IF(D15="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D15,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H15" s="12">
+        <f>IF(G15="","",IF(LEFT(G15,4)="Wall","Wall",IF(LEFT(G15,7)="Gondola","Gondola",IF(LEFT(G15,6)="Pallet","Pallet",IF(LEFT(G15,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I15" s="12">
+        <f>IF(A15="","",IF(D15="","CEK ID FIXTURE kosong",IF(G15="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H15="Endcap","CEK Endcap tidak ikut sambung",IF(H15&lt;&gt;B15,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C15="","CEK URUTAN kosong",IF(AND(E15&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E15)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="12">
+        <f>IF(D16="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D16,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H16" s="12">
+        <f>IF(G16="","",IF(LEFT(G16,4)="Wall","Wall",IF(LEFT(G16,7)="Gondola","Gondola",IF(LEFT(G16,6)="Pallet","Pallet",IF(LEFT(G16,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I16" s="12">
+        <f>IF(A16="","",IF(D16="","CEK ID FIXTURE kosong",IF(G16="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H16="Endcap","CEK Endcap tidak ikut sambung",IF(H16&lt;&gt;B16,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C16="","CEK URUTAN kosong",IF(AND(E16&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E16)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="12">
+        <f>IF(D17="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D17,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H17" s="12">
+        <f>IF(G17="","",IF(LEFT(G17,4)="Wall","Wall",IF(LEFT(G17,7)="Gondola","Gondola",IF(LEFT(G17,6)="Pallet","Pallet",IF(LEFT(G17,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I17" s="12">
+        <f>IF(A17="","",IF(D17="","CEK ID FIXTURE kosong",IF(G17="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H17="Endcap","CEK Endcap tidak ikut sambung",IF(H17&lt;&gt;B17,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C17="","CEK URUTAN kosong",IF(AND(E17&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E17)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="12">
+        <f>IF(D18="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D18,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H18" s="12">
+        <f>IF(G18="","",IF(LEFT(G18,4)="Wall","Wall",IF(LEFT(G18,7)="Gondola","Gondola",IF(LEFT(G18,6)="Pallet","Pallet",IF(LEFT(G18,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I18" s="12">
+        <f>IF(A18="","",IF(D18="","CEK ID FIXTURE kosong",IF(G18="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H18="Endcap","CEK Endcap tidak ikut sambung",IF(H18&lt;&gt;B18,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C18="","CEK URUTAN kosong",IF(AND(E18&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E18)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="12">
+        <f>IF(D19="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D19,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H19" s="12">
+        <f>IF(G19="","",IF(LEFT(G19,4)="Wall","Wall",IF(LEFT(G19,7)="Gondola","Gondola",IF(LEFT(G19,6)="Pallet","Pallet",IF(LEFT(G19,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I19" s="12">
+        <f>IF(A19="","",IF(D19="","CEK ID FIXTURE kosong",IF(G19="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H19="Endcap","CEK Endcap tidak ikut sambung",IF(H19&lt;&gt;B19,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C19="","CEK URUTAN kosong",IF(AND(E19&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E19)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="12">
+        <f>IF(D20="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D20,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H20" s="12">
+        <f>IF(G20="","",IF(LEFT(G20,4)="Wall","Wall",IF(LEFT(G20,7)="Gondola","Gondola",IF(LEFT(G20,6)="Pallet","Pallet",IF(LEFT(G20,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I20" s="12">
+        <f>IF(A20="","",IF(D20="","CEK ID FIXTURE kosong",IF(G20="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H20="Endcap","CEK Endcap tidak ikut sambung",IF(H20&lt;&gt;B20,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C20="","CEK URUTAN kosong",IF(AND(E20&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E20)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="12">
+        <f>IF(D21="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D21,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H21" s="12">
+        <f>IF(G21="","",IF(LEFT(G21,4)="Wall","Wall",IF(LEFT(G21,7)="Gondola","Gondola",IF(LEFT(G21,6)="Pallet","Pallet",IF(LEFT(G21,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I21" s="12">
+        <f>IF(A21="","",IF(D21="","CEK ID FIXTURE kosong",IF(G21="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H21="Endcap","CEK Endcap tidak ikut sambung",IF(H21&lt;&gt;B21,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C21="","CEK URUTAN kosong",IF(AND(E21&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E21)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="12">
+        <f>IF(D22="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D22,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H22" s="12">
+        <f>IF(G22="","",IF(LEFT(G22,4)="Wall","Wall",IF(LEFT(G22,7)="Gondola","Gondola",IF(LEFT(G22,6)="Pallet","Pallet",IF(LEFT(G22,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I22" s="12">
+        <f>IF(A22="","",IF(D22="","CEK ID FIXTURE kosong",IF(G22="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H22="Endcap","CEK Endcap tidak ikut sambung",IF(H22&lt;&gt;B22,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C22="","CEK URUTAN kosong",IF(AND(E22&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E22)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="12">
+        <f>IF(D23="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D23,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H23" s="12">
+        <f>IF(G23="","",IF(LEFT(G23,4)="Wall","Wall",IF(LEFT(G23,7)="Gondola","Gondola",IF(LEFT(G23,6)="Pallet","Pallet",IF(LEFT(G23,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I23" s="12">
+        <f>IF(A23="","",IF(D23="","CEK ID FIXTURE kosong",IF(G23="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H23="Endcap","CEK Endcap tidak ikut sambung",IF(H23&lt;&gt;B23,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C23="","CEK URUTAN kosong",IF(AND(E23&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E23)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="12">
+        <f>IF(D24="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D24,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H24" s="12">
+        <f>IF(G24="","",IF(LEFT(G24,4)="Wall","Wall",IF(LEFT(G24,7)="Gondola","Gondola",IF(LEFT(G24,6)="Pallet","Pallet",IF(LEFT(G24,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I24" s="12">
+        <f>IF(A24="","",IF(D24="","CEK ID FIXTURE kosong",IF(G24="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H24="Endcap","CEK Endcap tidak ikut sambung",IF(H24&lt;&gt;B24,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C24="","CEK URUTAN kosong",IF(AND(E24&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E24)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="12">
+        <f>IF(D25="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D25,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H25" s="12">
+        <f>IF(G25="","",IF(LEFT(G25,4)="Wall","Wall",IF(LEFT(G25,7)="Gondola","Gondola",IF(LEFT(G25,6)="Pallet","Pallet",IF(LEFT(G25,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I25" s="12">
+        <f>IF(A25="","",IF(D25="","CEK ID FIXTURE kosong",IF(G25="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H25="Endcap","CEK Endcap tidak ikut sambung",IF(H25&lt;&gt;B25,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C25="","CEK URUTAN kosong",IF(AND(E25&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E25)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="12">
+        <f>IF(D26="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D26,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H26" s="12">
+        <f>IF(G26="","",IF(LEFT(G26,4)="Wall","Wall",IF(LEFT(G26,7)="Gondola","Gondola",IF(LEFT(G26,6)="Pallet","Pallet",IF(LEFT(G26,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I26" s="12">
+        <f>IF(A26="","",IF(D26="","CEK ID FIXTURE kosong",IF(G26="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H26="Endcap","CEK Endcap tidak ikut sambung",IF(H26&lt;&gt;B26,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C26="","CEK URUTAN kosong",IF(AND(E26&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E26)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="12">
+        <f>IF(D27="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D27,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H27" s="12">
+        <f>IF(G27="","",IF(LEFT(G27,4)="Wall","Wall",IF(LEFT(G27,7)="Gondola","Gondola",IF(LEFT(G27,6)="Pallet","Pallet",IF(LEFT(G27,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I27" s="12">
+        <f>IF(A27="","",IF(D27="","CEK ID FIXTURE kosong",IF(G27="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H27="Endcap","CEK Endcap tidak ikut sambung",IF(H27&lt;&gt;B27,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C27="","CEK URUTAN kosong",IF(AND(E27&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E27)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="12">
+        <f>IF(D28="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D28,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H28" s="12">
+        <f>IF(G28="","",IF(LEFT(G28,4)="Wall","Wall",IF(LEFT(G28,7)="Gondola","Gondola",IF(LEFT(G28,6)="Pallet","Pallet",IF(LEFT(G28,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I28" s="12">
+        <f>IF(A28="","",IF(D28="","CEK ID FIXTURE kosong",IF(G28="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H28="Endcap","CEK Endcap tidak ikut sambung",IF(H28&lt;&gt;B28,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C28="","CEK URUTAN kosong",IF(AND(E28&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E28)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="12">
+        <f>IF(D29="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D29,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H29" s="12">
+        <f>IF(G29="","",IF(LEFT(G29,4)="Wall","Wall",IF(LEFT(G29,7)="Gondola","Gondola",IF(LEFT(G29,6)="Pallet","Pallet",IF(LEFT(G29,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I29" s="12">
+        <f>IF(A29="","",IF(D29="","CEK ID FIXTURE kosong",IF(G29="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H29="Endcap","CEK Endcap tidak ikut sambung",IF(H29&lt;&gt;B29,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C29="","CEK URUTAN kosong",IF(AND(E29&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E29)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="12">
+        <f>IF(D30="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D30,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H30" s="12">
+        <f>IF(G30="","",IF(LEFT(G30,4)="Wall","Wall",IF(LEFT(G30,7)="Gondola","Gondola",IF(LEFT(G30,6)="Pallet","Pallet",IF(LEFT(G30,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I30" s="12">
+        <f>IF(A30="","",IF(D30="","CEK ID FIXTURE kosong",IF(G30="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H30="Endcap","CEK Endcap tidak ikut sambung",IF(H30&lt;&gt;B30,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C30="","CEK URUTAN kosong",IF(AND(E30&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E30)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="12">
+        <f>IF(D31="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D31,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H31" s="12">
+        <f>IF(G31="","",IF(LEFT(G31,4)="Wall","Wall",IF(LEFT(G31,7)="Gondola","Gondola",IF(LEFT(G31,6)="Pallet","Pallet",IF(LEFT(G31,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I31" s="12">
+        <f>IF(A31="","",IF(D31="","CEK ID FIXTURE kosong",IF(G31="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H31="Endcap","CEK Endcap tidak ikut sambung",IF(H31&lt;&gt;B31,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C31="","CEK URUTAN kosong",IF(AND(E31&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E31)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="12">
+        <f>IF(D32="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D32,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H32" s="12">
+        <f>IF(G32="","",IF(LEFT(G32,4)="Wall","Wall",IF(LEFT(G32,7)="Gondola","Gondola",IF(LEFT(G32,6)="Pallet","Pallet",IF(LEFT(G32,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I32" s="12">
+        <f>IF(A32="","",IF(D32="","CEK ID FIXTURE kosong",IF(G32="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H32="Endcap","CEK Endcap tidak ikut sambung",IF(H32&lt;&gt;B32,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C32="","CEK URUTAN kosong",IF(AND(E32&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E32)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n"/>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="12">
+        <f>IF(D33="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D33,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H33" s="12">
+        <f>IF(G33="","",IF(LEFT(G33,4)="Wall","Wall",IF(LEFT(G33,7)="Gondola","Gondola",IF(LEFT(G33,6)="Pallet","Pallet",IF(LEFT(G33,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I33" s="12">
+        <f>IF(A33="","",IF(D33="","CEK ID FIXTURE kosong",IF(G33="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H33="Endcap","CEK Endcap tidak ikut sambung",IF(H33&lt;&gt;B33,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C33="","CEK URUTAN kosong",IF(AND(E33&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E33)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="11" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="12">
+        <f>IF(D34="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D34,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H34" s="12">
+        <f>IF(G34="","",IF(LEFT(G34,4)="Wall","Wall",IF(LEFT(G34,7)="Gondola","Gondola",IF(LEFT(G34,6)="Pallet","Pallet",IF(LEFT(G34,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I34" s="12">
+        <f>IF(A34="","",IF(D34="","CEK ID FIXTURE kosong",IF(G34="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H34="Endcap","CEK Endcap tidak ikut sambung",IF(H34&lt;&gt;B34,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C34="","CEK URUTAN kosong",IF(AND(E34&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E34)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n"/>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="12">
+        <f>IF(D35="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D35,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H35" s="12">
+        <f>IF(G35="","",IF(LEFT(G35,4)="Wall","Wall",IF(LEFT(G35,7)="Gondola","Gondola",IF(LEFT(G35,6)="Pallet","Pallet",IF(LEFT(G35,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I35" s="12">
+        <f>IF(A35="","",IF(D35="","CEK ID FIXTURE kosong",IF(G35="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H35="Endcap","CEK Endcap tidak ikut sambung",IF(H35&lt;&gt;B35,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C35="","CEK URUTAN kosong",IF(AND(E35&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E35)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="12">
+        <f>IF(D36="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D36,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H36" s="12">
+        <f>IF(G36="","",IF(LEFT(G36,4)="Wall","Wall",IF(LEFT(G36,7)="Gondola","Gondola",IF(LEFT(G36,6)="Pallet","Pallet",IF(LEFT(G36,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I36" s="12">
+        <f>IF(A36="","",IF(D36="","CEK ID FIXTURE kosong",IF(G36="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H36="Endcap","CEK Endcap tidak ikut sambung",IF(H36&lt;&gt;B36,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C36="","CEK URUTAN kosong",IF(AND(E36&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E36)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="12">
+        <f>IF(D37="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D37,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H37" s="12">
+        <f>IF(G37="","",IF(LEFT(G37,4)="Wall","Wall",IF(LEFT(G37,7)="Gondola","Gondola",IF(LEFT(G37,6)="Pallet","Pallet",IF(LEFT(G37,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I37" s="12">
+        <f>IF(A37="","",IF(D37="","CEK ID FIXTURE kosong",IF(G37="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H37="Endcap","CEK Endcap tidak ikut sambung",IF(H37&lt;&gt;B37,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C37="","CEK URUTAN kosong",IF(AND(E37&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E37)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="n"/>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="12">
+        <f>IF(D38="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D38,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H38" s="12">
+        <f>IF(G38="","",IF(LEFT(G38,4)="Wall","Wall",IF(LEFT(G38,7)="Gondola","Gondola",IF(LEFT(G38,6)="Pallet","Pallet",IF(LEFT(G38,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I38" s="12">
+        <f>IF(A38="","",IF(D38="","CEK ID FIXTURE kosong",IF(G38="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H38="Endcap","CEK Endcap tidak ikut sambung",IF(H38&lt;&gt;B38,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C38="","CEK URUTAN kosong",IF(AND(E38&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E38)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="10" t="n"/>
+      <c r="G39" s="12">
+        <f>IF(D39="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D39,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H39" s="12">
+        <f>IF(G39="","",IF(LEFT(G39,4)="Wall","Wall",IF(LEFT(G39,7)="Gondola","Gondola",IF(LEFT(G39,6)="Pallet","Pallet",IF(LEFT(G39,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I39" s="12">
+        <f>IF(A39="","",IF(D39="","CEK ID FIXTURE kosong",IF(G39="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H39="Endcap","CEK Endcap tidak ikut sambung",IF(H39&lt;&gt;B39,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C39="","CEK URUTAN kosong",IF(AND(E39&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E39)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="n"/>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="12">
+        <f>IF(D40="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D40,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H40" s="12">
+        <f>IF(G40="","",IF(LEFT(G40,4)="Wall","Wall",IF(LEFT(G40,7)="Gondola","Gondola",IF(LEFT(G40,6)="Pallet","Pallet",IF(LEFT(G40,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I40" s="12">
+        <f>IF(A40="","",IF(D40="","CEK ID FIXTURE kosong",IF(G40="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H40="Endcap","CEK Endcap tidak ikut sambung",IF(H40&lt;&gt;B40,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C40="","CEK URUTAN kosong",IF(AND(E40&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E40)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="n"/>
+      <c r="B41" s="10" t="n"/>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="12">
+        <f>IF(D41="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D41,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H41" s="12">
+        <f>IF(G41="","",IF(LEFT(G41,4)="Wall","Wall",IF(LEFT(G41,7)="Gondola","Gondola",IF(LEFT(G41,6)="Pallet","Pallet",IF(LEFT(G41,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I41" s="12">
+        <f>IF(A41="","",IF(D41="","CEK ID FIXTURE kosong",IF(G41="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H41="Endcap","CEK Endcap tidak ikut sambung",IF(H41&lt;&gt;B41,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C41="","CEK URUTAN kosong",IF(AND(E41&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E41)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="n"/>
+      <c r="B42" s="10" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="12">
+        <f>IF(D42="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D42,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H42" s="12">
+        <f>IF(G42="","",IF(LEFT(G42,4)="Wall","Wall",IF(LEFT(G42,7)="Gondola","Gondola",IF(LEFT(G42,6)="Pallet","Pallet",IF(LEFT(G42,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I42" s="12">
+        <f>IF(A42="","",IF(D42="","CEK ID FIXTURE kosong",IF(G42="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H42="Endcap","CEK Endcap tidak ikut sambung",IF(H42&lt;&gt;B42,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C42="","CEK URUTAN kosong",IF(AND(E42&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E42)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="n"/>
+      <c r="B43" s="10" t="n"/>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="12">
+        <f>IF(D43="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D43,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H43" s="12">
+        <f>IF(G43="","",IF(LEFT(G43,4)="Wall","Wall",IF(LEFT(G43,7)="Gondola","Gondola",IF(LEFT(G43,6)="Pallet","Pallet",IF(LEFT(G43,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I43" s="12">
+        <f>IF(A43="","",IF(D43="","CEK ID FIXTURE kosong",IF(G43="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H43="Endcap","CEK Endcap tidak ikut sambung",IF(H43&lt;&gt;B43,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C43="","CEK URUTAN kosong",IF(AND(E43&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E43)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="11" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="12">
+        <f>IF(D44="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D44,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H44" s="12">
+        <f>IF(G44="","",IF(LEFT(G44,4)="Wall","Wall",IF(LEFT(G44,7)="Gondola","Gondola",IF(LEFT(G44,6)="Pallet","Pallet",IF(LEFT(G44,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I44" s="12">
+        <f>IF(A44="","",IF(D44="","CEK ID FIXTURE kosong",IF(G44="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H44="Endcap","CEK Endcap tidak ikut sambung",IF(H44&lt;&gt;B44,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C44="","CEK URUTAN kosong",IF(AND(E44&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E44)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="n"/>
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="12">
+        <f>IF(D45="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D45,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H45" s="12">
+        <f>IF(G45="","",IF(LEFT(G45,4)="Wall","Wall",IF(LEFT(G45,7)="Gondola","Gondola",IF(LEFT(G45,6)="Pallet","Pallet",IF(LEFT(G45,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I45" s="12">
+        <f>IF(A45="","",IF(D45="","CEK ID FIXTURE kosong",IF(G45="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H45="Endcap","CEK Endcap tidak ikut sambung",IF(H45&lt;&gt;B45,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C45="","CEK URUTAN kosong",IF(AND(E45&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E45)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="11" t="n"/>
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="12">
+        <f>IF(D46="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D46,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H46" s="12">
+        <f>IF(G46="","",IF(LEFT(G46,4)="Wall","Wall",IF(LEFT(G46,7)="Gondola","Gondola",IF(LEFT(G46,6)="Pallet","Pallet",IF(LEFT(G46,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I46" s="12">
+        <f>IF(A46="","",IF(D46="","CEK ID FIXTURE kosong",IF(G46="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H46="Endcap","CEK Endcap tidak ikut sambung",IF(H46&lt;&gt;B46,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C46="","CEK URUTAN kosong",IF(AND(E46&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E46)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="n"/>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="10" t="n"/>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="12">
+        <f>IF(D47="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D47,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H47" s="12">
+        <f>IF(G47="","",IF(LEFT(G47,4)="Wall","Wall",IF(LEFT(G47,7)="Gondola","Gondola",IF(LEFT(G47,6)="Pallet","Pallet",IF(LEFT(G47,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I47" s="12">
+        <f>IF(A47="","",IF(D47="","CEK ID FIXTURE kosong",IF(G47="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H47="Endcap","CEK Endcap tidak ikut sambung",IF(H47&lt;&gt;B47,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C47="","CEK URUTAN kosong",IF(AND(E47&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E47)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="n"/>
+      <c r="B48" s="10" t="n"/>
+      <c r="C48" s="10" t="n"/>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="10" t="n"/>
+      <c r="F48" s="10" t="n"/>
+      <c r="G48" s="12">
+        <f>IF(D48="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D48,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H48" s="12">
+        <f>IF(G48="","",IF(LEFT(G48,4)="Wall","Wall",IF(LEFT(G48,7)="Gondola","Gondola",IF(LEFT(G48,6)="Pallet","Pallet",IF(LEFT(G48,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I48" s="12">
+        <f>IF(A48="","",IF(D48="","CEK ID FIXTURE kosong",IF(G48="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H48="Endcap","CEK Endcap tidak ikut sambung",IF(H48&lt;&gt;B48,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C48="","CEK URUTAN kosong",IF(AND(E48&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E48)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="n"/>
+      <c r="B49" s="10" t="n"/>
+      <c r="C49" s="10" t="n"/>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="10" t="n"/>
+      <c r="F49" s="10" t="n"/>
+      <c r="G49" s="12">
+        <f>IF(D49="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D49,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H49" s="12">
+        <f>IF(G49="","",IF(LEFT(G49,4)="Wall","Wall",IF(LEFT(G49,7)="Gondola","Gondola",IF(LEFT(G49,6)="Pallet","Pallet",IF(LEFT(G49,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I49" s="12">
+        <f>IF(A49="","",IF(D49="","CEK ID FIXTURE kosong",IF(G49="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H49="Endcap","CEK Endcap tidak ikut sambung",IF(H49&lt;&gt;B49,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C49="","CEK URUTAN kosong",IF(AND(E49&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E49)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="n"/>
+      <c r="B50" s="10" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="12">
+        <f>IF(D50="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D50,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H50" s="12">
+        <f>IF(G50="","",IF(LEFT(G50,4)="Wall","Wall",IF(LEFT(G50,7)="Gondola","Gondola",IF(LEFT(G50,6)="Pallet","Pallet",IF(LEFT(G50,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I50" s="12">
+        <f>IF(A50="","",IF(D50="","CEK ID FIXTURE kosong",IF(G50="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H50="Endcap","CEK Endcap tidak ikut sambung",IF(H50&lt;&gt;B50,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C50="","CEK URUTAN kosong",IF(AND(E50&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E50)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="n"/>
+      <c r="B51" s="10" t="n"/>
+      <c r="C51" s="10" t="n"/>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="10" t="n"/>
+      <c r="F51" s="10" t="n"/>
+      <c r="G51" s="12">
+        <f>IF(D51="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D51,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H51" s="12">
+        <f>IF(G51="","",IF(LEFT(G51,4)="Wall","Wall",IF(LEFT(G51,7)="Gondola","Gondola",IF(LEFT(G51,6)="Pallet","Pallet",IF(LEFT(G51,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I51" s="12">
+        <f>IF(A51="","",IF(D51="","CEK ID FIXTURE kosong",IF(G51="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H51="Endcap","CEK Endcap tidak ikut sambung",IF(H51&lt;&gt;B51,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C51="","CEK URUTAN kosong",IF(AND(E51&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E51)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="n"/>
+      <c r="B52" s="10" t="n"/>
+      <c r="C52" s="10" t="n"/>
+      <c r="D52" s="11" t="n"/>
+      <c r="E52" s="10" t="n"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="12">
+        <f>IF(D52="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D52,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H52" s="12">
+        <f>IF(G52="","",IF(LEFT(G52,4)="Wall","Wall",IF(LEFT(G52,7)="Gondola","Gondola",IF(LEFT(G52,6)="Pallet","Pallet",IF(LEFT(G52,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I52" s="12">
+        <f>IF(A52="","",IF(D52="","CEK ID FIXTURE kosong",IF(G52="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H52="Endcap","CEK Endcap tidak ikut sambung",IF(H52&lt;&gt;B52,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C52="","CEK URUTAN kosong",IF(AND(E52&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E52)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="n"/>
+      <c r="B53" s="10" t="n"/>
+      <c r="C53" s="10" t="n"/>
+      <c r="D53" s="11" t="n"/>
+      <c r="E53" s="10" t="n"/>
+      <c r="F53" s="10" t="n"/>
+      <c r="G53" s="12">
+        <f>IF(D53="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D53,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H53" s="12">
+        <f>IF(G53="","",IF(LEFT(G53,4)="Wall","Wall",IF(LEFT(G53,7)="Gondola","Gondola",IF(LEFT(G53,6)="Pallet","Pallet",IF(LEFT(G53,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I53" s="12">
+        <f>IF(A53="","",IF(D53="","CEK ID FIXTURE kosong",IF(G53="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H53="Endcap","CEK Endcap tidak ikut sambung",IF(H53&lt;&gt;B53,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C53="","CEK URUTAN kosong",IF(AND(E53&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E53)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n"/>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="10" t="n"/>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="10" t="n"/>
+      <c r="F54" s="10" t="n"/>
+      <c r="G54" s="12">
+        <f>IF(D54="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D54,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H54" s="12">
+        <f>IF(G54="","",IF(LEFT(G54,4)="Wall","Wall",IF(LEFT(G54,7)="Gondola","Gondola",IF(LEFT(G54,6)="Pallet","Pallet",IF(LEFT(G54,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I54" s="12">
+        <f>IF(A54="","",IF(D54="","CEK ID FIXTURE kosong",IF(G54="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H54="Endcap","CEK Endcap tidak ikut sambung",IF(H54&lt;&gt;B54,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C54="","CEK URUTAN kosong",IF(AND(E54&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E54)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="n"/>
+      <c r="B55" s="10" t="n"/>
+      <c r="C55" s="10" t="n"/>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="10" t="n"/>
+      <c r="F55" s="10" t="n"/>
+      <c r="G55" s="12">
+        <f>IF(D55="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D55,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H55" s="12">
+        <f>IF(G55="","",IF(LEFT(G55,4)="Wall","Wall",IF(LEFT(G55,7)="Gondola","Gondola",IF(LEFT(G55,6)="Pallet","Pallet",IF(LEFT(G55,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I55" s="12">
+        <f>IF(A55="","",IF(D55="","CEK ID FIXTURE kosong",IF(G55="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H55="Endcap","CEK Endcap tidak ikut sambung",IF(H55&lt;&gt;B55,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C55="","CEK URUTAN kosong",IF(AND(E55&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E55)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n"/>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="11" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="12">
+        <f>IF(D56="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D56,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H56" s="12">
+        <f>IF(G56="","",IF(LEFT(G56,4)="Wall","Wall",IF(LEFT(G56,7)="Gondola","Gondola",IF(LEFT(G56,6)="Pallet","Pallet",IF(LEFT(G56,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I56" s="12">
+        <f>IF(A56="","",IF(D56="","CEK ID FIXTURE kosong",IF(G56="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H56="Endcap","CEK Endcap tidak ikut sambung",IF(H56&lt;&gt;B56,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C56="","CEK URUTAN kosong",IF(AND(E56&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E56)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="n"/>
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="10" t="n"/>
+      <c r="D57" s="11" t="n"/>
+      <c r="E57" s="10" t="n"/>
+      <c r="F57" s="10" t="n"/>
+      <c r="G57" s="12">
+        <f>IF(D57="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D57,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H57" s="12">
+        <f>IF(G57="","",IF(LEFT(G57,4)="Wall","Wall",IF(LEFT(G57,7)="Gondola","Gondola",IF(LEFT(G57,6)="Pallet","Pallet",IF(LEFT(G57,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I57" s="12">
+        <f>IF(A57="","",IF(D57="","CEK ID FIXTURE kosong",IF(G57="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H57="Endcap","CEK Endcap tidak ikut sambung",IF(H57&lt;&gt;B57,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C57="","CEK URUTAN kosong",IF(AND(E57&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E57)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n"/>
+      <c r="B58" s="10" t="n"/>
+      <c r="C58" s="10" t="n"/>
+      <c r="D58" s="11" t="n"/>
+      <c r="E58" s="10" t="n"/>
+      <c r="F58" s="10" t="n"/>
+      <c r="G58" s="12">
+        <f>IF(D58="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D58,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H58" s="12">
+        <f>IF(G58="","",IF(LEFT(G58,4)="Wall","Wall",IF(LEFT(G58,7)="Gondola","Gondola",IF(LEFT(G58,6)="Pallet","Pallet",IF(LEFT(G58,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I58" s="12">
+        <f>IF(A58="","",IF(D58="","CEK ID FIXTURE kosong",IF(G58="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H58="Endcap","CEK Endcap tidak ikut sambung",IF(H58&lt;&gt;B58,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C58="","CEK URUTAN kosong",IF(AND(E58&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E58)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="n"/>
+      <c r="B59" s="10" t="n"/>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="11" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="10" t="n"/>
+      <c r="G59" s="12">
+        <f>IF(D59="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D59,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H59" s="12">
+        <f>IF(G59="","",IF(LEFT(G59,4)="Wall","Wall",IF(LEFT(G59,7)="Gondola","Gondola",IF(LEFT(G59,6)="Pallet","Pallet",IF(LEFT(G59,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I59" s="12">
+        <f>IF(A59="","",IF(D59="","CEK ID FIXTURE kosong",IF(G59="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H59="Endcap","CEK Endcap tidak ikut sambung",IF(H59&lt;&gt;B59,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C59="","CEK URUTAN kosong",IF(AND(E59&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E59)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="n"/>
+      <c r="B60" s="10" t="n"/>
+      <c r="C60" s="10" t="n"/>
+      <c r="D60" s="11" t="n"/>
+      <c r="E60" s="10" t="n"/>
+      <c r="F60" s="10" t="n"/>
+      <c r="G60" s="12">
+        <f>IF(D60="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D60,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H60" s="12">
+        <f>IF(G60="","",IF(LEFT(G60,4)="Wall","Wall",IF(LEFT(G60,7)="Gondola","Gondola",IF(LEFT(G60,6)="Pallet","Pallet",IF(LEFT(G60,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I60" s="12">
+        <f>IF(A60="","",IF(D60="","CEK ID FIXTURE kosong",IF(G60="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H60="Endcap","CEK Endcap tidak ikut sambung",IF(H60&lt;&gt;B60,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C60="","CEK URUTAN kosong",IF(AND(E60&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E60)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="n"/>
+      <c r="B61" s="10" t="n"/>
+      <c r="C61" s="10" t="n"/>
+      <c r="D61" s="11" t="n"/>
+      <c r="E61" s="10" t="n"/>
+      <c r="F61" s="10" t="n"/>
+      <c r="G61" s="12">
+        <f>IF(D61="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D61,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H61" s="12">
+        <f>IF(G61="","",IF(LEFT(G61,4)="Wall","Wall",IF(LEFT(G61,7)="Gondola","Gondola",IF(LEFT(G61,6)="Pallet","Pallet",IF(LEFT(G61,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I61" s="12">
+        <f>IF(A61="","",IF(D61="","CEK ID FIXTURE kosong",IF(G61="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H61="Endcap","CEK Endcap tidak ikut sambung",IF(H61&lt;&gt;B61,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C61="","CEK URUTAN kosong",IF(AND(E61&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E61)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="n"/>
+      <c r="B62" s="10" t="n"/>
+      <c r="C62" s="10" t="n"/>
+      <c r="D62" s="11" t="n"/>
+      <c r="E62" s="10" t="n"/>
+      <c r="F62" s="10" t="n"/>
+      <c r="G62" s="12">
+        <f>IF(D62="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D62,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H62" s="12">
+        <f>IF(G62="","",IF(LEFT(G62,4)="Wall","Wall",IF(LEFT(G62,7)="Gondola","Gondola",IF(LEFT(G62,6)="Pallet","Pallet",IF(LEFT(G62,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I62" s="12">
+        <f>IF(A62="","",IF(D62="","CEK ID FIXTURE kosong",IF(G62="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H62="Endcap","CEK Endcap tidak ikut sambung",IF(H62&lt;&gt;B62,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C62="","CEK URUTAN kosong",IF(AND(E62&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E62)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="n"/>
+      <c r="B63" s="10" t="n"/>
+      <c r="C63" s="10" t="n"/>
+      <c r="D63" s="11" t="n"/>
+      <c r="E63" s="10" t="n"/>
+      <c r="F63" s="10" t="n"/>
+      <c r="G63" s="12">
+        <f>IF(D63="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D63,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H63" s="12">
+        <f>IF(G63="","",IF(LEFT(G63,4)="Wall","Wall",IF(LEFT(G63,7)="Gondola","Gondola",IF(LEFT(G63,6)="Pallet","Pallet",IF(LEFT(G63,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I63" s="12">
+        <f>IF(A63="","",IF(D63="","CEK ID FIXTURE kosong",IF(G63="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H63="Endcap","CEK Endcap tidak ikut sambung",IF(H63&lt;&gt;B63,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C63="","CEK URUTAN kosong",IF(AND(E63&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E63)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="n"/>
+      <c r="B64" s="10" t="n"/>
+      <c r="C64" s="10" t="n"/>
+      <c r="D64" s="11" t="n"/>
+      <c r="E64" s="10" t="n"/>
+      <c r="F64" s="10" t="n"/>
+      <c r="G64" s="12">
+        <f>IF(D64="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D64,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H64" s="12">
+        <f>IF(G64="","",IF(LEFT(G64,4)="Wall","Wall",IF(LEFT(G64,7)="Gondola","Gondola",IF(LEFT(G64,6)="Pallet","Pallet",IF(LEFT(G64,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I64" s="12">
+        <f>IF(A64="","",IF(D64="","CEK ID FIXTURE kosong",IF(G64="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H64="Endcap","CEK Endcap tidak ikut sambung",IF(H64&lt;&gt;B64,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C64="","CEK URUTAN kosong",IF(AND(E64&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E64)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="n"/>
+      <c r="B65" s="10" t="n"/>
+      <c r="C65" s="10" t="n"/>
+      <c r="D65" s="11" t="n"/>
+      <c r="E65" s="10" t="n"/>
+      <c r="F65" s="10" t="n"/>
+      <c r="G65" s="12">
+        <f>IF(D65="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D65,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H65" s="12">
+        <f>IF(G65="","",IF(LEFT(G65,4)="Wall","Wall",IF(LEFT(G65,7)="Gondola","Gondola",IF(LEFT(G65,6)="Pallet","Pallet",IF(LEFT(G65,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I65" s="12">
+        <f>IF(A65="","",IF(D65="","CEK ID FIXTURE kosong",IF(G65="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H65="Endcap","CEK Endcap tidak ikut sambung",IF(H65&lt;&gt;B65,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C65="","CEK URUTAN kosong",IF(AND(E65&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E65)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="10" t="n"/>
+      <c r="B66" s="10" t="n"/>
+      <c r="C66" s="10" t="n"/>
+      <c r="D66" s="11" t="n"/>
+      <c r="E66" s="10" t="n"/>
+      <c r="F66" s="10" t="n"/>
+      <c r="G66" s="12">
+        <f>IF(D66="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D66,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H66" s="12">
+        <f>IF(G66="","",IF(LEFT(G66,4)="Wall","Wall",IF(LEFT(G66,7)="Gondola","Gondola",IF(LEFT(G66,6)="Pallet","Pallet",IF(LEFT(G66,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I66" s="12">
+        <f>IF(A66="","",IF(D66="","CEK ID FIXTURE kosong",IF(G66="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H66="Endcap","CEK Endcap tidak ikut sambung",IF(H66&lt;&gt;B66,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C66="","CEK URUTAN kosong",IF(AND(E66&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E66)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="n"/>
+      <c r="B67" s="10" t="n"/>
+      <c r="C67" s="10" t="n"/>
+      <c r="D67" s="11" t="n"/>
+      <c r="E67" s="10" t="n"/>
+      <c r="F67" s="10" t="n"/>
+      <c r="G67" s="12">
+        <f>IF(D67="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D67,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H67" s="12">
+        <f>IF(G67="","",IF(LEFT(G67,4)="Wall","Wall",IF(LEFT(G67,7)="Gondola","Gondola",IF(LEFT(G67,6)="Pallet","Pallet",IF(LEFT(G67,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I67" s="12">
+        <f>IF(A67="","",IF(D67="","CEK ID FIXTURE kosong",IF(G67="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H67="Endcap","CEK Endcap tidak ikut sambung",IF(H67&lt;&gt;B67,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C67="","CEK URUTAN kosong",IF(AND(E67&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E67)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="n"/>
+      <c r="B68" s="10" t="n"/>
+      <c r="C68" s="10" t="n"/>
+      <c r="D68" s="11" t="n"/>
+      <c r="E68" s="10" t="n"/>
+      <c r="F68" s="10" t="n"/>
+      <c r="G68" s="12">
+        <f>IF(D68="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D68,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H68" s="12">
+        <f>IF(G68="","",IF(LEFT(G68,4)="Wall","Wall",IF(LEFT(G68,7)="Gondola","Gondola",IF(LEFT(G68,6)="Pallet","Pallet",IF(LEFT(G68,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I68" s="12">
+        <f>IF(A68="","",IF(D68="","CEK ID FIXTURE kosong",IF(G68="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H68="Endcap","CEK Endcap tidak ikut sambung",IF(H68&lt;&gt;B68,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C68="","CEK URUTAN kosong",IF(AND(E68&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E68)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="n"/>
+      <c r="B69" s="10" t="n"/>
+      <c r="C69" s="10" t="n"/>
+      <c r="D69" s="11" t="n"/>
+      <c r="E69" s="10" t="n"/>
+      <c r="F69" s="10" t="n"/>
+      <c r="G69" s="12">
+        <f>IF(D69="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D69,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H69" s="12">
+        <f>IF(G69="","",IF(LEFT(G69,4)="Wall","Wall",IF(LEFT(G69,7)="Gondola","Gondola",IF(LEFT(G69,6)="Pallet","Pallet",IF(LEFT(G69,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I69" s="12">
+        <f>IF(A69="","",IF(D69="","CEK ID FIXTURE kosong",IF(G69="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H69="Endcap","CEK Endcap tidak ikut sambung",IF(H69&lt;&gt;B69,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C69="","CEK URUTAN kosong",IF(AND(E69&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E69)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="10" t="n"/>
+      <c r="B70" s="10" t="n"/>
+      <c r="C70" s="10" t="n"/>
+      <c r="D70" s="11" t="n"/>
+      <c r="E70" s="10" t="n"/>
+      <c r="F70" s="10" t="n"/>
+      <c r="G70" s="12">
+        <f>IF(D70="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D70,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H70" s="12">
+        <f>IF(G70="","",IF(LEFT(G70,4)="Wall","Wall",IF(LEFT(G70,7)="Gondola","Gondola",IF(LEFT(G70,6)="Pallet","Pallet",IF(LEFT(G70,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I70" s="12">
+        <f>IF(A70="","",IF(D70="","CEK ID FIXTURE kosong",IF(G70="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H70="Endcap","CEK Endcap tidak ikut sambung",IF(H70&lt;&gt;B70,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C70="","CEK URUTAN kosong",IF(AND(E70&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E70)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="10" t="n"/>
+      <c r="B71" s="10" t="n"/>
+      <c r="C71" s="10" t="n"/>
+      <c r="D71" s="11" t="n"/>
+      <c r="E71" s="10" t="n"/>
+      <c r="F71" s="10" t="n"/>
+      <c r="G71" s="12">
+        <f>IF(D71="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D71,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H71" s="12">
+        <f>IF(G71="","",IF(LEFT(G71,4)="Wall","Wall",IF(LEFT(G71,7)="Gondola","Gondola",IF(LEFT(G71,6)="Pallet","Pallet",IF(LEFT(G71,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I71" s="12">
+        <f>IF(A71="","",IF(D71="","CEK ID FIXTURE kosong",IF(G71="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H71="Endcap","CEK Endcap tidak ikut sambung",IF(H71&lt;&gt;B71,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C71="","CEK URUTAN kosong",IF(AND(E71&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E71)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="n"/>
+      <c r="B72" s="10" t="n"/>
+      <c r="C72" s="10" t="n"/>
+      <c r="D72" s="11" t="n"/>
+      <c r="E72" s="10" t="n"/>
+      <c r="F72" s="10" t="n"/>
+      <c r="G72" s="12">
+        <f>IF(D72="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D72,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H72" s="12">
+        <f>IF(G72="","",IF(LEFT(G72,4)="Wall","Wall",IF(LEFT(G72,7)="Gondola","Gondola",IF(LEFT(G72,6)="Pallet","Pallet",IF(LEFT(G72,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I72" s="12">
+        <f>IF(A72="","",IF(D72="","CEK ID FIXTURE kosong",IF(G72="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H72="Endcap","CEK Endcap tidak ikut sambung",IF(H72&lt;&gt;B72,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C72="","CEK URUTAN kosong",IF(AND(E72&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E72)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="n"/>
+      <c r="B73" s="10" t="n"/>
+      <c r="C73" s="10" t="n"/>
+      <c r="D73" s="11" t="n"/>
+      <c r="E73" s="10" t="n"/>
+      <c r="F73" s="10" t="n"/>
+      <c r="G73" s="12">
+        <f>IF(D73="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D73,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H73" s="12">
+        <f>IF(G73="","",IF(LEFT(G73,4)="Wall","Wall",IF(LEFT(G73,7)="Gondola","Gondola",IF(LEFT(G73,6)="Pallet","Pallet",IF(LEFT(G73,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I73" s="12">
+        <f>IF(A73="","",IF(D73="","CEK ID FIXTURE kosong",IF(G73="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H73="Endcap","CEK Endcap tidak ikut sambung",IF(H73&lt;&gt;B73,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C73="","CEK URUTAN kosong",IF(AND(E73&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E73)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="n"/>
+      <c r="B74" s="10" t="n"/>
+      <c r="C74" s="10" t="n"/>
+      <c r="D74" s="11" t="n"/>
+      <c r="E74" s="10" t="n"/>
+      <c r="F74" s="10" t="n"/>
+      <c r="G74" s="12">
+        <f>IF(D74="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D74,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H74" s="12">
+        <f>IF(G74="","",IF(LEFT(G74,4)="Wall","Wall",IF(LEFT(G74,7)="Gondola","Gondola",IF(LEFT(G74,6)="Pallet","Pallet",IF(LEFT(G74,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I74" s="12">
+        <f>IF(A74="","",IF(D74="","CEK ID FIXTURE kosong",IF(G74="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H74="Endcap","CEK Endcap tidak ikut sambung",IF(H74&lt;&gt;B74,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C74="","CEK URUTAN kosong",IF(AND(E74&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E74)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="n"/>
+      <c r="B75" s="10" t="n"/>
+      <c r="C75" s="10" t="n"/>
+      <c r="D75" s="11" t="n"/>
+      <c r="E75" s="10" t="n"/>
+      <c r="F75" s="10" t="n"/>
+      <c r="G75" s="12">
+        <f>IF(D75="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D75,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H75" s="12">
+        <f>IF(G75="","",IF(LEFT(G75,4)="Wall","Wall",IF(LEFT(G75,7)="Gondola","Gondola",IF(LEFT(G75,6)="Pallet","Pallet",IF(LEFT(G75,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I75" s="12">
+        <f>IF(A75="","",IF(D75="","CEK ID FIXTURE kosong",IF(G75="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H75="Endcap","CEK Endcap tidak ikut sambung",IF(H75&lt;&gt;B75,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C75="","CEK URUTAN kosong",IF(AND(E75&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E75)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="n"/>
+      <c r="B76" s="10" t="n"/>
+      <c r="C76" s="10" t="n"/>
+      <c r="D76" s="11" t="n"/>
+      <c r="E76" s="10" t="n"/>
+      <c r="F76" s="10" t="n"/>
+      <c r="G76" s="12">
+        <f>IF(D76="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D76,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H76" s="12">
+        <f>IF(G76="","",IF(LEFT(G76,4)="Wall","Wall",IF(LEFT(G76,7)="Gondola","Gondola",IF(LEFT(G76,6)="Pallet","Pallet",IF(LEFT(G76,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I76" s="12">
+        <f>IF(A76="","",IF(D76="","CEK ID FIXTURE kosong",IF(G76="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H76="Endcap","CEK Endcap tidak ikut sambung",IF(H76&lt;&gt;B76,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C76="","CEK URUTAN kosong",IF(AND(E76&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E76)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="n"/>
+      <c r="B77" s="10" t="n"/>
+      <c r="C77" s="10" t="n"/>
+      <c r="D77" s="11" t="n"/>
+      <c r="E77" s="10" t="n"/>
+      <c r="F77" s="10" t="n"/>
+      <c r="G77" s="12">
+        <f>IF(D77="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D77,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H77" s="12">
+        <f>IF(G77="","",IF(LEFT(G77,4)="Wall","Wall",IF(LEFT(G77,7)="Gondola","Gondola",IF(LEFT(G77,6)="Pallet","Pallet",IF(LEFT(G77,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I77" s="12">
+        <f>IF(A77="","",IF(D77="","CEK ID FIXTURE kosong",IF(G77="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H77="Endcap","CEK Endcap tidak ikut sambung",IF(H77&lt;&gt;B77,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C77="","CEK URUTAN kosong",IF(AND(E77&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E77)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="n"/>
+      <c r="B78" s="10" t="n"/>
+      <c r="C78" s="10" t="n"/>
+      <c r="D78" s="11" t="n"/>
+      <c r="E78" s="10" t="n"/>
+      <c r="F78" s="10" t="n"/>
+      <c r="G78" s="12">
+        <f>IF(D78="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D78,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H78" s="12">
+        <f>IF(G78="","",IF(LEFT(G78,4)="Wall","Wall",IF(LEFT(G78,7)="Gondola","Gondola",IF(LEFT(G78,6)="Pallet","Pallet",IF(LEFT(G78,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I78" s="12">
+        <f>IF(A78="","",IF(D78="","CEK ID FIXTURE kosong",IF(G78="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H78="Endcap","CEK Endcap tidak ikut sambung",IF(H78&lt;&gt;B78,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C78="","CEK URUTAN kosong",IF(AND(E78&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E78)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="n"/>
+      <c r="B79" s="10" t="n"/>
+      <c r="C79" s="10" t="n"/>
+      <c r="D79" s="11" t="n"/>
+      <c r="E79" s="10" t="n"/>
+      <c r="F79" s="10" t="n"/>
+      <c r="G79" s="12">
+        <f>IF(D79="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D79,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H79" s="12">
+        <f>IF(G79="","",IF(LEFT(G79,4)="Wall","Wall",IF(LEFT(G79,7)="Gondola","Gondola",IF(LEFT(G79,6)="Pallet","Pallet",IF(LEFT(G79,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I79" s="12">
+        <f>IF(A79="","",IF(D79="","CEK ID FIXTURE kosong",IF(G79="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H79="Endcap","CEK Endcap tidak ikut sambung",IF(H79&lt;&gt;B79,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C79="","CEK URUTAN kosong",IF(AND(E79&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E79)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="n"/>
+      <c r="B80" s="10" t="n"/>
+      <c r="C80" s="10" t="n"/>
+      <c r="D80" s="11" t="n"/>
+      <c r="E80" s="10" t="n"/>
+      <c r="F80" s="10" t="n"/>
+      <c r="G80" s="12">
+        <f>IF(D80="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D80,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H80" s="12">
+        <f>IF(G80="","",IF(LEFT(G80,4)="Wall","Wall",IF(LEFT(G80,7)="Gondola","Gondola",IF(LEFT(G80,6)="Pallet","Pallet",IF(LEFT(G80,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I80" s="12">
+        <f>IF(A80="","",IF(D80="","CEK ID FIXTURE kosong",IF(G80="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H80="Endcap","CEK Endcap tidak ikut sambung",IF(H80&lt;&gt;B80,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C80="","CEK URUTAN kosong",IF(AND(E80&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E80)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="n"/>
+      <c r="B81" s="10" t="n"/>
+      <c r="C81" s="10" t="n"/>
+      <c r="D81" s="11" t="n"/>
+      <c r="E81" s="10" t="n"/>
+      <c r="F81" s="10" t="n"/>
+      <c r="G81" s="12">
+        <f>IF(D81="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D81,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H81" s="12">
+        <f>IF(G81="","",IF(LEFT(G81,4)="Wall","Wall",IF(LEFT(G81,7)="Gondola","Gondola",IF(LEFT(G81,6)="Pallet","Pallet",IF(LEFT(G81,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I81" s="12">
+        <f>IF(A81="","",IF(D81="","CEK ID FIXTURE kosong",IF(G81="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H81="Endcap","CEK Endcap tidak ikut sambung",IF(H81&lt;&gt;B81,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C81="","CEK URUTAN kosong",IF(AND(E81&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E81)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="n"/>
+      <c r="B82" s="10" t="n"/>
+      <c r="C82" s="10" t="n"/>
+      <c r="D82" s="11" t="n"/>
+      <c r="E82" s="10" t="n"/>
+      <c r="F82" s="10" t="n"/>
+      <c r="G82" s="12">
+        <f>IF(D82="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D82,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H82" s="12">
+        <f>IF(G82="","",IF(LEFT(G82,4)="Wall","Wall",IF(LEFT(G82,7)="Gondola","Gondola",IF(LEFT(G82,6)="Pallet","Pallet",IF(LEFT(G82,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I82" s="12">
+        <f>IF(A82="","",IF(D82="","CEK ID FIXTURE kosong",IF(G82="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H82="Endcap","CEK Endcap tidak ikut sambung",IF(H82&lt;&gt;B82,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C82="","CEK URUTAN kosong",IF(AND(E82&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E82)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n"/>
+      <c r="B83" s="10" t="n"/>
+      <c r="C83" s="10" t="n"/>
+      <c r="D83" s="11" t="n"/>
+      <c r="E83" s="10" t="n"/>
+      <c r="F83" s="10" t="n"/>
+      <c r="G83" s="12">
+        <f>IF(D83="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D83,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H83" s="12">
+        <f>IF(G83="","",IF(LEFT(G83,4)="Wall","Wall",IF(LEFT(G83,7)="Gondola","Gondola",IF(LEFT(G83,6)="Pallet","Pallet",IF(LEFT(G83,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I83" s="12">
+        <f>IF(A83="","",IF(D83="","CEK ID FIXTURE kosong",IF(G83="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H83="Endcap","CEK Endcap tidak ikut sambung",IF(H83&lt;&gt;B83,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C83="","CEK URUTAN kosong",IF(AND(E83&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E83)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n"/>
+      <c r="B84" s="10" t="n"/>
+      <c r="C84" s="10" t="n"/>
+      <c r="D84" s="11" t="n"/>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="10" t="n"/>
+      <c r="G84" s="12">
+        <f>IF(D84="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D84,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H84" s="12">
+        <f>IF(G84="","",IF(LEFT(G84,4)="Wall","Wall",IF(LEFT(G84,7)="Gondola","Gondola",IF(LEFT(G84,6)="Pallet","Pallet",IF(LEFT(G84,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I84" s="12">
+        <f>IF(A84="","",IF(D84="","CEK ID FIXTURE kosong",IF(G84="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H84="Endcap","CEK Endcap tidak ikut sambung",IF(H84&lt;&gt;B84,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C84="","CEK URUTAN kosong",IF(AND(E84&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E84)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="n"/>
+      <c r="B85" s="10" t="n"/>
+      <c r="C85" s="10" t="n"/>
+      <c r="D85" s="11" t="n"/>
+      <c r="E85" s="10" t="n"/>
+      <c r="F85" s="10" t="n"/>
+      <c r="G85" s="12">
+        <f>IF(D85="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D85,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H85" s="12">
+        <f>IF(G85="","",IF(LEFT(G85,4)="Wall","Wall",IF(LEFT(G85,7)="Gondola","Gondola",IF(LEFT(G85,6)="Pallet","Pallet",IF(LEFT(G85,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I85" s="12">
+        <f>IF(A85="","",IF(D85="","CEK ID FIXTURE kosong",IF(G85="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H85="Endcap","CEK Endcap tidak ikut sambung",IF(H85&lt;&gt;B85,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C85="","CEK URUTAN kosong",IF(AND(E85&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E85)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n"/>
+      <c r="B86" s="10" t="n"/>
+      <c r="C86" s="10" t="n"/>
+      <c r="D86" s="11" t="n"/>
+      <c r="E86" s="10" t="n"/>
+      <c r="F86" s="10" t="n"/>
+      <c r="G86" s="12">
+        <f>IF(D86="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D86,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H86" s="12">
+        <f>IF(G86="","",IF(LEFT(G86,4)="Wall","Wall",IF(LEFT(G86,7)="Gondola","Gondola",IF(LEFT(G86,6)="Pallet","Pallet",IF(LEFT(G86,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I86" s="12">
+        <f>IF(A86="","",IF(D86="","CEK ID FIXTURE kosong",IF(G86="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H86="Endcap","CEK Endcap tidak ikut sambung",IF(H86&lt;&gt;B86,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C86="","CEK URUTAN kosong",IF(AND(E86&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E86)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="n"/>
+      <c r="B87" s="10" t="n"/>
+      <c r="C87" s="10" t="n"/>
+      <c r="D87" s="11" t="n"/>
+      <c r="E87" s="10" t="n"/>
+      <c r="F87" s="10" t="n"/>
+      <c r="G87" s="12">
+        <f>IF(D87="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D87,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H87" s="12">
+        <f>IF(G87="","",IF(LEFT(G87,4)="Wall","Wall",IF(LEFT(G87,7)="Gondola","Gondola",IF(LEFT(G87,6)="Pallet","Pallet",IF(LEFT(G87,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I87" s="12">
+        <f>IF(A87="","",IF(D87="","CEK ID FIXTURE kosong",IF(G87="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H87="Endcap","CEK Endcap tidak ikut sambung",IF(H87&lt;&gt;B87,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C87="","CEK URUTAN kosong",IF(AND(E87&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E87)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="n"/>
+      <c r="B88" s="10" t="n"/>
+      <c r="C88" s="10" t="n"/>
+      <c r="D88" s="11" t="n"/>
+      <c r="E88" s="10" t="n"/>
+      <c r="F88" s="10" t="n"/>
+      <c r="G88" s="12">
+        <f>IF(D88="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D88,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H88" s="12">
+        <f>IF(G88="","",IF(LEFT(G88,4)="Wall","Wall",IF(LEFT(G88,7)="Gondola","Gondola",IF(LEFT(G88,6)="Pallet","Pallet",IF(LEFT(G88,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I88" s="12">
+        <f>IF(A88="","",IF(D88="","CEK ID FIXTURE kosong",IF(G88="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H88="Endcap","CEK Endcap tidak ikut sambung",IF(H88&lt;&gt;B88,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C88="","CEK URUTAN kosong",IF(AND(E88&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E88)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="n"/>
+      <c r="B89" s="10" t="n"/>
+      <c r="C89" s="10" t="n"/>
+      <c r="D89" s="11" t="n"/>
+      <c r="E89" s="10" t="n"/>
+      <c r="F89" s="10" t="n"/>
+      <c r="G89" s="12">
+        <f>IF(D89="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D89,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H89" s="12">
+        <f>IF(G89="","",IF(LEFT(G89,4)="Wall","Wall",IF(LEFT(G89,7)="Gondola","Gondola",IF(LEFT(G89,6)="Pallet","Pallet",IF(LEFT(G89,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I89" s="12">
+        <f>IF(A89="","",IF(D89="","CEK ID FIXTURE kosong",IF(G89="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H89="Endcap","CEK Endcap tidak ikut sambung",IF(H89&lt;&gt;B89,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C89="","CEK URUTAN kosong",IF(AND(E89&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E89)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="n"/>
+      <c r="B90" s="10" t="n"/>
+      <c r="C90" s="10" t="n"/>
+      <c r="D90" s="11" t="n"/>
+      <c r="E90" s="10" t="n"/>
+      <c r="F90" s="10" t="n"/>
+      <c r="G90" s="12">
+        <f>IF(D90="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D90,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H90" s="12">
+        <f>IF(G90="","",IF(LEFT(G90,4)="Wall","Wall",IF(LEFT(G90,7)="Gondola","Gondola",IF(LEFT(G90,6)="Pallet","Pallet",IF(LEFT(G90,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I90" s="12">
+        <f>IF(A90="","",IF(D90="","CEK ID FIXTURE kosong",IF(G90="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H90="Endcap","CEK Endcap tidak ikut sambung",IF(H90&lt;&gt;B90,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C90="","CEK URUTAN kosong",IF(AND(E90&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E90)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="n"/>
+      <c r="B91" s="10" t="n"/>
+      <c r="C91" s="10" t="n"/>
+      <c r="D91" s="11" t="n"/>
+      <c r="E91" s="10" t="n"/>
+      <c r="F91" s="10" t="n"/>
+      <c r="G91" s="12">
+        <f>IF(D91="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D91,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H91" s="12">
+        <f>IF(G91="","",IF(LEFT(G91,4)="Wall","Wall",IF(LEFT(G91,7)="Gondola","Gondola",IF(LEFT(G91,6)="Pallet","Pallet",IF(LEFT(G91,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I91" s="12">
+        <f>IF(A91="","",IF(D91="","CEK ID FIXTURE kosong",IF(G91="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H91="Endcap","CEK Endcap tidak ikut sambung",IF(H91&lt;&gt;B91,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C91="","CEK URUTAN kosong",IF(AND(E91&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E91)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="n"/>
+      <c r="B92" s="10" t="n"/>
+      <c r="C92" s="10" t="n"/>
+      <c r="D92" s="11" t="n"/>
+      <c r="E92" s="10" t="n"/>
+      <c r="F92" s="10" t="n"/>
+      <c r="G92" s="12">
+        <f>IF(D92="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D92,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H92" s="12">
+        <f>IF(G92="","",IF(LEFT(G92,4)="Wall","Wall",IF(LEFT(G92,7)="Gondola","Gondola",IF(LEFT(G92,6)="Pallet","Pallet",IF(LEFT(G92,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I92" s="12">
+        <f>IF(A92="","",IF(D92="","CEK ID FIXTURE kosong",IF(G92="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H92="Endcap","CEK Endcap tidak ikut sambung",IF(H92&lt;&gt;B92,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C92="","CEK URUTAN kosong",IF(AND(E92&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E92)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="n"/>
+      <c r="B93" s="10" t="n"/>
+      <c r="C93" s="10" t="n"/>
+      <c r="D93" s="11" t="n"/>
+      <c r="E93" s="10" t="n"/>
+      <c r="F93" s="10" t="n"/>
+      <c r="G93" s="12">
+        <f>IF(D93="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D93,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H93" s="12">
+        <f>IF(G93="","",IF(LEFT(G93,4)="Wall","Wall",IF(LEFT(G93,7)="Gondola","Gondola",IF(LEFT(G93,6)="Pallet","Pallet",IF(LEFT(G93,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I93" s="12">
+        <f>IF(A93="","",IF(D93="","CEK ID FIXTURE kosong",IF(G93="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H93="Endcap","CEK Endcap tidak ikut sambung",IF(H93&lt;&gt;B93,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C93="","CEK URUTAN kosong",IF(AND(E93&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E93)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="n"/>
+      <c r="B94" s="10" t="n"/>
+      <c r="C94" s="10" t="n"/>
+      <c r="D94" s="11" t="n"/>
+      <c r="E94" s="10" t="n"/>
+      <c r="F94" s="10" t="n"/>
+      <c r="G94" s="12">
+        <f>IF(D94="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D94,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H94" s="12">
+        <f>IF(G94="","",IF(LEFT(G94,4)="Wall","Wall",IF(LEFT(G94,7)="Gondola","Gondola",IF(LEFT(G94,6)="Pallet","Pallet",IF(LEFT(G94,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I94" s="12">
+        <f>IF(A94="","",IF(D94="","CEK ID FIXTURE kosong",IF(G94="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H94="Endcap","CEK Endcap tidak ikut sambung",IF(H94&lt;&gt;B94,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C94="","CEK URUTAN kosong",IF(AND(E94&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E94)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="n"/>
+      <c r="B95" s="10" t="n"/>
+      <c r="C95" s="10" t="n"/>
+      <c r="D95" s="11" t="n"/>
+      <c r="E95" s="10" t="n"/>
+      <c r="F95" s="10" t="n"/>
+      <c r="G95" s="12">
+        <f>IF(D95="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D95,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H95" s="12">
+        <f>IF(G95="","",IF(LEFT(G95,4)="Wall","Wall",IF(LEFT(G95,7)="Gondola","Gondola",IF(LEFT(G95,6)="Pallet","Pallet",IF(LEFT(G95,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I95" s="12">
+        <f>IF(A95="","",IF(D95="","CEK ID FIXTURE kosong",IF(G95="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H95="Endcap","CEK Endcap tidak ikut sambung",IF(H95&lt;&gt;B95,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C95="","CEK URUTAN kosong",IF(AND(E95&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E95)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="n"/>
+      <c r="B96" s="10" t="n"/>
+      <c r="C96" s="10" t="n"/>
+      <c r="D96" s="11" t="n"/>
+      <c r="E96" s="10" t="n"/>
+      <c r="F96" s="10" t="n"/>
+      <c r="G96" s="12">
+        <f>IF(D96="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D96,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H96" s="12">
+        <f>IF(G96="","",IF(LEFT(G96,4)="Wall","Wall",IF(LEFT(G96,7)="Gondola","Gondola",IF(LEFT(G96,6)="Pallet","Pallet",IF(LEFT(G96,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I96" s="12">
+        <f>IF(A96="","",IF(D96="","CEK ID FIXTURE kosong",IF(G96="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H96="Endcap","CEK Endcap tidak ikut sambung",IF(H96&lt;&gt;B96,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C96="","CEK URUTAN kosong",IF(AND(E96&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E96)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="n"/>
+      <c r="B97" s="10" t="n"/>
+      <c r="C97" s="10" t="n"/>
+      <c r="D97" s="11" t="n"/>
+      <c r="E97" s="10" t="n"/>
+      <c r="F97" s="10" t="n"/>
+      <c r="G97" s="12">
+        <f>IF(D97="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D97,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H97" s="12">
+        <f>IF(G97="","",IF(LEFT(G97,4)="Wall","Wall",IF(LEFT(G97,7)="Gondola","Gondola",IF(LEFT(G97,6)="Pallet","Pallet",IF(LEFT(G97,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I97" s="12">
+        <f>IF(A97="","",IF(D97="","CEK ID FIXTURE kosong",IF(G97="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H97="Endcap","CEK Endcap tidak ikut sambung",IF(H97&lt;&gt;B97,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C97="","CEK URUTAN kosong",IF(AND(E97&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E97)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="n"/>
+      <c r="B98" s="10" t="n"/>
+      <c r="C98" s="10" t="n"/>
+      <c r="D98" s="11" t="n"/>
+      <c r="E98" s="10" t="n"/>
+      <c r="F98" s="10" t="n"/>
+      <c r="G98" s="12">
+        <f>IF(D98="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D98,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H98" s="12">
+        <f>IF(G98="","",IF(LEFT(G98,4)="Wall","Wall",IF(LEFT(G98,7)="Gondola","Gondola",IF(LEFT(G98,6)="Pallet","Pallet",IF(LEFT(G98,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I98" s="12">
+        <f>IF(A98="","",IF(D98="","CEK ID FIXTURE kosong",IF(G98="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H98="Endcap","CEK Endcap tidak ikut sambung",IF(H98&lt;&gt;B98,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C98="","CEK URUTAN kosong",IF(AND(E98&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E98)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="n"/>
+      <c r="B99" s="10" t="n"/>
+      <c r="C99" s="10" t="n"/>
+      <c r="D99" s="11" t="n"/>
+      <c r="E99" s="10" t="n"/>
+      <c r="F99" s="10" t="n"/>
+      <c r="G99" s="12">
+        <f>IF(D99="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D99,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H99" s="12">
+        <f>IF(G99="","",IF(LEFT(G99,4)="Wall","Wall",IF(LEFT(G99,7)="Gondola","Gondola",IF(LEFT(G99,6)="Pallet","Pallet",IF(LEFT(G99,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I99" s="12">
+        <f>IF(A99="","",IF(D99="","CEK ID FIXTURE kosong",IF(G99="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H99="Endcap","CEK Endcap tidak ikut sambung",IF(H99&lt;&gt;B99,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C99="","CEK URUTAN kosong",IF(AND(E99&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E99)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="n"/>
+      <c r="B100" s="10" t="n"/>
+      <c r="C100" s="10" t="n"/>
+      <c r="D100" s="11" t="n"/>
+      <c r="E100" s="10" t="n"/>
+      <c r="F100" s="10" t="n"/>
+      <c r="G100" s="12">
+        <f>IF(D100="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D100,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H100" s="12">
+        <f>IF(G100="","",IF(LEFT(G100,4)="Wall","Wall",IF(LEFT(G100,7)="Gondola","Gondola",IF(LEFT(G100,6)="Pallet","Pallet",IF(LEFT(G100,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I100" s="12">
+        <f>IF(A100="","",IF(D100="","CEK ID FIXTURE kosong",IF(G100="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H100="Endcap","CEK Endcap tidak ikut sambung",IF(H100&lt;&gt;B100,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C100="","CEK URUTAN kosong",IF(AND(E100&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E100)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="n"/>
+      <c r="B101" s="10" t="n"/>
+      <c r="C101" s="10" t="n"/>
+      <c r="D101" s="11" t="n"/>
+      <c r="E101" s="10" t="n"/>
+      <c r="F101" s="10" t="n"/>
+      <c r="G101" s="12">
+        <f>IF(D101="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D101,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H101" s="12">
+        <f>IF(G101="","",IF(LEFT(G101,4)="Wall","Wall",IF(LEFT(G101,7)="Gondola","Gondola",IF(LEFT(G101,6)="Pallet","Pallet",IF(LEFT(G101,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I101" s="12">
+        <f>IF(A101="","",IF(D101="","CEK ID FIXTURE kosong",IF(G101="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H101="Endcap","CEK Endcap tidak ikut sambung",IF(H101&lt;&gt;B101,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C101="","CEK URUTAN kosong",IF(AND(E101&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E101)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="n"/>
+      <c r="B102" s="10" t="n"/>
+      <c r="C102" s="10" t="n"/>
+      <c r="D102" s="11" t="n"/>
+      <c r="E102" s="10" t="n"/>
+      <c r="F102" s="10" t="n"/>
+      <c r="G102" s="12">
+        <f>IF(D102="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D102,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H102" s="12">
+        <f>IF(G102="","",IF(LEFT(G102,4)="Wall","Wall",IF(LEFT(G102,7)="Gondola","Gondola",IF(LEFT(G102,6)="Pallet","Pallet",IF(LEFT(G102,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I102" s="12">
+        <f>IF(A102="","",IF(D102="","CEK ID FIXTURE kosong",IF(G102="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H102="Endcap","CEK Endcap tidak ikut sambung",IF(H102&lt;&gt;B102,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C102="","CEK URUTAN kosong",IF(AND(E102&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E102)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="n"/>
+      <c r="B103" s="10" t="n"/>
+      <c r="C103" s="10" t="n"/>
+      <c r="D103" s="11" t="n"/>
+      <c r="E103" s="10" t="n"/>
+      <c r="F103" s="10" t="n"/>
+      <c r="G103" s="12">
+        <f>IF(D103="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D103,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H103" s="12">
+        <f>IF(G103="","",IF(LEFT(G103,4)="Wall","Wall",IF(LEFT(G103,7)="Gondola","Gondola",IF(LEFT(G103,6)="Pallet","Pallet",IF(LEFT(G103,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I103" s="12">
+        <f>IF(A103="","",IF(D103="","CEK ID FIXTURE kosong",IF(G103="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H103="Endcap","CEK Endcap tidak ikut sambung",IF(H103&lt;&gt;B103,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C103="","CEK URUTAN kosong",IF(AND(E103&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E103)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="n"/>
+      <c r="B104" s="10" t="n"/>
+      <c r="C104" s="10" t="n"/>
+      <c r="D104" s="11" t="n"/>
+      <c r="E104" s="10" t="n"/>
+      <c r="F104" s="10" t="n"/>
+      <c r="G104" s="12">
+        <f>IF(D104="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D104,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H104" s="12">
+        <f>IF(G104="","",IF(LEFT(G104,4)="Wall","Wall",IF(LEFT(G104,7)="Gondola","Gondola",IF(LEFT(G104,6)="Pallet","Pallet",IF(LEFT(G104,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I104" s="12">
+        <f>IF(A104="","",IF(D104="","CEK ID FIXTURE kosong",IF(G104="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H104="Endcap","CEK Endcap tidak ikut sambung",IF(H104&lt;&gt;B104,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C104="","CEK URUTAN kosong",IF(AND(E104&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E104)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="n"/>
+      <c r="B105" s="10" t="n"/>
+      <c r="C105" s="10" t="n"/>
+      <c r="D105" s="11" t="n"/>
+      <c r="E105" s="10" t="n"/>
+      <c r="F105" s="10" t="n"/>
+      <c r="G105" s="12">
+        <f>IF(D105="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D105,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H105" s="12">
+        <f>IF(G105="","",IF(LEFT(G105,4)="Wall","Wall",IF(LEFT(G105,7)="Gondola","Gondola",IF(LEFT(G105,6)="Pallet","Pallet",IF(LEFT(G105,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I105" s="12">
+        <f>IF(A105="","",IF(D105="","CEK ID FIXTURE kosong",IF(G105="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H105="Endcap","CEK Endcap tidak ikut sambung",IF(H105&lt;&gt;B105,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C105="","CEK URUTAN kosong",IF(AND(E105&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E105)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="n"/>
+      <c r="B106" s="10" t="n"/>
+      <c r="C106" s="10" t="n"/>
+      <c r="D106" s="11" t="n"/>
+      <c r="E106" s="10" t="n"/>
+      <c r="F106" s="10" t="n"/>
+      <c r="G106" s="12">
+        <f>IF(D106="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D106,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H106" s="12">
+        <f>IF(G106="","",IF(LEFT(G106,4)="Wall","Wall",IF(LEFT(G106,7)="Gondola","Gondola",IF(LEFT(G106,6)="Pallet","Pallet",IF(LEFT(G106,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I106" s="12">
+        <f>IF(A106="","",IF(D106="","CEK ID FIXTURE kosong",IF(G106="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H106="Endcap","CEK Endcap tidak ikut sambung",IF(H106&lt;&gt;B106,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C106="","CEK URUTAN kosong",IF(AND(E106&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E106)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="n"/>
+      <c r="B107" s="10" t="n"/>
+      <c r="C107" s="10" t="n"/>
+      <c r="D107" s="11" t="n"/>
+      <c r="E107" s="10" t="n"/>
+      <c r="F107" s="10" t="n"/>
+      <c r="G107" s="12">
+        <f>IF(D107="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D107,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H107" s="12">
+        <f>IF(G107="","",IF(LEFT(G107,4)="Wall","Wall",IF(LEFT(G107,7)="Gondola","Gondola",IF(LEFT(G107,6)="Pallet","Pallet",IF(LEFT(G107,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I107" s="12">
+        <f>IF(A107="","",IF(D107="","CEK ID FIXTURE kosong",IF(G107="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H107="Endcap","CEK Endcap tidak ikut sambung",IF(H107&lt;&gt;B107,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C107="","CEK URUTAN kosong",IF(AND(E107&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E107)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="10" t="n"/>
+      <c r="B108" s="10" t="n"/>
+      <c r="C108" s="10" t="n"/>
+      <c r="D108" s="11" t="n"/>
+      <c r="E108" s="10" t="n"/>
+      <c r="F108" s="10" t="n"/>
+      <c r="G108" s="12">
+        <f>IF(D108="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D108,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H108" s="12">
+        <f>IF(G108="","",IF(LEFT(G108,4)="Wall","Wall",IF(LEFT(G108,7)="Gondola","Gondola",IF(LEFT(G108,6)="Pallet","Pallet",IF(LEFT(G108,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I108" s="12">
+        <f>IF(A108="","",IF(D108="","CEK ID FIXTURE kosong",IF(G108="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H108="Endcap","CEK Endcap tidak ikut sambung",IF(H108&lt;&gt;B108,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C108="","CEK URUTAN kosong",IF(AND(E108&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E108)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="n"/>
+      <c r="B109" s="10" t="n"/>
+      <c r="C109" s="10" t="n"/>
+      <c r="D109" s="11" t="n"/>
+      <c r="E109" s="10" t="n"/>
+      <c r="F109" s="10" t="n"/>
+      <c r="G109" s="12">
+        <f>IF(D109="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D109,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H109" s="12">
+        <f>IF(G109="","",IF(LEFT(G109,4)="Wall","Wall",IF(LEFT(G109,7)="Gondola","Gondola",IF(LEFT(G109,6)="Pallet","Pallet",IF(LEFT(G109,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I109" s="12">
+        <f>IF(A109="","",IF(D109="","CEK ID FIXTURE kosong",IF(G109="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H109="Endcap","CEK Endcap tidak ikut sambung",IF(H109&lt;&gt;B109,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C109="","CEK URUTAN kosong",IF(AND(E109&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E109)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="n"/>
+      <c r="B110" s="10" t="n"/>
+      <c r="C110" s="10" t="n"/>
+      <c r="D110" s="11" t="n"/>
+      <c r="E110" s="10" t="n"/>
+      <c r="F110" s="10" t="n"/>
+      <c r="G110" s="12">
+        <f>IF(D110="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D110,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H110" s="12">
+        <f>IF(G110="","",IF(LEFT(G110,4)="Wall","Wall",IF(LEFT(G110,7)="Gondola","Gondola",IF(LEFT(G110,6)="Pallet","Pallet",IF(LEFT(G110,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I110" s="12">
+        <f>IF(A110="","",IF(D110="","CEK ID FIXTURE kosong",IF(G110="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H110="Endcap","CEK Endcap tidak ikut sambung",IF(H110&lt;&gt;B110,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C110="","CEK URUTAN kosong",IF(AND(E110&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E110)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="n"/>
+      <c r="B111" s="10" t="n"/>
+      <c r="C111" s="10" t="n"/>
+      <c r="D111" s="11" t="n"/>
+      <c r="E111" s="10" t="n"/>
+      <c r="F111" s="10" t="n"/>
+      <c r="G111" s="12">
+        <f>IF(D111="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D111,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H111" s="12">
+        <f>IF(G111="","",IF(LEFT(G111,4)="Wall","Wall",IF(LEFT(G111,7)="Gondola","Gondola",IF(LEFT(G111,6)="Pallet","Pallet",IF(LEFT(G111,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I111" s="12">
+        <f>IF(A111="","",IF(D111="","CEK ID FIXTURE kosong",IF(G111="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H111="Endcap","CEK Endcap tidak ikut sambung",IF(H111&lt;&gt;B111,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C111="","CEK URUTAN kosong",IF(AND(E111&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E111)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="n"/>
+      <c r="B112" s="10" t="n"/>
+      <c r="C112" s="10" t="n"/>
+      <c r="D112" s="11" t="n"/>
+      <c r="E112" s="10" t="n"/>
+      <c r="F112" s="10" t="n"/>
+      <c r="G112" s="12">
+        <f>IF(D112="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D112,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H112" s="12">
+        <f>IF(G112="","",IF(LEFT(G112,4)="Wall","Wall",IF(LEFT(G112,7)="Gondola","Gondola",IF(LEFT(G112,6)="Pallet","Pallet",IF(LEFT(G112,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I112" s="12">
+        <f>IF(A112="","",IF(D112="","CEK ID FIXTURE kosong",IF(G112="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H112="Endcap","CEK Endcap tidak ikut sambung",IF(H112&lt;&gt;B112,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C112="","CEK URUTAN kosong",IF(AND(E112&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E112)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="n"/>
+      <c r="B113" s="10" t="n"/>
+      <c r="C113" s="10" t="n"/>
+      <c r="D113" s="11" t="n"/>
+      <c r="E113" s="10" t="n"/>
+      <c r="F113" s="10" t="n"/>
+      <c r="G113" s="12">
+        <f>IF(D113="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D113,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H113" s="12">
+        <f>IF(G113="","",IF(LEFT(G113,4)="Wall","Wall",IF(LEFT(G113,7)="Gondola","Gondola",IF(LEFT(G113,6)="Pallet","Pallet",IF(LEFT(G113,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I113" s="12">
+        <f>IF(A113="","",IF(D113="","CEK ID FIXTURE kosong",IF(G113="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H113="Endcap","CEK Endcap tidak ikut sambung",IF(H113&lt;&gt;B113,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C113="","CEK URUTAN kosong",IF(AND(E113&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E113)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="n"/>
+      <c r="B114" s="10" t="n"/>
+      <c r="C114" s="10" t="n"/>
+      <c r="D114" s="11" t="n"/>
+      <c r="E114" s="10" t="n"/>
+      <c r="F114" s="10" t="n"/>
+      <c r="G114" s="12">
+        <f>IF(D114="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D114,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H114" s="12">
+        <f>IF(G114="","",IF(LEFT(G114,4)="Wall","Wall",IF(LEFT(G114,7)="Gondola","Gondola",IF(LEFT(G114,6)="Pallet","Pallet",IF(LEFT(G114,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I114" s="12">
+        <f>IF(A114="","",IF(D114="","CEK ID FIXTURE kosong",IF(G114="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H114="Endcap","CEK Endcap tidak ikut sambung",IF(H114&lt;&gt;B114,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C114="","CEK URUTAN kosong",IF(AND(E114&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E114)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="n"/>
+      <c r="B115" s="10" t="n"/>
+      <c r="C115" s="10" t="n"/>
+      <c r="D115" s="11" t="n"/>
+      <c r="E115" s="10" t="n"/>
+      <c r="F115" s="10" t="n"/>
+      <c r="G115" s="12">
+        <f>IF(D115="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D115,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H115" s="12">
+        <f>IF(G115="","",IF(LEFT(G115,4)="Wall","Wall",IF(LEFT(G115,7)="Gondola","Gondola",IF(LEFT(G115,6)="Pallet","Pallet",IF(LEFT(G115,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I115" s="12">
+        <f>IF(A115="","",IF(D115="","CEK ID FIXTURE kosong",IF(G115="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H115="Endcap","CEK Endcap tidak ikut sambung",IF(H115&lt;&gt;B115,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C115="","CEK URUTAN kosong",IF(AND(E115&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E115)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="n"/>
+      <c r="B116" s="10" t="n"/>
+      <c r="C116" s="10" t="n"/>
+      <c r="D116" s="11" t="n"/>
+      <c r="E116" s="10" t="n"/>
+      <c r="F116" s="10" t="n"/>
+      <c r="G116" s="12">
+        <f>IF(D116="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D116,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H116" s="12">
+        <f>IF(G116="","",IF(LEFT(G116,4)="Wall","Wall",IF(LEFT(G116,7)="Gondola","Gondola",IF(LEFT(G116,6)="Pallet","Pallet",IF(LEFT(G116,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I116" s="12">
+        <f>IF(A116="","",IF(D116="","CEK ID FIXTURE kosong",IF(G116="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H116="Endcap","CEK Endcap tidak ikut sambung",IF(H116&lt;&gt;B116,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C116="","CEK URUTAN kosong",IF(AND(E116&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E116)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="n"/>
+      <c r="B117" s="10" t="n"/>
+      <c r="C117" s="10" t="n"/>
+      <c r="D117" s="11" t="n"/>
+      <c r="E117" s="10" t="n"/>
+      <c r="F117" s="10" t="n"/>
+      <c r="G117" s="12">
+        <f>IF(D117="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D117,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H117" s="12">
+        <f>IF(G117="","",IF(LEFT(G117,4)="Wall","Wall",IF(LEFT(G117,7)="Gondola","Gondola",IF(LEFT(G117,6)="Pallet","Pallet",IF(LEFT(G117,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I117" s="12">
+        <f>IF(A117="","",IF(D117="","CEK ID FIXTURE kosong",IF(G117="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H117="Endcap","CEK Endcap tidak ikut sambung",IF(H117&lt;&gt;B117,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C117="","CEK URUTAN kosong",IF(AND(E117&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E117)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="n"/>
+      <c r="B118" s="10" t="n"/>
+      <c r="C118" s="10" t="n"/>
+      <c r="D118" s="11" t="n"/>
+      <c r="E118" s="10" t="n"/>
+      <c r="F118" s="10" t="n"/>
+      <c r="G118" s="12">
+        <f>IF(D118="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D118,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H118" s="12">
+        <f>IF(G118="","",IF(LEFT(G118,4)="Wall","Wall",IF(LEFT(G118,7)="Gondola","Gondola",IF(LEFT(G118,6)="Pallet","Pallet",IF(LEFT(G118,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I118" s="12">
+        <f>IF(A118="","",IF(D118="","CEK ID FIXTURE kosong",IF(G118="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H118="Endcap","CEK Endcap tidak ikut sambung",IF(H118&lt;&gt;B118,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C118="","CEK URUTAN kosong",IF(AND(E118&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E118)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="n"/>
+      <c r="B119" s="10" t="n"/>
+      <c r="C119" s="10" t="n"/>
+      <c r="D119" s="11" t="n"/>
+      <c r="E119" s="10" t="n"/>
+      <c r="F119" s="10" t="n"/>
+      <c r="G119" s="12">
+        <f>IF(D119="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D119,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H119" s="12">
+        <f>IF(G119="","",IF(LEFT(G119,4)="Wall","Wall",IF(LEFT(G119,7)="Gondola","Gondola",IF(LEFT(G119,6)="Pallet","Pallet",IF(LEFT(G119,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I119" s="12">
+        <f>IF(A119="","",IF(D119="","CEK ID FIXTURE kosong",IF(G119="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H119="Endcap","CEK Endcap tidak ikut sambung",IF(H119&lt;&gt;B119,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C119="","CEK URUTAN kosong",IF(AND(E119&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E119)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="n"/>
+      <c r="B120" s="10" t="n"/>
+      <c r="C120" s="10" t="n"/>
+      <c r="D120" s="11" t="n"/>
+      <c r="E120" s="10" t="n"/>
+      <c r="F120" s="10" t="n"/>
+      <c r="G120" s="12">
+        <f>IF(D120="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D120,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H120" s="12">
+        <f>IF(G120="","",IF(LEFT(G120,4)="Wall","Wall",IF(LEFT(G120,7)="Gondola","Gondola",IF(LEFT(G120,6)="Pallet","Pallet",IF(LEFT(G120,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I120" s="12">
+        <f>IF(A120="","",IF(D120="","CEK ID FIXTURE kosong",IF(G120="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H120="Endcap","CEK Endcap tidak ikut sambung",IF(H120&lt;&gt;B120,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C120="","CEK URUTAN kosong",IF(AND(E120&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E120)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="n"/>
+      <c r="B121" s="10" t="n"/>
+      <c r="C121" s="10" t="n"/>
+      <c r="D121" s="11" t="n"/>
+      <c r="E121" s="10" t="n"/>
+      <c r="F121" s="10" t="n"/>
+      <c r="G121" s="12">
+        <f>IF(D121="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D121,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H121" s="12">
+        <f>IF(G121="","",IF(LEFT(G121,4)="Wall","Wall",IF(LEFT(G121,7)="Gondola","Gondola",IF(LEFT(G121,6)="Pallet","Pallet",IF(LEFT(G121,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I121" s="12">
+        <f>IF(A121="","",IF(D121="","CEK ID FIXTURE kosong",IF(G121="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H121="Endcap","CEK Endcap tidak ikut sambung",IF(H121&lt;&gt;B121,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C121="","CEK URUTAN kosong",IF(AND(E121&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E121)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="n"/>
+      <c r="B122" s="10" t="n"/>
+      <c r="C122" s="10" t="n"/>
+      <c r="D122" s="11" t="n"/>
+      <c r="E122" s="10" t="n"/>
+      <c r="F122" s="10" t="n"/>
+      <c r="G122" s="12">
+        <f>IF(D122="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D122,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H122" s="12">
+        <f>IF(G122="","",IF(LEFT(G122,4)="Wall","Wall",IF(LEFT(G122,7)="Gondola","Gondola",IF(LEFT(G122,6)="Pallet","Pallet",IF(LEFT(G122,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I122" s="12">
+        <f>IF(A122="","",IF(D122="","CEK ID FIXTURE kosong",IF(G122="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H122="Endcap","CEK Endcap tidak ikut sambung",IF(H122&lt;&gt;B122,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C122="","CEK URUTAN kosong",IF(AND(E122&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E122)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="n"/>
+      <c r="B123" s="10" t="n"/>
+      <c r="C123" s="10" t="n"/>
+      <c r="D123" s="11" t="n"/>
+      <c r="E123" s="10" t="n"/>
+      <c r="F123" s="10" t="n"/>
+      <c r="G123" s="12">
+        <f>IF(D123="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D123,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H123" s="12">
+        <f>IF(G123="","",IF(LEFT(G123,4)="Wall","Wall",IF(LEFT(G123,7)="Gondola","Gondola",IF(LEFT(G123,6)="Pallet","Pallet",IF(LEFT(G123,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I123" s="12">
+        <f>IF(A123="","",IF(D123="","CEK ID FIXTURE kosong",IF(G123="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H123="Endcap","CEK Endcap tidak ikut sambung",IF(H123&lt;&gt;B123,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C123="","CEK URUTAN kosong",IF(AND(E123&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E123)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="n"/>
+      <c r="B124" s="10" t="n"/>
+      <c r="C124" s="10" t="n"/>
+      <c r="D124" s="11" t="n"/>
+      <c r="E124" s="10" t="n"/>
+      <c r="F124" s="10" t="n"/>
+      <c r="G124" s="12">
+        <f>IF(D124="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D124,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H124" s="12">
+        <f>IF(G124="","",IF(LEFT(G124,4)="Wall","Wall",IF(LEFT(G124,7)="Gondola","Gondola",IF(LEFT(G124,6)="Pallet","Pallet",IF(LEFT(G124,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I124" s="12">
+        <f>IF(A124="","",IF(D124="","CEK ID FIXTURE kosong",IF(G124="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H124="Endcap","CEK Endcap tidak ikut sambung",IF(H124&lt;&gt;B124,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C124="","CEK URUTAN kosong",IF(AND(E124&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E124)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="n"/>
+      <c r="B125" s="10" t="n"/>
+      <c r="C125" s="10" t="n"/>
+      <c r="D125" s="11" t="n"/>
+      <c r="E125" s="10" t="n"/>
+      <c r="F125" s="10" t="n"/>
+      <c r="G125" s="12">
+        <f>IF(D125="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D125,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H125" s="12">
+        <f>IF(G125="","",IF(LEFT(G125,4)="Wall","Wall",IF(LEFT(G125,7)="Gondola","Gondola",IF(LEFT(G125,6)="Pallet","Pallet",IF(LEFT(G125,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I125" s="12">
+        <f>IF(A125="","",IF(D125="","CEK ID FIXTURE kosong",IF(G125="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H125="Endcap","CEK Endcap tidak ikut sambung",IF(H125&lt;&gt;B125,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C125="","CEK URUTAN kosong",IF(AND(E125&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E125)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="n"/>
+      <c r="B126" s="10" t="n"/>
+      <c r="C126" s="10" t="n"/>
+      <c r="D126" s="11" t="n"/>
+      <c r="E126" s="10" t="n"/>
+      <c r="F126" s="10" t="n"/>
+      <c r="G126" s="12">
+        <f>IF(D126="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D126,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H126" s="12">
+        <f>IF(G126="","",IF(LEFT(G126,4)="Wall","Wall",IF(LEFT(G126,7)="Gondola","Gondola",IF(LEFT(G126,6)="Pallet","Pallet",IF(LEFT(G126,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I126" s="12">
+        <f>IF(A126="","",IF(D126="","CEK ID FIXTURE kosong",IF(G126="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H126="Endcap","CEK Endcap tidak ikut sambung",IF(H126&lt;&gt;B126,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C126="","CEK URUTAN kosong",IF(AND(E126&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E126)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="n"/>
+      <c r="B127" s="10" t="n"/>
+      <c r="C127" s="10" t="n"/>
+      <c r="D127" s="11" t="n"/>
+      <c r="E127" s="10" t="n"/>
+      <c r="F127" s="10" t="n"/>
+      <c r="G127" s="12">
+        <f>IF(D127="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D127,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H127" s="12">
+        <f>IF(G127="","",IF(LEFT(G127,4)="Wall","Wall",IF(LEFT(G127,7)="Gondola","Gondola",IF(LEFT(G127,6)="Pallet","Pallet",IF(LEFT(G127,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I127" s="12">
+        <f>IF(A127="","",IF(D127="","CEK ID FIXTURE kosong",IF(G127="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H127="Endcap","CEK Endcap tidak ikut sambung",IF(H127&lt;&gt;B127,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C127="","CEK URUTAN kosong",IF(AND(E127&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E127)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="n"/>
+      <c r="B128" s="10" t="n"/>
+      <c r="C128" s="10" t="n"/>
+      <c r="D128" s="11" t="n"/>
+      <c r="E128" s="10" t="n"/>
+      <c r="F128" s="10" t="n"/>
+      <c r="G128" s="12">
+        <f>IF(D128="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D128,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H128" s="12">
+        <f>IF(G128="","",IF(LEFT(G128,4)="Wall","Wall",IF(LEFT(G128,7)="Gondola","Gondola",IF(LEFT(G128,6)="Pallet","Pallet",IF(LEFT(G128,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I128" s="12">
+        <f>IF(A128="","",IF(D128="","CEK ID FIXTURE kosong",IF(G128="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H128="Endcap","CEK Endcap tidak ikut sambung",IF(H128&lt;&gt;B128,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C128="","CEK URUTAN kosong",IF(AND(E128&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E128)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="n"/>
+      <c r="B129" s="10" t="n"/>
+      <c r="C129" s="10" t="n"/>
+      <c r="D129" s="11" t="n"/>
+      <c r="E129" s="10" t="n"/>
+      <c r="F129" s="10" t="n"/>
+      <c r="G129" s="12">
+        <f>IF(D129="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D129,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H129" s="12">
+        <f>IF(G129="","",IF(LEFT(G129,4)="Wall","Wall",IF(LEFT(G129,7)="Gondola","Gondola",IF(LEFT(G129,6)="Pallet","Pallet",IF(LEFT(G129,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I129" s="12">
+        <f>IF(A129="","",IF(D129="","CEK ID FIXTURE kosong",IF(G129="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H129="Endcap","CEK Endcap tidak ikut sambung",IF(H129&lt;&gt;B129,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C129="","CEK URUTAN kosong",IF(AND(E129&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E129)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="n"/>
+      <c r="B130" s="10" t="n"/>
+      <c r="C130" s="10" t="n"/>
+      <c r="D130" s="11" t="n"/>
+      <c r="E130" s="10" t="n"/>
+      <c r="F130" s="10" t="n"/>
+      <c r="G130" s="12">
+        <f>IF(D130="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D130,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H130" s="12">
+        <f>IF(G130="","",IF(LEFT(G130,4)="Wall","Wall",IF(LEFT(G130,7)="Gondola","Gondola",IF(LEFT(G130,6)="Pallet","Pallet",IF(LEFT(G130,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I130" s="12">
+        <f>IF(A130="","",IF(D130="","CEK ID FIXTURE kosong",IF(G130="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H130="Endcap","CEK Endcap tidak ikut sambung",IF(H130&lt;&gt;B130,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C130="","CEK URUTAN kosong",IF(AND(E130&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E130)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="n"/>
+      <c r="B131" s="10" t="n"/>
+      <c r="C131" s="10" t="n"/>
+      <c r="D131" s="11" t="n"/>
+      <c r="E131" s="10" t="n"/>
+      <c r="F131" s="10" t="n"/>
+      <c r="G131" s="12">
+        <f>IF(D131="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D131,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H131" s="12">
+        <f>IF(G131="","",IF(LEFT(G131,4)="Wall","Wall",IF(LEFT(G131,7)="Gondola","Gondola",IF(LEFT(G131,6)="Pallet","Pallet",IF(LEFT(G131,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I131" s="12">
+        <f>IF(A131="","",IF(D131="","CEK ID FIXTURE kosong",IF(G131="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H131="Endcap","CEK Endcap tidak ikut sambung",IF(H131&lt;&gt;B131,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C131="","CEK URUTAN kosong",IF(AND(E131&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E131)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="n"/>
+      <c r="B132" s="10" t="n"/>
+      <c r="C132" s="10" t="n"/>
+      <c r="D132" s="11" t="n"/>
+      <c r="E132" s="10" t="n"/>
+      <c r="F132" s="10" t="n"/>
+      <c r="G132" s="12">
+        <f>IF(D132="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D132,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H132" s="12">
+        <f>IF(G132="","",IF(LEFT(G132,4)="Wall","Wall",IF(LEFT(G132,7)="Gondola","Gondola",IF(LEFT(G132,6)="Pallet","Pallet",IF(LEFT(G132,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I132" s="12">
+        <f>IF(A132="","",IF(D132="","CEK ID FIXTURE kosong",IF(G132="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H132="Endcap","CEK Endcap tidak ikut sambung",IF(H132&lt;&gt;B132,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C132="","CEK URUTAN kosong",IF(AND(E132&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E132)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="n"/>
+      <c r="B133" s="10" t="n"/>
+      <c r="C133" s="10" t="n"/>
+      <c r="D133" s="11" t="n"/>
+      <c r="E133" s="10" t="n"/>
+      <c r="F133" s="10" t="n"/>
+      <c r="G133" s="12">
+        <f>IF(D133="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D133,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H133" s="12">
+        <f>IF(G133="","",IF(LEFT(G133,4)="Wall","Wall",IF(LEFT(G133,7)="Gondola","Gondola",IF(LEFT(G133,6)="Pallet","Pallet",IF(LEFT(G133,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I133" s="12">
+        <f>IF(A133="","",IF(D133="","CEK ID FIXTURE kosong",IF(G133="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H133="Endcap","CEK Endcap tidak ikut sambung",IF(H133&lt;&gt;B133,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C133="","CEK URUTAN kosong",IF(AND(E133&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E133)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="10" t="n"/>
+      <c r="B134" s="10" t="n"/>
+      <c r="C134" s="10" t="n"/>
+      <c r="D134" s="11" t="n"/>
+      <c r="E134" s="10" t="n"/>
+      <c r="F134" s="10" t="n"/>
+      <c r="G134" s="12">
+        <f>IF(D134="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D134,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H134" s="12">
+        <f>IF(G134="","",IF(LEFT(G134,4)="Wall","Wall",IF(LEFT(G134,7)="Gondola","Gondola",IF(LEFT(G134,6)="Pallet","Pallet",IF(LEFT(G134,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I134" s="12">
+        <f>IF(A134="","",IF(D134="","CEK ID FIXTURE kosong",IF(G134="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H134="Endcap","CEK Endcap tidak ikut sambung",IF(H134&lt;&gt;B134,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C134="","CEK URUTAN kosong",IF(AND(E134&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E134)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="10" t="n"/>
+      <c r="B135" s="10" t="n"/>
+      <c r="C135" s="10" t="n"/>
+      <c r="D135" s="11" t="n"/>
+      <c r="E135" s="10" t="n"/>
+      <c r="F135" s="10" t="n"/>
+      <c r="G135" s="12">
+        <f>IF(D135="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D135,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H135" s="12">
+        <f>IF(G135="","",IF(LEFT(G135,4)="Wall","Wall",IF(LEFT(G135,7)="Gondola","Gondola",IF(LEFT(G135,6)="Pallet","Pallet",IF(LEFT(G135,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I135" s="12">
+        <f>IF(A135="","",IF(D135="","CEK ID FIXTURE kosong",IF(G135="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H135="Endcap","CEK Endcap tidak ikut sambung",IF(H135&lt;&gt;B135,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C135="","CEK URUTAN kosong",IF(AND(E135&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E135)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="10" t="n"/>
+      <c r="B136" s="10" t="n"/>
+      <c r="C136" s="10" t="n"/>
+      <c r="D136" s="11" t="n"/>
+      <c r="E136" s="10" t="n"/>
+      <c r="F136" s="10" t="n"/>
+      <c r="G136" s="12">
+        <f>IF(D136="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D136,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H136" s="12">
+        <f>IF(G136="","",IF(LEFT(G136,4)="Wall","Wall",IF(LEFT(G136,7)="Gondola","Gondola",IF(LEFT(G136,6)="Pallet","Pallet",IF(LEFT(G136,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I136" s="12">
+        <f>IF(A136="","",IF(D136="","CEK ID FIXTURE kosong",IF(G136="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H136="Endcap","CEK Endcap tidak ikut sambung",IF(H136&lt;&gt;B136,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C136="","CEK URUTAN kosong",IF(AND(E136&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E136)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="10" t="n"/>
+      <c r="B137" s="10" t="n"/>
+      <c r="C137" s="10" t="n"/>
+      <c r="D137" s="11" t="n"/>
+      <c r="E137" s="10" t="n"/>
+      <c r="F137" s="10" t="n"/>
+      <c r="G137" s="12">
+        <f>IF(D137="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D137,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H137" s="12">
+        <f>IF(G137="","",IF(LEFT(G137,4)="Wall","Wall",IF(LEFT(G137,7)="Gondola","Gondola",IF(LEFT(G137,6)="Pallet","Pallet",IF(LEFT(G137,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I137" s="12">
+        <f>IF(A137="","",IF(D137="","CEK ID FIXTURE kosong",IF(G137="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H137="Endcap","CEK Endcap tidak ikut sambung",IF(H137&lt;&gt;B137,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C137="","CEK URUTAN kosong",IF(AND(E137&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E137)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="10" t="n"/>
+      <c r="B138" s="10" t="n"/>
+      <c r="C138" s="10" t="n"/>
+      <c r="D138" s="11" t="n"/>
+      <c r="E138" s="10" t="n"/>
+      <c r="F138" s="10" t="n"/>
+      <c r="G138" s="12">
+        <f>IF(D138="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D138,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H138" s="12">
+        <f>IF(G138="","",IF(LEFT(G138,4)="Wall","Wall",IF(LEFT(G138,7)="Gondola","Gondola",IF(LEFT(G138,6)="Pallet","Pallet",IF(LEFT(G138,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I138" s="12">
+        <f>IF(A138="","",IF(D138="","CEK ID FIXTURE kosong",IF(G138="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H138="Endcap","CEK Endcap tidak ikut sambung",IF(H138&lt;&gt;B138,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C138="","CEK URUTAN kosong",IF(AND(E138&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E138)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="10" t="n"/>
+      <c r="B139" s="10" t="n"/>
+      <c r="C139" s="10" t="n"/>
+      <c r="D139" s="11" t="n"/>
+      <c r="E139" s="10" t="n"/>
+      <c r="F139" s="10" t="n"/>
+      <c r="G139" s="12">
+        <f>IF(D139="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D139,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H139" s="12">
+        <f>IF(G139="","",IF(LEFT(G139,4)="Wall","Wall",IF(LEFT(G139,7)="Gondola","Gondola",IF(LEFT(G139,6)="Pallet","Pallet",IF(LEFT(G139,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I139" s="12">
+        <f>IF(A139="","",IF(D139="","CEK ID FIXTURE kosong",IF(G139="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H139="Endcap","CEK Endcap tidak ikut sambung",IF(H139&lt;&gt;B139,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C139="","CEK URUTAN kosong",IF(AND(E139&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E139)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="10" t="n"/>
+      <c r="B140" s="10" t="n"/>
+      <c r="C140" s="10" t="n"/>
+      <c r="D140" s="11" t="n"/>
+      <c r="E140" s="10" t="n"/>
+      <c r="F140" s="10" t="n"/>
+      <c r="G140" s="12">
+        <f>IF(D140="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D140,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H140" s="12">
+        <f>IF(G140="","",IF(LEFT(G140,4)="Wall","Wall",IF(LEFT(G140,7)="Gondola","Gondola",IF(LEFT(G140,6)="Pallet","Pallet",IF(LEFT(G140,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I140" s="12">
+        <f>IF(A140="","",IF(D140="","CEK ID FIXTURE kosong",IF(G140="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H140="Endcap","CEK Endcap tidak ikut sambung",IF(H140&lt;&gt;B140,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C140="","CEK URUTAN kosong",IF(AND(E140&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E140)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="10" t="n"/>
+      <c r="B141" s="10" t="n"/>
+      <c r="C141" s="10" t="n"/>
+      <c r="D141" s="11" t="n"/>
+      <c r="E141" s="10" t="n"/>
+      <c r="F141" s="10" t="n"/>
+      <c r="G141" s="12">
+        <f>IF(D141="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D141,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H141" s="12">
+        <f>IF(G141="","",IF(LEFT(G141,4)="Wall","Wall",IF(LEFT(G141,7)="Gondola","Gondola",IF(LEFT(G141,6)="Pallet","Pallet",IF(LEFT(G141,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I141" s="12">
+        <f>IF(A141="","",IF(D141="","CEK ID FIXTURE kosong",IF(G141="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H141="Endcap","CEK Endcap tidak ikut sambung",IF(H141&lt;&gt;B141,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C141="","CEK URUTAN kosong",IF(AND(E141&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E141)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="10" t="n"/>
+      <c r="B142" s="10" t="n"/>
+      <c r="C142" s="10" t="n"/>
+      <c r="D142" s="11" t="n"/>
+      <c r="E142" s="10" t="n"/>
+      <c r="F142" s="10" t="n"/>
+      <c r="G142" s="12">
+        <f>IF(D142="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D142,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H142" s="12">
+        <f>IF(G142="","",IF(LEFT(G142,4)="Wall","Wall",IF(LEFT(G142,7)="Gondola","Gondola",IF(LEFT(G142,6)="Pallet","Pallet",IF(LEFT(G142,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I142" s="12">
+        <f>IF(A142="","",IF(D142="","CEK ID FIXTURE kosong",IF(G142="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H142="Endcap","CEK Endcap tidak ikut sambung",IF(H142&lt;&gt;B142,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C142="","CEK URUTAN kosong",IF(AND(E142&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E142)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="10" t="n"/>
+      <c r="B143" s="10" t="n"/>
+      <c r="C143" s="10" t="n"/>
+      <c r="D143" s="11" t="n"/>
+      <c r="E143" s="10" t="n"/>
+      <c r="F143" s="10" t="n"/>
+      <c r="G143" s="12">
+        <f>IF(D143="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D143,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H143" s="12">
+        <f>IF(G143="","",IF(LEFT(G143,4)="Wall","Wall",IF(LEFT(G143,7)="Gondola","Gondola",IF(LEFT(G143,6)="Pallet","Pallet",IF(LEFT(G143,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I143" s="12">
+        <f>IF(A143="","",IF(D143="","CEK ID FIXTURE kosong",IF(G143="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H143="Endcap","CEK Endcap tidak ikut sambung",IF(H143&lt;&gt;B143,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C143="","CEK URUTAN kosong",IF(AND(E143&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E143)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="n"/>
+      <c r="B144" s="10" t="n"/>
+      <c r="C144" s="10" t="n"/>
+      <c r="D144" s="11" t="n"/>
+      <c r="E144" s="10" t="n"/>
+      <c r="F144" s="10" t="n"/>
+      <c r="G144" s="12">
+        <f>IF(D144="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D144,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H144" s="12">
+        <f>IF(G144="","",IF(LEFT(G144,4)="Wall","Wall",IF(LEFT(G144,7)="Gondola","Gondola",IF(LEFT(G144,6)="Pallet","Pallet",IF(LEFT(G144,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I144" s="12">
+        <f>IF(A144="","",IF(D144="","CEK ID FIXTURE kosong",IF(G144="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H144="Endcap","CEK Endcap tidak ikut sambung",IF(H144&lt;&gt;B144,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C144="","CEK URUTAN kosong",IF(AND(E144&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E144)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="10" t="n"/>
+      <c r="B145" s="10" t="n"/>
+      <c r="C145" s="10" t="n"/>
+      <c r="D145" s="11" t="n"/>
+      <c r="E145" s="10" t="n"/>
+      <c r="F145" s="10" t="n"/>
+      <c r="G145" s="12">
+        <f>IF(D145="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D145,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H145" s="12">
+        <f>IF(G145="","",IF(LEFT(G145,4)="Wall","Wall",IF(LEFT(G145,7)="Gondola","Gondola",IF(LEFT(G145,6)="Pallet","Pallet",IF(LEFT(G145,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I145" s="12">
+        <f>IF(A145="","",IF(D145="","CEK ID FIXTURE kosong",IF(G145="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H145="Endcap","CEK Endcap tidak ikut sambung",IF(H145&lt;&gt;B145,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C145="","CEK URUTAN kosong",IF(AND(E145&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E145)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="10" t="n"/>
+      <c r="B146" s="10" t="n"/>
+      <c r="C146" s="10" t="n"/>
+      <c r="D146" s="11" t="n"/>
+      <c r="E146" s="10" t="n"/>
+      <c r="F146" s="10" t="n"/>
+      <c r="G146" s="12">
+        <f>IF(D146="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D146,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H146" s="12">
+        <f>IF(G146="","",IF(LEFT(G146,4)="Wall","Wall",IF(LEFT(G146,7)="Gondola","Gondola",IF(LEFT(G146,6)="Pallet","Pallet",IF(LEFT(G146,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I146" s="12">
+        <f>IF(A146="","",IF(D146="","CEK ID FIXTURE kosong",IF(G146="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H146="Endcap","CEK Endcap tidak ikut sambung",IF(H146&lt;&gt;B146,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C146="","CEK URUTAN kosong",IF(AND(E146&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E146)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="10" t="n"/>
+      <c r="B147" s="10" t="n"/>
+      <c r="C147" s="10" t="n"/>
+      <c r="D147" s="11" t="n"/>
+      <c r="E147" s="10" t="n"/>
+      <c r="F147" s="10" t="n"/>
+      <c r="G147" s="12">
+        <f>IF(D147="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D147,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H147" s="12">
+        <f>IF(G147="","",IF(LEFT(G147,4)="Wall","Wall",IF(LEFT(G147,7)="Gondola","Gondola",IF(LEFT(G147,6)="Pallet","Pallet",IF(LEFT(G147,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I147" s="12">
+        <f>IF(A147="","",IF(D147="","CEK ID FIXTURE kosong",IF(G147="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H147="Endcap","CEK Endcap tidak ikut sambung",IF(H147&lt;&gt;B147,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C147="","CEK URUTAN kosong",IF(AND(E147&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E147)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="10" t="n"/>
+      <c r="B148" s="10" t="n"/>
+      <c r="C148" s="10" t="n"/>
+      <c r="D148" s="11" t="n"/>
+      <c r="E148" s="10" t="n"/>
+      <c r="F148" s="10" t="n"/>
+      <c r="G148" s="12">
+        <f>IF(D148="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D148,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H148" s="12">
+        <f>IF(G148="","",IF(LEFT(G148,4)="Wall","Wall",IF(LEFT(G148,7)="Gondola","Gondola",IF(LEFT(G148,6)="Pallet","Pallet",IF(LEFT(G148,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I148" s="12">
+        <f>IF(A148="","",IF(D148="","CEK ID FIXTURE kosong",IF(G148="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H148="Endcap","CEK Endcap tidak ikut sambung",IF(H148&lt;&gt;B148,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C148="","CEK URUTAN kosong",IF(AND(E148&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E148)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="10" t="n"/>
+      <c r="B149" s="10" t="n"/>
+      <c r="C149" s="10" t="n"/>
+      <c r="D149" s="11" t="n"/>
+      <c r="E149" s="10" t="n"/>
+      <c r="F149" s="10" t="n"/>
+      <c r="G149" s="12">
+        <f>IF(D149="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D149,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H149" s="12">
+        <f>IF(G149="","",IF(LEFT(G149,4)="Wall","Wall",IF(LEFT(G149,7)="Gondola","Gondola",IF(LEFT(G149,6)="Pallet","Pallet",IF(LEFT(G149,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I149" s="12">
+        <f>IF(A149="","",IF(D149="","CEK ID FIXTURE kosong",IF(G149="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H149="Endcap","CEK Endcap tidak ikut sambung",IF(H149&lt;&gt;B149,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C149="","CEK URUTAN kosong",IF(AND(E149&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E149)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="10" t="n"/>
+      <c r="B150" s="10" t="n"/>
+      <c r="C150" s="10" t="n"/>
+      <c r="D150" s="11" t="n"/>
+      <c r="E150" s="10" t="n"/>
+      <c r="F150" s="10" t="n"/>
+      <c r="G150" s="12">
+        <f>IF(D150="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D150,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H150" s="12">
+        <f>IF(G150="","",IF(LEFT(G150,4)="Wall","Wall",IF(LEFT(G150,7)="Gondola","Gondola",IF(LEFT(G150,6)="Pallet","Pallet",IF(LEFT(G150,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I150" s="12">
+        <f>IF(A150="","",IF(D150="","CEK ID FIXTURE kosong",IF(G150="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H150="Endcap","CEK Endcap tidak ikut sambung",IF(H150&lt;&gt;B150,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C150="","CEK URUTAN kosong",IF(AND(E150&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E150)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="10" t="n"/>
+      <c r="B151" s="10" t="n"/>
+      <c r="C151" s="10" t="n"/>
+      <c r="D151" s="11" t="n"/>
+      <c r="E151" s="10" t="n"/>
+      <c r="F151" s="10" t="n"/>
+      <c r="G151" s="12">
+        <f>IF(D151="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D151,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H151" s="12">
+        <f>IF(G151="","",IF(LEFT(G151,4)="Wall","Wall",IF(LEFT(G151,7)="Gondola","Gondola",IF(LEFT(G151,6)="Pallet","Pallet",IF(LEFT(G151,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I151" s="12">
+        <f>IF(A151="","",IF(D151="","CEK ID FIXTURE kosong",IF(G151="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H151="Endcap","CEK Endcap tidak ikut sambung",IF(H151&lt;&gt;B151,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C151="","CEK URUTAN kosong",IF(AND(E151&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E151)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="10" t="n"/>
+      <c r="B152" s="10" t="n"/>
+      <c r="C152" s="10" t="n"/>
+      <c r="D152" s="11" t="n"/>
+      <c r="E152" s="10" t="n"/>
+      <c r="F152" s="10" t="n"/>
+      <c r="G152" s="12">
+        <f>IF(D152="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D152,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H152" s="12">
+        <f>IF(G152="","",IF(LEFT(G152,4)="Wall","Wall",IF(LEFT(G152,7)="Gondola","Gondola",IF(LEFT(G152,6)="Pallet","Pallet",IF(LEFT(G152,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I152" s="12">
+        <f>IF(A152="","",IF(D152="","CEK ID FIXTURE kosong",IF(G152="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H152="Endcap","CEK Endcap tidak ikut sambung",IF(H152&lt;&gt;B152,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C152="","CEK URUTAN kosong",IF(AND(E152&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E152)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="10" t="n"/>
+      <c r="B153" s="10" t="n"/>
+      <c r="C153" s="10" t="n"/>
+      <c r="D153" s="11" t="n"/>
+      <c r="E153" s="10" t="n"/>
+      <c r="F153" s="10" t="n"/>
+      <c r="G153" s="12">
+        <f>IF(D153="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D153,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H153" s="12">
+        <f>IF(G153="","",IF(LEFT(G153,4)="Wall","Wall",IF(LEFT(G153,7)="Gondola","Gondola",IF(LEFT(G153,6)="Pallet","Pallet",IF(LEFT(G153,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I153" s="12">
+        <f>IF(A153="","",IF(D153="","CEK ID FIXTURE kosong",IF(G153="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H153="Endcap","CEK Endcap tidak ikut sambung",IF(H153&lt;&gt;B153,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C153="","CEK URUTAN kosong",IF(AND(E153&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E153)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="10" t="n"/>
+      <c r="B154" s="10" t="n"/>
+      <c r="C154" s="10" t="n"/>
+      <c r="D154" s="11" t="n"/>
+      <c r="E154" s="10" t="n"/>
+      <c r="F154" s="10" t="n"/>
+      <c r="G154" s="12">
+        <f>IF(D154="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D154,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H154" s="12">
+        <f>IF(G154="","",IF(LEFT(G154,4)="Wall","Wall",IF(LEFT(G154,7)="Gondola","Gondola",IF(LEFT(G154,6)="Pallet","Pallet",IF(LEFT(G154,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I154" s="12">
+        <f>IF(A154="","",IF(D154="","CEK ID FIXTURE kosong",IF(G154="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H154="Endcap","CEK Endcap tidak ikut sambung",IF(H154&lt;&gt;B154,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C154="","CEK URUTAN kosong",IF(AND(E154&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E154)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="10" t="n"/>
+      <c r="B155" s="10" t="n"/>
+      <c r="C155" s="10" t="n"/>
+      <c r="D155" s="11" t="n"/>
+      <c r="E155" s="10" t="n"/>
+      <c r="F155" s="10" t="n"/>
+      <c r="G155" s="12">
+        <f>IF(D155="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D155,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H155" s="12">
+        <f>IF(G155="","",IF(LEFT(G155,4)="Wall","Wall",IF(LEFT(G155,7)="Gondola","Gondola",IF(LEFT(G155,6)="Pallet","Pallet",IF(LEFT(G155,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I155" s="12">
+        <f>IF(A155="","",IF(D155="","CEK ID FIXTURE kosong",IF(G155="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H155="Endcap","CEK Endcap tidak ikut sambung",IF(H155&lt;&gt;B155,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C155="","CEK URUTAN kosong",IF(AND(E155&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E155)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="10" t="n"/>
+      <c r="B156" s="10" t="n"/>
+      <c r="C156" s="10" t="n"/>
+      <c r="D156" s="11" t="n"/>
+      <c r="E156" s="10" t="n"/>
+      <c r="F156" s="10" t="n"/>
+      <c r="G156" s="12">
+        <f>IF(D156="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D156,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H156" s="12">
+        <f>IF(G156="","",IF(LEFT(G156,4)="Wall","Wall",IF(LEFT(G156,7)="Gondola","Gondola",IF(LEFT(G156,6)="Pallet","Pallet",IF(LEFT(G156,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I156" s="12">
+        <f>IF(A156="","",IF(D156="","CEK ID FIXTURE kosong",IF(G156="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H156="Endcap","CEK Endcap tidak ikut sambung",IF(H156&lt;&gt;B156,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C156="","CEK URUTAN kosong",IF(AND(E156&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E156)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="10" t="n"/>
+      <c r="B157" s="10" t="n"/>
+      <c r="C157" s="10" t="n"/>
+      <c r="D157" s="11" t="n"/>
+      <c r="E157" s="10" t="n"/>
+      <c r="F157" s="10" t="n"/>
+      <c r="G157" s="12">
+        <f>IF(D157="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D157,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H157" s="12">
+        <f>IF(G157="","",IF(LEFT(G157,4)="Wall","Wall",IF(LEFT(G157,7)="Gondola","Gondola",IF(LEFT(G157,6)="Pallet","Pallet",IF(LEFT(G157,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I157" s="12">
+        <f>IF(A157="","",IF(D157="","CEK ID FIXTURE kosong",IF(G157="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H157="Endcap","CEK Endcap tidak ikut sambung",IF(H157&lt;&gt;B157,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C157="","CEK URUTAN kosong",IF(AND(E157&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E157)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="10" t="n"/>
+      <c r="B158" s="10" t="n"/>
+      <c r="C158" s="10" t="n"/>
+      <c r="D158" s="11" t="n"/>
+      <c r="E158" s="10" t="n"/>
+      <c r="F158" s="10" t="n"/>
+      <c r="G158" s="12">
+        <f>IF(D158="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D158,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H158" s="12">
+        <f>IF(G158="","",IF(LEFT(G158,4)="Wall","Wall",IF(LEFT(G158,7)="Gondola","Gondola",IF(LEFT(G158,6)="Pallet","Pallet",IF(LEFT(G158,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I158" s="12">
+        <f>IF(A158="","",IF(D158="","CEK ID FIXTURE kosong",IF(G158="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H158="Endcap","CEK Endcap tidak ikut sambung",IF(H158&lt;&gt;B158,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C158="","CEK URUTAN kosong",IF(AND(E158&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E158)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="10" t="n"/>
+      <c r="B159" s="10" t="n"/>
+      <c r="C159" s="10" t="n"/>
+      <c r="D159" s="11" t="n"/>
+      <c r="E159" s="10" t="n"/>
+      <c r="F159" s="10" t="n"/>
+      <c r="G159" s="12">
+        <f>IF(D159="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D159,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H159" s="12">
+        <f>IF(G159="","",IF(LEFT(G159,4)="Wall","Wall",IF(LEFT(G159,7)="Gondola","Gondola",IF(LEFT(G159,6)="Pallet","Pallet",IF(LEFT(G159,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I159" s="12">
+        <f>IF(A159="","",IF(D159="","CEK ID FIXTURE kosong",IF(G159="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H159="Endcap","CEK Endcap tidak ikut sambung",IF(H159&lt;&gt;B159,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C159="","CEK URUTAN kosong",IF(AND(E159&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E159)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="10" t="n"/>
+      <c r="B160" s="10" t="n"/>
+      <c r="C160" s="10" t="n"/>
+      <c r="D160" s="11" t="n"/>
+      <c r="E160" s="10" t="n"/>
+      <c r="F160" s="10" t="n"/>
+      <c r="G160" s="12">
+        <f>IF(D160="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D160,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H160" s="12">
+        <f>IF(G160="","",IF(LEFT(G160,4)="Wall","Wall",IF(LEFT(G160,7)="Gondola","Gondola",IF(LEFT(G160,6)="Pallet","Pallet",IF(LEFT(G160,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I160" s="12">
+        <f>IF(A160="","",IF(D160="","CEK ID FIXTURE kosong",IF(G160="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H160="Endcap","CEK Endcap tidak ikut sambung",IF(H160&lt;&gt;B160,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C160="","CEK URUTAN kosong",IF(AND(E160&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E160)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="10" t="n"/>
+      <c r="B161" s="10" t="n"/>
+      <c r="C161" s="10" t="n"/>
+      <c r="D161" s="11" t="n"/>
+      <c r="E161" s="10" t="n"/>
+      <c r="F161" s="10" t="n"/>
+      <c r="G161" s="12">
+        <f>IF(D161="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D161,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H161" s="12">
+        <f>IF(G161="","",IF(LEFT(G161,4)="Wall","Wall",IF(LEFT(G161,7)="Gondola","Gondola",IF(LEFT(G161,6)="Pallet","Pallet",IF(LEFT(G161,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I161" s="12">
+        <f>IF(A161="","",IF(D161="","CEK ID FIXTURE kosong",IF(G161="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H161="Endcap","CEK Endcap tidak ikut sambung",IF(H161&lt;&gt;B161,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C161="","CEK URUTAN kosong",IF(AND(E161&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E161)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="10" t="n"/>
+      <c r="B162" s="10" t="n"/>
+      <c r="C162" s="10" t="n"/>
+      <c r="D162" s="11" t="n"/>
+      <c r="E162" s="10" t="n"/>
+      <c r="F162" s="10" t="n"/>
+      <c r="G162" s="12">
+        <f>IF(D162="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D162,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H162" s="12">
+        <f>IF(G162="","",IF(LEFT(G162,4)="Wall","Wall",IF(LEFT(G162,7)="Gondola","Gondola",IF(LEFT(G162,6)="Pallet","Pallet",IF(LEFT(G162,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I162" s="12">
+        <f>IF(A162="","",IF(D162="","CEK ID FIXTURE kosong",IF(G162="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H162="Endcap","CEK Endcap tidak ikut sambung",IF(H162&lt;&gt;B162,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C162="","CEK URUTAN kosong",IF(AND(E162&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E162)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="10" t="n"/>
+      <c r="B163" s="10" t="n"/>
+      <c r="C163" s="10" t="n"/>
+      <c r="D163" s="11" t="n"/>
+      <c r="E163" s="10" t="n"/>
+      <c r="F163" s="10" t="n"/>
+      <c r="G163" s="12">
+        <f>IF(D163="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D163,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H163" s="12">
+        <f>IF(G163="","",IF(LEFT(G163,4)="Wall","Wall",IF(LEFT(G163,7)="Gondola","Gondola",IF(LEFT(G163,6)="Pallet","Pallet",IF(LEFT(G163,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I163" s="12">
+        <f>IF(A163="","",IF(D163="","CEK ID FIXTURE kosong",IF(G163="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H163="Endcap","CEK Endcap tidak ikut sambung",IF(H163&lt;&gt;B163,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C163="","CEK URUTAN kosong",IF(AND(E163&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E163)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="10" t="n"/>
+      <c r="B164" s="10" t="n"/>
+      <c r="C164" s="10" t="n"/>
+      <c r="D164" s="11" t="n"/>
+      <c r="E164" s="10" t="n"/>
+      <c r="F164" s="10" t="n"/>
+      <c r="G164" s="12">
+        <f>IF(D164="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D164,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H164" s="12">
+        <f>IF(G164="","",IF(LEFT(G164,4)="Wall","Wall",IF(LEFT(G164,7)="Gondola","Gondola",IF(LEFT(G164,6)="Pallet","Pallet",IF(LEFT(G164,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I164" s="12">
+        <f>IF(A164="","",IF(D164="","CEK ID FIXTURE kosong",IF(G164="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H164="Endcap","CEK Endcap tidak ikut sambung",IF(H164&lt;&gt;B164,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C164="","CEK URUTAN kosong",IF(AND(E164&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E164)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="10" t="n"/>
+      <c r="B165" s="10" t="n"/>
+      <c r="C165" s="10" t="n"/>
+      <c r="D165" s="11" t="n"/>
+      <c r="E165" s="10" t="n"/>
+      <c r="F165" s="10" t="n"/>
+      <c r="G165" s="12">
+        <f>IF(D165="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D165,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H165" s="12">
+        <f>IF(G165="","",IF(LEFT(G165,4)="Wall","Wall",IF(LEFT(G165,7)="Gondola","Gondola",IF(LEFT(G165,6)="Pallet","Pallet",IF(LEFT(G165,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I165" s="12">
+        <f>IF(A165="","",IF(D165="","CEK ID FIXTURE kosong",IF(G165="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H165="Endcap","CEK Endcap tidak ikut sambung",IF(H165&lt;&gt;B165,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C165="","CEK URUTAN kosong",IF(AND(E165&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E165)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="10" t="n"/>
+      <c r="B166" s="10" t="n"/>
+      <c r="C166" s="10" t="n"/>
+      <c r="D166" s="11" t="n"/>
+      <c r="E166" s="10" t="n"/>
+      <c r="F166" s="10" t="n"/>
+      <c r="G166" s="12">
+        <f>IF(D166="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D166,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H166" s="12">
+        <f>IF(G166="","",IF(LEFT(G166,4)="Wall","Wall",IF(LEFT(G166,7)="Gondola","Gondola",IF(LEFT(G166,6)="Pallet","Pallet",IF(LEFT(G166,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I166" s="12">
+        <f>IF(A166="","",IF(D166="","CEK ID FIXTURE kosong",IF(G166="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H166="Endcap","CEK Endcap tidak ikut sambung",IF(H166&lt;&gt;B166,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C166="","CEK URUTAN kosong",IF(AND(E166&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E166)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="10" t="n"/>
+      <c r="B167" s="10" t="n"/>
+      <c r="C167" s="10" t="n"/>
+      <c r="D167" s="11" t="n"/>
+      <c r="E167" s="10" t="n"/>
+      <c r="F167" s="10" t="n"/>
+      <c r="G167" s="12">
+        <f>IF(D167="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D167,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H167" s="12">
+        <f>IF(G167="","",IF(LEFT(G167,4)="Wall","Wall",IF(LEFT(G167,7)="Gondola","Gondola",IF(LEFT(G167,6)="Pallet","Pallet",IF(LEFT(G167,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I167" s="12">
+        <f>IF(A167="","",IF(D167="","CEK ID FIXTURE kosong",IF(G167="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H167="Endcap","CEK Endcap tidak ikut sambung",IF(H167&lt;&gt;B167,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C167="","CEK URUTAN kosong",IF(AND(E167&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E167)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="10" t="n"/>
+      <c r="B168" s="10" t="n"/>
+      <c r="C168" s="10" t="n"/>
+      <c r="D168" s="11" t="n"/>
+      <c r="E168" s="10" t="n"/>
+      <c r="F168" s="10" t="n"/>
+      <c r="G168" s="12">
+        <f>IF(D168="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D168,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H168" s="12">
+        <f>IF(G168="","",IF(LEFT(G168,4)="Wall","Wall",IF(LEFT(G168,7)="Gondola","Gondola",IF(LEFT(G168,6)="Pallet","Pallet",IF(LEFT(G168,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I168" s="12">
+        <f>IF(A168="","",IF(D168="","CEK ID FIXTURE kosong",IF(G168="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H168="Endcap","CEK Endcap tidak ikut sambung",IF(H168&lt;&gt;B168,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C168="","CEK URUTAN kosong",IF(AND(E168&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E168)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="10" t="n"/>
+      <c r="B169" s="10" t="n"/>
+      <c r="C169" s="10" t="n"/>
+      <c r="D169" s="11" t="n"/>
+      <c r="E169" s="10" t="n"/>
+      <c r="F169" s="10" t="n"/>
+      <c r="G169" s="12">
+        <f>IF(D169="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D169,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H169" s="12">
+        <f>IF(G169="","",IF(LEFT(G169,4)="Wall","Wall",IF(LEFT(G169,7)="Gondola","Gondola",IF(LEFT(G169,6)="Pallet","Pallet",IF(LEFT(G169,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I169" s="12">
+        <f>IF(A169="","",IF(D169="","CEK ID FIXTURE kosong",IF(G169="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H169="Endcap","CEK Endcap tidak ikut sambung",IF(H169&lt;&gt;B169,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C169="","CEK URUTAN kosong",IF(AND(E169&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E169)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="10" t="n"/>
+      <c r="B170" s="10" t="n"/>
+      <c r="C170" s="10" t="n"/>
+      <c r="D170" s="11" t="n"/>
+      <c r="E170" s="10" t="n"/>
+      <c r="F170" s="10" t="n"/>
+      <c r="G170" s="12">
+        <f>IF(D170="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D170,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H170" s="12">
+        <f>IF(G170="","",IF(LEFT(G170,4)="Wall","Wall",IF(LEFT(G170,7)="Gondola","Gondola",IF(LEFT(G170,6)="Pallet","Pallet",IF(LEFT(G170,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I170" s="12">
+        <f>IF(A170="","",IF(D170="","CEK ID FIXTURE kosong",IF(G170="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H170="Endcap","CEK Endcap tidak ikut sambung",IF(H170&lt;&gt;B170,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C170="","CEK URUTAN kosong",IF(AND(E170&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E170)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="10" t="n"/>
+      <c r="B171" s="10" t="n"/>
+      <c r="C171" s="10" t="n"/>
+      <c r="D171" s="11" t="n"/>
+      <c r="E171" s="10" t="n"/>
+      <c r="F171" s="10" t="n"/>
+      <c r="G171" s="12">
+        <f>IF(D171="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D171,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H171" s="12">
+        <f>IF(G171="","",IF(LEFT(G171,4)="Wall","Wall",IF(LEFT(G171,7)="Gondola","Gondola",IF(LEFT(G171,6)="Pallet","Pallet",IF(LEFT(G171,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I171" s="12">
+        <f>IF(A171="","",IF(D171="","CEK ID FIXTURE kosong",IF(G171="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H171="Endcap","CEK Endcap tidak ikut sambung",IF(H171&lt;&gt;B171,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C171="","CEK URUTAN kosong",IF(AND(E171&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E171)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="10" t="n"/>
+      <c r="B172" s="10" t="n"/>
+      <c r="C172" s="10" t="n"/>
+      <c r="D172" s="11" t="n"/>
+      <c r="E172" s="10" t="n"/>
+      <c r="F172" s="10" t="n"/>
+      <c r="G172" s="12">
+        <f>IF(D172="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D172,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H172" s="12">
+        <f>IF(G172="","",IF(LEFT(G172,4)="Wall","Wall",IF(LEFT(G172,7)="Gondola","Gondola",IF(LEFT(G172,6)="Pallet","Pallet",IF(LEFT(G172,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I172" s="12">
+        <f>IF(A172="","",IF(D172="","CEK ID FIXTURE kosong",IF(G172="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H172="Endcap","CEK Endcap tidak ikut sambung",IF(H172&lt;&gt;B172,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C172="","CEK URUTAN kosong",IF(AND(E172&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E172)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="10" t="n"/>
+      <c r="B173" s="10" t="n"/>
+      <c r="C173" s="10" t="n"/>
+      <c r="D173" s="11" t="n"/>
+      <c r="E173" s="10" t="n"/>
+      <c r="F173" s="10" t="n"/>
+      <c r="G173" s="12">
+        <f>IF(D173="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D173,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H173" s="12">
+        <f>IF(G173="","",IF(LEFT(G173,4)="Wall","Wall",IF(LEFT(G173,7)="Gondola","Gondola",IF(LEFT(G173,6)="Pallet","Pallet",IF(LEFT(G173,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I173" s="12">
+        <f>IF(A173="","",IF(D173="","CEK ID FIXTURE kosong",IF(G173="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H173="Endcap","CEK Endcap tidak ikut sambung",IF(H173&lt;&gt;B173,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C173="","CEK URUTAN kosong",IF(AND(E173&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E173)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="10" t="n"/>
+      <c r="B174" s="10" t="n"/>
+      <c r="C174" s="10" t="n"/>
+      <c r="D174" s="11" t="n"/>
+      <c r="E174" s="10" t="n"/>
+      <c r="F174" s="10" t="n"/>
+      <c r="G174" s="12">
+        <f>IF(D174="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D174,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H174" s="12">
+        <f>IF(G174="","",IF(LEFT(G174,4)="Wall","Wall",IF(LEFT(G174,7)="Gondola","Gondola",IF(LEFT(G174,6)="Pallet","Pallet",IF(LEFT(G174,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I174" s="12">
+        <f>IF(A174="","",IF(D174="","CEK ID FIXTURE kosong",IF(G174="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H174="Endcap","CEK Endcap tidak ikut sambung",IF(H174&lt;&gt;B174,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C174="","CEK URUTAN kosong",IF(AND(E174&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E174)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="10" t="n"/>
+      <c r="B175" s="10" t="n"/>
+      <c r="C175" s="10" t="n"/>
+      <c r="D175" s="11" t="n"/>
+      <c r="E175" s="10" t="n"/>
+      <c r="F175" s="10" t="n"/>
+      <c r="G175" s="12">
+        <f>IF(D175="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D175,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H175" s="12">
+        <f>IF(G175="","",IF(LEFT(G175,4)="Wall","Wall",IF(LEFT(G175,7)="Gondola","Gondola",IF(LEFT(G175,6)="Pallet","Pallet",IF(LEFT(G175,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I175" s="12">
+        <f>IF(A175="","",IF(D175="","CEK ID FIXTURE kosong",IF(G175="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H175="Endcap","CEK Endcap tidak ikut sambung",IF(H175&lt;&gt;B175,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C175="","CEK URUTAN kosong",IF(AND(E175&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E175)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="10" t="n"/>
+      <c r="B176" s="10" t="n"/>
+      <c r="C176" s="10" t="n"/>
+      <c r="D176" s="11" t="n"/>
+      <c r="E176" s="10" t="n"/>
+      <c r="F176" s="10" t="n"/>
+      <c r="G176" s="12">
+        <f>IF(D176="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D176,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H176" s="12">
+        <f>IF(G176="","",IF(LEFT(G176,4)="Wall","Wall",IF(LEFT(G176,7)="Gondola","Gondola",IF(LEFT(G176,6)="Pallet","Pallet",IF(LEFT(G176,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I176" s="12">
+        <f>IF(A176="","",IF(D176="","CEK ID FIXTURE kosong",IF(G176="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H176="Endcap","CEK Endcap tidak ikut sambung",IF(H176&lt;&gt;B176,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C176="","CEK URUTAN kosong",IF(AND(E176&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E176)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="10" t="n"/>
+      <c r="B177" s="10" t="n"/>
+      <c r="C177" s="10" t="n"/>
+      <c r="D177" s="11" t="n"/>
+      <c r="E177" s="10" t="n"/>
+      <c r="F177" s="10" t="n"/>
+      <c r="G177" s="12">
+        <f>IF(D177="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D177,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H177" s="12">
+        <f>IF(G177="","",IF(LEFT(G177,4)="Wall","Wall",IF(LEFT(G177,7)="Gondola","Gondola",IF(LEFT(G177,6)="Pallet","Pallet",IF(LEFT(G177,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I177" s="12">
+        <f>IF(A177="","",IF(D177="","CEK ID FIXTURE kosong",IF(G177="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H177="Endcap","CEK Endcap tidak ikut sambung",IF(H177&lt;&gt;B177,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C177="","CEK URUTAN kosong",IF(AND(E177&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E177)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="10" t="n"/>
+      <c r="B178" s="10" t="n"/>
+      <c r="C178" s="10" t="n"/>
+      <c r="D178" s="11" t="n"/>
+      <c r="E178" s="10" t="n"/>
+      <c r="F178" s="10" t="n"/>
+      <c r="G178" s="12">
+        <f>IF(D178="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D178,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H178" s="12">
+        <f>IF(G178="","",IF(LEFT(G178,4)="Wall","Wall",IF(LEFT(G178,7)="Gondola","Gondola",IF(LEFT(G178,6)="Pallet","Pallet",IF(LEFT(G178,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I178" s="12">
+        <f>IF(A178="","",IF(D178="","CEK ID FIXTURE kosong",IF(G178="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H178="Endcap","CEK Endcap tidak ikut sambung",IF(H178&lt;&gt;B178,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C178="","CEK URUTAN kosong",IF(AND(E178&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E178)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="10" t="n"/>
+      <c r="B179" s="10" t="n"/>
+      <c r="C179" s="10" t="n"/>
+      <c r="D179" s="11" t="n"/>
+      <c r="E179" s="10" t="n"/>
+      <c r="F179" s="10" t="n"/>
+      <c r="G179" s="12">
+        <f>IF(D179="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D179,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H179" s="12">
+        <f>IF(G179="","",IF(LEFT(G179,4)="Wall","Wall",IF(LEFT(G179,7)="Gondola","Gondola",IF(LEFT(G179,6)="Pallet","Pallet",IF(LEFT(G179,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I179" s="12">
+        <f>IF(A179="","",IF(D179="","CEK ID FIXTURE kosong",IF(G179="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H179="Endcap","CEK Endcap tidak ikut sambung",IF(H179&lt;&gt;B179,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C179="","CEK URUTAN kosong",IF(AND(E179&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E179)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="10" t="n"/>
+      <c r="B180" s="10" t="n"/>
+      <c r="C180" s="10" t="n"/>
+      <c r="D180" s="11" t="n"/>
+      <c r="E180" s="10" t="n"/>
+      <c r="F180" s="10" t="n"/>
+      <c r="G180" s="12">
+        <f>IF(D180="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D180,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H180" s="12">
+        <f>IF(G180="","",IF(LEFT(G180,4)="Wall","Wall",IF(LEFT(G180,7)="Gondola","Gondola",IF(LEFT(G180,6)="Pallet","Pallet",IF(LEFT(G180,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I180" s="12">
+        <f>IF(A180="","",IF(D180="","CEK ID FIXTURE kosong",IF(G180="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H180="Endcap","CEK Endcap tidak ikut sambung",IF(H180&lt;&gt;B180,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C180="","CEK URUTAN kosong",IF(AND(E180&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E180)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="10" t="n"/>
+      <c r="B181" s="10" t="n"/>
+      <c r="C181" s="10" t="n"/>
+      <c r="D181" s="11" t="n"/>
+      <c r="E181" s="10" t="n"/>
+      <c r="F181" s="10" t="n"/>
+      <c r="G181" s="12">
+        <f>IF(D181="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D181,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H181" s="12">
+        <f>IF(G181="","",IF(LEFT(G181,4)="Wall","Wall",IF(LEFT(G181,7)="Gondola","Gondola",IF(LEFT(G181,6)="Pallet","Pallet",IF(LEFT(G181,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I181" s="12">
+        <f>IF(A181="","",IF(D181="","CEK ID FIXTURE kosong",IF(G181="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H181="Endcap","CEK Endcap tidak ikut sambung",IF(H181&lt;&gt;B181,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C181="","CEK URUTAN kosong",IF(AND(E181&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E181)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="10" t="n"/>
+      <c r="B182" s="10" t="n"/>
+      <c r="C182" s="10" t="n"/>
+      <c r="D182" s="11" t="n"/>
+      <c r="E182" s="10" t="n"/>
+      <c r="F182" s="10" t="n"/>
+      <c r="G182" s="12">
+        <f>IF(D182="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D182,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H182" s="12">
+        <f>IF(G182="","",IF(LEFT(G182,4)="Wall","Wall",IF(LEFT(G182,7)="Gondola","Gondola",IF(LEFT(G182,6)="Pallet","Pallet",IF(LEFT(G182,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I182" s="12">
+        <f>IF(A182="","",IF(D182="","CEK ID FIXTURE kosong",IF(G182="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H182="Endcap","CEK Endcap tidak ikut sambung",IF(H182&lt;&gt;B182,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C182="","CEK URUTAN kosong",IF(AND(E182&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E182)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="10" t="n"/>
+      <c r="B183" s="10" t="n"/>
+      <c r="C183" s="10" t="n"/>
+      <c r="D183" s="11" t="n"/>
+      <c r="E183" s="10" t="n"/>
+      <c r="F183" s="10" t="n"/>
+      <c r="G183" s="12">
+        <f>IF(D183="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D183,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H183" s="12">
+        <f>IF(G183="","",IF(LEFT(G183,4)="Wall","Wall",IF(LEFT(G183,7)="Gondola","Gondola",IF(LEFT(G183,6)="Pallet","Pallet",IF(LEFT(G183,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I183" s="12">
+        <f>IF(A183="","",IF(D183="","CEK ID FIXTURE kosong",IF(G183="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H183="Endcap","CEK Endcap tidak ikut sambung",IF(H183&lt;&gt;B183,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C183="","CEK URUTAN kosong",IF(AND(E183&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E183)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="10" t="n"/>
+      <c r="B184" s="10" t="n"/>
+      <c r="C184" s="10" t="n"/>
+      <c r="D184" s="11" t="n"/>
+      <c r="E184" s="10" t="n"/>
+      <c r="F184" s="10" t="n"/>
+      <c r="G184" s="12">
+        <f>IF(D184="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D184,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H184" s="12">
+        <f>IF(G184="","",IF(LEFT(G184,4)="Wall","Wall",IF(LEFT(G184,7)="Gondola","Gondola",IF(LEFT(G184,6)="Pallet","Pallet",IF(LEFT(G184,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I184" s="12">
+        <f>IF(A184="","",IF(D184="","CEK ID FIXTURE kosong",IF(G184="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H184="Endcap","CEK Endcap tidak ikut sambung",IF(H184&lt;&gt;B184,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C184="","CEK URUTAN kosong",IF(AND(E184&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E184)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="10" t="n"/>
+      <c r="B185" s="10" t="n"/>
+      <c r="C185" s="10" t="n"/>
+      <c r="D185" s="11" t="n"/>
+      <c r="E185" s="10" t="n"/>
+      <c r="F185" s="10" t="n"/>
+      <c r="G185" s="12">
+        <f>IF(D185="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D185,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H185" s="12">
+        <f>IF(G185="","",IF(LEFT(G185,4)="Wall","Wall",IF(LEFT(G185,7)="Gondola","Gondola",IF(LEFT(G185,6)="Pallet","Pallet",IF(LEFT(G185,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I185" s="12">
+        <f>IF(A185="","",IF(D185="","CEK ID FIXTURE kosong",IF(G185="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H185="Endcap","CEK Endcap tidak ikut sambung",IF(H185&lt;&gt;B185,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C185="","CEK URUTAN kosong",IF(AND(E185&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E185)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="10" t="n"/>
+      <c r="B186" s="10" t="n"/>
+      <c r="C186" s="10" t="n"/>
+      <c r="D186" s="11" t="n"/>
+      <c r="E186" s="10" t="n"/>
+      <c r="F186" s="10" t="n"/>
+      <c r="G186" s="12">
+        <f>IF(D186="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D186,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H186" s="12">
+        <f>IF(G186="","",IF(LEFT(G186,4)="Wall","Wall",IF(LEFT(G186,7)="Gondola","Gondola",IF(LEFT(G186,6)="Pallet","Pallet",IF(LEFT(G186,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I186" s="12">
+        <f>IF(A186="","",IF(D186="","CEK ID FIXTURE kosong",IF(G186="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H186="Endcap","CEK Endcap tidak ikut sambung",IF(H186&lt;&gt;B186,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C186="","CEK URUTAN kosong",IF(AND(E186&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E186)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="10" t="n"/>
+      <c r="B187" s="10" t="n"/>
+      <c r="C187" s="10" t="n"/>
+      <c r="D187" s="11" t="n"/>
+      <c r="E187" s="10" t="n"/>
+      <c r="F187" s="10" t="n"/>
+      <c r="G187" s="12">
+        <f>IF(D187="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D187,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H187" s="12">
+        <f>IF(G187="","",IF(LEFT(G187,4)="Wall","Wall",IF(LEFT(G187,7)="Gondola","Gondola",IF(LEFT(G187,6)="Pallet","Pallet",IF(LEFT(G187,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I187" s="12">
+        <f>IF(A187="","",IF(D187="","CEK ID FIXTURE kosong",IF(G187="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H187="Endcap","CEK Endcap tidak ikut sambung",IF(H187&lt;&gt;B187,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C187="","CEK URUTAN kosong",IF(AND(E187&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E187)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="10" t="n"/>
+      <c r="B188" s="10" t="n"/>
+      <c r="C188" s="10" t="n"/>
+      <c r="D188" s="11" t="n"/>
+      <c r="E188" s="10" t="n"/>
+      <c r="F188" s="10" t="n"/>
+      <c r="G188" s="12">
+        <f>IF(D188="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D188,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H188" s="12">
+        <f>IF(G188="","",IF(LEFT(G188,4)="Wall","Wall",IF(LEFT(G188,7)="Gondola","Gondola",IF(LEFT(G188,6)="Pallet","Pallet",IF(LEFT(G188,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I188" s="12">
+        <f>IF(A188="","",IF(D188="","CEK ID FIXTURE kosong",IF(G188="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H188="Endcap","CEK Endcap tidak ikut sambung",IF(H188&lt;&gt;B188,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C188="","CEK URUTAN kosong",IF(AND(E188&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E188)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="10" t="n"/>
+      <c r="B189" s="10" t="n"/>
+      <c r="C189" s="10" t="n"/>
+      <c r="D189" s="11" t="n"/>
+      <c r="E189" s="10" t="n"/>
+      <c r="F189" s="10" t="n"/>
+      <c r="G189" s="12">
+        <f>IF(D189="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D189,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H189" s="12">
+        <f>IF(G189="","",IF(LEFT(G189,4)="Wall","Wall",IF(LEFT(G189,7)="Gondola","Gondola",IF(LEFT(G189,6)="Pallet","Pallet",IF(LEFT(G189,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I189" s="12">
+        <f>IF(A189="","",IF(D189="","CEK ID FIXTURE kosong",IF(G189="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H189="Endcap","CEK Endcap tidak ikut sambung",IF(H189&lt;&gt;B189,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C189="","CEK URUTAN kosong",IF(AND(E189&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E189)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="10" t="n"/>
+      <c r="B190" s="10" t="n"/>
+      <c r="C190" s="10" t="n"/>
+      <c r="D190" s="11" t="n"/>
+      <c r="E190" s="10" t="n"/>
+      <c r="F190" s="10" t="n"/>
+      <c r="G190" s="12">
+        <f>IF(D190="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D190,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H190" s="12">
+        <f>IF(G190="","",IF(LEFT(G190,4)="Wall","Wall",IF(LEFT(G190,7)="Gondola","Gondola",IF(LEFT(G190,6)="Pallet","Pallet",IF(LEFT(G190,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I190" s="12">
+        <f>IF(A190="","",IF(D190="","CEK ID FIXTURE kosong",IF(G190="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H190="Endcap","CEK Endcap tidak ikut sambung",IF(H190&lt;&gt;B190,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C190="","CEK URUTAN kosong",IF(AND(E190&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E190)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="10" t="n"/>
+      <c r="B191" s="10" t="n"/>
+      <c r="C191" s="10" t="n"/>
+      <c r="D191" s="11" t="n"/>
+      <c r="E191" s="10" t="n"/>
+      <c r="F191" s="10" t="n"/>
+      <c r="G191" s="12">
+        <f>IF(D191="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D191,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H191" s="12">
+        <f>IF(G191="","",IF(LEFT(G191,4)="Wall","Wall",IF(LEFT(G191,7)="Gondola","Gondola",IF(LEFT(G191,6)="Pallet","Pallet",IF(LEFT(G191,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I191" s="12">
+        <f>IF(A191="","",IF(D191="","CEK ID FIXTURE kosong",IF(G191="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H191="Endcap","CEK Endcap tidak ikut sambung",IF(H191&lt;&gt;B191,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C191="","CEK URUTAN kosong",IF(AND(E191&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E191)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="10" t="n"/>
+      <c r="B192" s="10" t="n"/>
+      <c r="C192" s="10" t="n"/>
+      <c r="D192" s="11" t="n"/>
+      <c r="E192" s="10" t="n"/>
+      <c r="F192" s="10" t="n"/>
+      <c r="G192" s="12">
+        <f>IF(D192="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D192,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H192" s="12">
+        <f>IF(G192="","",IF(LEFT(G192,4)="Wall","Wall",IF(LEFT(G192,7)="Gondola","Gondola",IF(LEFT(G192,6)="Pallet","Pallet",IF(LEFT(G192,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I192" s="12">
+        <f>IF(A192="","",IF(D192="","CEK ID FIXTURE kosong",IF(G192="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H192="Endcap","CEK Endcap tidak ikut sambung",IF(H192&lt;&gt;B192,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C192="","CEK URUTAN kosong",IF(AND(E192&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E192)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="10" t="n"/>
+      <c r="B193" s="10" t="n"/>
+      <c r="C193" s="10" t="n"/>
+      <c r="D193" s="11" t="n"/>
+      <c r="E193" s="10" t="n"/>
+      <c r="F193" s="10" t="n"/>
+      <c r="G193" s="12">
+        <f>IF(D193="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D193,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H193" s="12">
+        <f>IF(G193="","",IF(LEFT(G193,4)="Wall","Wall",IF(LEFT(G193,7)="Gondola","Gondola",IF(LEFT(G193,6)="Pallet","Pallet",IF(LEFT(G193,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I193" s="12">
+        <f>IF(A193="","",IF(D193="","CEK ID FIXTURE kosong",IF(G193="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H193="Endcap","CEK Endcap tidak ikut sambung",IF(H193&lt;&gt;B193,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C193="","CEK URUTAN kosong",IF(AND(E193&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E193)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="10" t="n"/>
+      <c r="B194" s="10" t="n"/>
+      <c r="C194" s="10" t="n"/>
+      <c r="D194" s="11" t="n"/>
+      <c r="E194" s="10" t="n"/>
+      <c r="F194" s="10" t="n"/>
+      <c r="G194" s="12">
+        <f>IF(D194="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D194,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H194" s="12">
+        <f>IF(G194="","",IF(LEFT(G194,4)="Wall","Wall",IF(LEFT(G194,7)="Gondola","Gondola",IF(LEFT(G194,6)="Pallet","Pallet",IF(LEFT(G194,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I194" s="12">
+        <f>IF(A194="","",IF(D194="","CEK ID FIXTURE kosong",IF(G194="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H194="Endcap","CEK Endcap tidak ikut sambung",IF(H194&lt;&gt;B194,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C194="","CEK URUTAN kosong",IF(AND(E194&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E194)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="10" t="n"/>
+      <c r="B195" s="10" t="n"/>
+      <c r="C195" s="10" t="n"/>
+      <c r="D195" s="11" t="n"/>
+      <c r="E195" s="10" t="n"/>
+      <c r="F195" s="10" t="n"/>
+      <c r="G195" s="12">
+        <f>IF(D195="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D195,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H195" s="12">
+        <f>IF(G195="","",IF(LEFT(G195,4)="Wall","Wall",IF(LEFT(G195,7)="Gondola","Gondola",IF(LEFT(G195,6)="Pallet","Pallet",IF(LEFT(G195,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I195" s="12">
+        <f>IF(A195="","",IF(D195="","CEK ID FIXTURE kosong",IF(G195="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H195="Endcap","CEK Endcap tidak ikut sambung",IF(H195&lt;&gt;B195,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C195="","CEK URUTAN kosong",IF(AND(E195&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E195)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="10" t="n"/>
+      <c r="B196" s="10" t="n"/>
+      <c r="C196" s="10" t="n"/>
+      <c r="D196" s="11" t="n"/>
+      <c r="E196" s="10" t="n"/>
+      <c r="F196" s="10" t="n"/>
+      <c r="G196" s="12">
+        <f>IF(D196="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D196,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H196" s="12">
+        <f>IF(G196="","",IF(LEFT(G196,4)="Wall","Wall",IF(LEFT(G196,7)="Gondola","Gondola",IF(LEFT(G196,6)="Pallet","Pallet",IF(LEFT(G196,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I196" s="12">
+        <f>IF(A196="","",IF(D196="","CEK ID FIXTURE kosong",IF(G196="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H196="Endcap","CEK Endcap tidak ikut sambung",IF(H196&lt;&gt;B196,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C196="","CEK URUTAN kosong",IF(AND(E196&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E196)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="10" t="n"/>
+      <c r="B197" s="10" t="n"/>
+      <c r="C197" s="10" t="n"/>
+      <c r="D197" s="11" t="n"/>
+      <c r="E197" s="10" t="n"/>
+      <c r="F197" s="10" t="n"/>
+      <c r="G197" s="12">
+        <f>IF(D197="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D197,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H197" s="12">
+        <f>IF(G197="","",IF(LEFT(G197,4)="Wall","Wall",IF(LEFT(G197,7)="Gondola","Gondola",IF(LEFT(G197,6)="Pallet","Pallet",IF(LEFT(G197,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I197" s="12">
+        <f>IF(A197="","",IF(D197="","CEK ID FIXTURE kosong",IF(G197="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H197="Endcap","CEK Endcap tidak ikut sambung",IF(H197&lt;&gt;B197,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C197="","CEK URUTAN kosong",IF(AND(E197&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E197)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="10" t="n"/>
+      <c r="B198" s="10" t="n"/>
+      <c r="C198" s="10" t="n"/>
+      <c r="D198" s="11" t="n"/>
+      <c r="E198" s="10" t="n"/>
+      <c r="F198" s="10" t="n"/>
+      <c r="G198" s="12">
+        <f>IF(D198="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D198,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H198" s="12">
+        <f>IF(G198="","",IF(LEFT(G198,4)="Wall","Wall",IF(LEFT(G198,7)="Gondola","Gondola",IF(LEFT(G198,6)="Pallet","Pallet",IF(LEFT(G198,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I198" s="12">
+        <f>IF(A198="","",IF(D198="","CEK ID FIXTURE kosong",IF(G198="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H198="Endcap","CEK Endcap tidak ikut sambung",IF(H198&lt;&gt;B198,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C198="","CEK URUTAN kosong",IF(AND(E198&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E198)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="10" t="n"/>
+      <c r="B199" s="10" t="n"/>
+      <c r="C199" s="10" t="n"/>
+      <c r="D199" s="11" t="n"/>
+      <c r="E199" s="10" t="n"/>
+      <c r="F199" s="10" t="n"/>
+      <c r="G199" s="12">
+        <f>IF(D199="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D199,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H199" s="12">
+        <f>IF(G199="","",IF(LEFT(G199,4)="Wall","Wall",IF(LEFT(G199,7)="Gondola","Gondola",IF(LEFT(G199,6)="Pallet","Pallet",IF(LEFT(G199,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I199" s="12">
+        <f>IF(A199="","",IF(D199="","CEK ID FIXTURE kosong",IF(G199="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H199="Endcap","CEK Endcap tidak ikut sambung",IF(H199&lt;&gt;B199,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C199="","CEK URUTAN kosong",IF(AND(E199&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E199)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="10" t="n"/>
+      <c r="B200" s="10" t="n"/>
+      <c r="C200" s="10" t="n"/>
+      <c r="D200" s="11" t="n"/>
+      <c r="E200" s="10" t="n"/>
+      <c r="F200" s="10" t="n"/>
+      <c r="G200" s="12">
+        <f>IF(D200="","",IFERROR(INDEX(DAFTAR_FIXTURE!$B$2:$B$51,MATCH(D200,DAFTAR_FIXTURE!$A$2:$A$51,0)),""))</f>
+        <v/>
+      </c>
+      <c r="H200" s="12">
+        <f>IF(G200="","",IF(LEFT(G200,4)="Wall","Wall",IF(LEFT(G200,7)="Gondola","Gondola",IF(LEFT(G200,6)="Pallet","Pallet",IF(LEFT(G200,6)="Endcap","Endcap","")))))</f>
+        <v/>
+      </c>
+      <c r="I200" s="12">
+        <f>IF(A200="","",IF(D200="","CEK ID FIXTURE kosong",IF(G200="","CEK ID FIXTURE tidak ada di DAFTAR_FIXTURE",IF(H200="Endcap","CEK Endcap tidak ikut sambung",IF(H200&lt;&gt;B200,"CEK kategori fixture tidak sama dengan KATEGORI",IF(C200="","CEK URUTAN kosong",IF(AND(E200&lt;&gt;"",COUNTIFS(DATA!$I$2:$I$500,E200)=0),"CEK Series tidak ada di DATA","OK")))))))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I200"/>
+  <conditionalFormatting sqref="I2:I200">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>LEFT($I2,3)="CEK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="4">
+      <formula>$I2="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="KATEGORI" error="Pilih Wall, Gondola, atau Pallet (Endcap tidak ikut sambung)." type="list">
+      <formula1>"Wall,Gondola,Pallet"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="URUTAN" error="Isi angka bulat mulai 1 (urutan dari kiri ke kanan)." type="whole" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ID FIXTURE" error="Pilih ID dari daftar (kelola di sheet DAFTAR_FIXTURE)." type="list">
+      <formula1>FIXTURE_IDS</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -35904,7 +40170,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>